<commit_message>
Actualización reclamación 3664 | DC-AB032: 'PENDIENTE' → 'En proceso' por Juan perez (10/06/2026 22:24)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2202,33 +2202,31 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="R24" s="1" t="n">
+        <v>46183</v>
+      </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Enviada</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>[10/06/2026 22:21 · juan perez] en acuerdo con proveedor</t>
-        </is>
-      </c>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>juan perez</t>
+          <t>Juan perez</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>10/06/2026 22:21:27</t>
+          <t>10/06/2026 22:24:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización reclamación 163 | DC-AB011: 'PENDIENTE' → 'En proceso' por Juan perez (10/06/2026 22:49)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -584,29 +584,45 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>46183</v>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="R2" s="1" t="n">
+        <v>46183</v>
+      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>[10/06/2026 22:49 · Juan perez] En espera de fecha de devolucion</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Juan perez</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>10/06/2026 22:49:14</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -2194,41 +2210,29 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="P24" s="1" t="n">
-        <v>46183</v>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="R24" s="1" t="n">
-        <v>46183</v>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>PENDIENTE</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Juan perez</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>10/06/2026 22:31:40</t>
-        </is>
-      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">

</xml_diff>

<commit_message>
Actualización reclamación 163 | DC-AB011: 'En proceso' → 'Terminado' por Juan perez (10/06/2026 22:50)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -605,12 +605,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>[10/06/2026 22:49 · Juan perez] En espera de fecha de devolucion</t>
+          <t>[10/06/2026 22:49 · Juan perez] En espera de fecha de devolucion | [10/06/2026 22:50 · Juan perez] En espera de fecha de devolucion</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>10/06/2026 22:49:14</t>
+          <t>10/06/2026 22:50:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización reclamación 163 | DC-AB011: 'Terminado' → 'Rechazado' por Fernando Treviño (10/06/2026 23:09)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>Rechazado</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -615,12 +615,12 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Juan perez</t>
+          <t>Fernando Treviño</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>10/06/2026 22:50:19</t>
+          <t>10/06/2026 23:09:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización reclamación 163 | DC-AB011: 'Rechazado' → 'Rechazado' por Fernando Treviño (10/06/2026 23:10)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>[10/06/2026 22:49 · Juan perez] En espera de fecha de devolucion | [10/06/2026 22:50 · Juan perez] En espera de fecha de devolucion</t>
+          <t>[10/06/2026 22:49 · Juan perez] En espera de fecha de devolucion | [10/06/2026 22:50 · Juan perez] En espera de fecha de devolucion | [10/06/2026 23:10 · Fernando Treviño] Proveedor rechaza reclamo ya que dice que es por causa del transportista</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>10/06/2026 23:09:24</t>
+          <t>10/06/2026 23:10:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización reclamación 1870 | DC-MZ002: 'PENDIENTE' → 'Aceptado' por Francisco (10/06/2026 23:47)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3877,12 +3877,24 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr"/>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>[10/06/2026 23:47 · Francisco] En espera de respuesta de proveedor</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>10/06/2026 23:47:54</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">

</xml_diff>

<commit_message>
Actualización reclamación 1870 | DC-MZ002: 'Aceptado' → 'Aceptado' por Francisco (10/06/2026 23:48)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3882,7 +3882,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>[10/06/2026 23:47 · Francisco] En espera de respuesta de proveedor</t>
+          <t>[10/06/2026 23:47 · Francisco] En espera de respuesta de proveedor | [10/06/2026 23:47 · Francisco] En espera de respuesta de proveedor | [10/06/2026 23:48 · Francisco] En espera de respuesta de proveedor</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>10/06/2026 23:47:54</t>
+          <t>10/06/2026 23:48:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar (por Silvino, 13/06/2026 04:27)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,15 +865,19 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>Cuentas por pagar</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
@@ -916,17 +920,47 @@
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Se debe proceder a destruccion el proveedor se compromete a enviar la nota de credito el 20 de junio</t>
+        </is>
+      </c>
+      <c r="AG2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Silvino</t>
+        </is>
+      </c>
+      <c r="AI2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Silvino</t>
+        </is>
+      </c>
+      <c r="AK2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Silvino</t>
+        </is>
+      </c>
       <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
+      <c r="AN2" s="1" t="n">
+        <v>46193</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>23</v>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
@@ -940,7 +974,11 @@
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
@@ -961,12 +999,12 @@
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Silvino</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:26:03</t>
+          <t>13/06/2026 04:27:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 'Reporte de reclamo' reactivada (por Reactivación, 13/06/2026 04:28)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,12 +865,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
@@ -999,12 +999,12 @@
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Silvino</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:27:42</t>
+          <t>13/06/2026 04:28:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Yolanda, 13/06/2026 04:28)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,12 +865,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr"/>
@@ -999,12 +999,12 @@
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:28:30</t>
+          <t>13/06/2026 04:28:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 'Gestión' reactivada (por Reactivación, 13/06/2026 04:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,7 +865,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:29 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr"/>
@@ -999,12 +999,12 @@
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:28:45</t>
+          <t>13/06/2026 04:29:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Silvino, 13/06/2026 04:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,17 +865,17 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:29 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:29 · Reactivación] Etapa 'Gestión' reactivada | [13/06/2026 04:29 · Silvino] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Destrucción</t>
+          <t>Recolección</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -949,7 +949,9 @@
           <t>Silvino</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" s="1" t="n">
+        <v>46186</v>
+      </c>
       <c r="AN2" s="1" t="n">
         <v>46193</v>
       </c>
@@ -958,7 +960,7 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr"/>
@@ -976,7 +978,7 @@
       <c r="BC2" t="inlineStr"/>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>Destrucción</t>
+          <t>Recolección</t>
         </is>
       </c>
       <c r="BE2" t="inlineStr"/>
@@ -995,16 +997,18 @@
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
+      <c r="BU2" s="1" t="n">
+        <v>46206</v>
+      </c>
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Silvino</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:29:33</t>
+          <t>13/06/2026 04:29:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB011: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por yolanda, 13/06/2026 04:30)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -865,12 +865,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:29 · Reactivación] Etapa 'Gestión' reactivada | [13/06/2026 04:29 · Silvino] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[13/06/2026 04:26 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:27 · Silvino] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [13/06/2026 04:28 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [13/06/2026 04:28 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 04:29 · Reactivación] Etapa 'Gestión' reactivada | [13/06/2026 04:29 · Silvino] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [13/06/2026 04:30 · yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -982,7 +982,11 @@
         </is>
       </c>
       <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>Se destruye el material con el folio de destruccion 202345</t>
+        </is>
+      </c>
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
@@ -991,24 +995,46 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
+      <c r="BO2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BQ2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BS2" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU2" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="BV2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Silvino</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/06/2026 04:29:50</t>
+          <t>13/06/2026 04:30:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB013: Avance en Reporte de reclamo (por Juan Perez, 13/06/2026 15:43)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1101,7 +1101,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO</t>
+          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1111,14 +1111,26 @@
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Se recibe el folio 153025</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
+      <c r="AB3" s="1" t="n">
+        <v>46163</v>
+      </c>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
@@ -1165,8 +1177,16 @@
       <c r="BT3" t="inlineStr"/>
       <c r="BU3" t="inlineStr"/>
       <c r="BV3" t="inlineStr"/>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr">
+        <is>
+          <t>13/06/2026 15:43:32</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB013: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Juan Perez, 13/06/2026 15:44)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1101,19 +1101,19 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo</t>
+          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Se recibe el folio 153025</t>
+          <t>Se recibe el folio 153025, se envia al comprador Juan Martinez</t>
         </is>
       </c>
       <c r="V3" s="1" t="n">
@@ -1124,15 +1124,33 @@
           <t>Juan Perez</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
+      <c r="X3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
       <c r="AB3" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
+      <c r="AC3" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
@@ -1184,7 +1202,7 @@
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>13/06/2026 15:43:32</t>
+          <t>13/06/2026 15:44:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB013: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Juan Martinez, 13/06/2026 15:46)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1101,15 +1101,19 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 15:46 · Juan Martinez] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr"/>
+          <t>Destino final</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
@@ -1152,17 +1156,49 @@
         </is>
       </c>
       <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>El proveedor enviara la unidad de Transportes juanito a recogerlo el 26/06</t>
+        </is>
+      </c>
+      <c r="AG3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="AI3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="AK3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="AM3" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AN3" s="1" t="n">
+        <v>46193</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>23</v>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
@@ -1176,7 +1212,11 @@
       <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="inlineStr"/>
       <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="inlineStr"/>
@@ -1193,16 +1233,18 @@
       <c r="BR3" t="inlineStr"/>
       <c r="BS3" t="inlineStr"/>
       <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
+      <c r="BU3" s="1" t="n">
+        <v>46206</v>
+      </c>
       <c r="BV3" t="inlineStr"/>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Juan Perez</t>
+          <t>Juan Martinez</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>13/06/2026 15:44:17</t>
+          <t>13/06/2026 15:46:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB013: Avance en Destino final (por Pedro perez, 13/06/2026 15:58)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1101,7 +1101,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 15:46 · Juan Martinez] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 15:46 · Juan Martinez] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [13/06/2026 15:58 · Pedro perez] Avance en Destino final</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1227,10 +1227,22 @@
       <c r="BL3" t="inlineStr"/>
       <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
+      <c r="BO3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
+      <c r="BQ3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BR3" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
       <c r="BS3" t="inlineStr"/>
       <c r="BT3" t="inlineStr"/>
       <c r="BU3" s="1" t="n">
@@ -1239,12 +1251,12 @@
       <c r="BV3" t="inlineStr"/>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Juan Martinez</t>
+          <t>Pedro perez</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>13/06/2026 15:46:05</t>
+          <t>13/06/2026 15:58:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB013: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Martin martinez, 13/06/2026 15:58)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1101,12 +1101,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 15:46 · Juan Martinez] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [13/06/2026 15:58 · Pedro perez] Avance en Destino final</t>
+          <t>RECOLECTA VENDEDOR PRIMER SEMANA DE JUNIO | [13/06/2026 15:43 · Juan Perez] Avance en Reporte de reclamo | [13/06/2026 15:44 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 15:46 · Juan Martinez] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [13/06/2026 15:58 · Pedro perez] Avance en Destino final | [13/06/2026 15:58 · Martin martinez] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1218,7 +1218,11 @@
         </is>
       </c>
       <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>Folio de devolucion 55675</t>
+        </is>
+      </c>
       <c r="BG3" t="inlineStr"/>
       <c r="BH3" t="inlineStr"/>
       <c r="BI3" t="inlineStr"/>
@@ -1243,20 +1247,30 @@
           <t>Pedro perez</t>
         </is>
       </c>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
+      <c r="BS3" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="BT3" t="inlineStr">
+        <is>
+          <t>Martin martinez</t>
+        </is>
+      </c>
       <c r="BU3" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="BV3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Pedro perez</t>
+          <t>Martin martinez</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>13/06/2026 15:58:11</t>
+          <t>13/06/2026 15:58:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB026: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por yolanda, 13/06/2026 16:40)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1335,24 +1335,54 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>[13/06/2026 16:40 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
+      <c r="V4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AB4" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
@@ -1397,8 +1427,16 @@
       <c r="BT4" t="inlineStr"/>
       <c r="BU4" t="inlineStr"/>
       <c r="BV4" t="inlineStr"/>
-      <c r="BW4" t="inlineStr"/>
-      <c r="BX4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr">
+        <is>
+          <t>13/06/2026 16:40:33</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB026: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por juanuito, 13/06/2026 16:41)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1337,15 +1337,19 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>[13/06/2026 16:40 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[13/06/2026 16:40 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 16:41 · juanuito] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
+          <t>Destino final</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" s="1" t="n">
@@ -1385,16 +1389,44 @@
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
+      <c r="AG4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>juanuito</t>
+        </is>
+      </c>
+      <c r="AI4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>juanuito</t>
+        </is>
+      </c>
+      <c r="AK4" s="1" t="n">
+        <v>46186</v>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>juanuito</t>
+        </is>
+      </c>
+      <c r="AM4" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="AN4" s="1" t="n">
+        <v>46193</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>23</v>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ4" t="inlineStr"/>
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
@@ -1408,7 +1440,11 @@
       <c r="BA4" t="inlineStr"/>
       <c r="BB4" t="inlineStr"/>
       <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="inlineStr"/>
@@ -1425,16 +1461,18 @@
       <c r="BR4" t="inlineStr"/>
       <c r="BS4" t="inlineStr"/>
       <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
+      <c r="BU4" s="1" t="n">
+        <v>46206</v>
+      </c>
       <c r="BV4" t="inlineStr"/>
       <c r="BW4" t="inlineStr">
         <is>
-          <t>yolanda</t>
+          <t>juanuito</t>
         </is>
       </c>
       <c r="BX4" t="inlineStr">
         <is>
-          <t>13/06/2026 16:40:33</t>
+          <t>13/06/2026 16:41:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ044: Avance en Reporte de reclamo (por Fernando Treviño, 30/06/2026 19:28)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12051,7 +12051,11 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>[30/06/2026 19:28 · Fernando Treviño] Avance en Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="R88" t="inlineStr">
         <is>
           <t>Reporte de reclamo</t>
@@ -12060,13 +12064,21 @@
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr"/>
-      <c r="W88" t="inlineStr"/>
+      <c r="V88" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
       <c r="X88" t="inlineStr"/>
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="inlineStr"/>
       <c r="AA88" t="inlineStr"/>
-      <c r="AB88" t="inlineStr"/>
+      <c r="AB88" s="1" t="n">
+        <v>46133</v>
+      </c>
       <c r="AC88" t="inlineStr"/>
       <c r="AD88" t="inlineStr"/>
       <c r="AE88" t="inlineStr"/>
@@ -12113,8 +12125,16 @@
       <c r="BT88" t="inlineStr"/>
       <c r="BU88" t="inlineStr"/>
       <c r="BV88" t="inlineStr"/>
-      <c r="BW88" t="inlineStr"/>
-      <c r="BX88" t="inlineStr"/>
+      <c r="BW88" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="BX88" t="inlineStr">
+        <is>
+          <t>30/06/2026 19:28:35</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ029: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Fernando Treviño, 30/06/2026 19:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10023,24 +10023,58 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="Q72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
-      <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
-      <c r="Z72" t="inlineStr"/>
-      <c r="AA72" t="inlineStr"/>
-      <c r="AB72" t="inlineStr"/>
-      <c r="AC72" t="inlineStr"/>
-      <c r="AD72" t="inlineStr"/>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Se envio al comprador la informacion para su seguimiento</t>
+        </is>
+      </c>
+      <c r="V72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="X72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="Z72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="AB72" s="1" t="n">
+        <v>46133</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>77</v>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE72" t="inlineStr"/>
       <c r="AF72" t="inlineStr"/>
       <c r="AG72" t="inlineStr"/>
@@ -10085,8 +10119,16 @@
       <c r="BT72" t="inlineStr"/>
       <c r="BU72" t="inlineStr"/>
       <c r="BV72" t="inlineStr"/>
-      <c r="BW72" t="inlineStr"/>
-      <c r="BX72" t="inlineStr"/>
+      <c r="BW72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="BX72" t="inlineStr">
+        <is>
+          <t>30/06/2026 19:29:25</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ029: Avance en Gestión (por Fernando Treviño, 30/06/2026 19:30)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10025,7 +10025,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
@@ -10033,7 +10033,11 @@
           <t>Gestión</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr">
         <is>
@@ -10077,14 +10081,30 @@
       </c>
       <c r="AE72" t="inlineStr"/>
       <c r="AF72" t="inlineStr"/>
-      <c r="AG72" t="inlineStr"/>
-      <c r="AH72" t="inlineStr"/>
-      <c r="AI72" t="inlineStr"/>
-      <c r="AJ72" t="inlineStr"/>
+      <c r="AG72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AH72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="AI72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
       <c r="AK72" t="inlineStr"/>
       <c r="AL72" t="inlineStr"/>
-      <c r="AM72" t="inlineStr"/>
-      <c r="AN72" t="inlineStr"/>
+      <c r="AM72" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AN72" s="1" t="n">
+        <v>46163</v>
+      </c>
       <c r="AO72" t="inlineStr"/>
       <c r="AP72" t="inlineStr"/>
       <c r="AQ72" t="inlineStr"/>
@@ -10126,7 +10146,7 @@
       </c>
       <c r="BX72" t="inlineStr">
         <is>
-          <t>30/06/2026 19:29:25</t>
+          <t>30/06/2026 19:30:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Avance en Reporte de reclamo (por Juan Martinez, 30/06/2026 19:31)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9519,7 +9519,11 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="R68" t="inlineStr">
         <is>
           <t>Reporte de reclamo</t>
@@ -9528,13 +9532,27 @@
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
+      <c r="V68" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="X68" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
       <c r="Z68" t="inlineStr"/>
       <c r="AA68" t="inlineStr"/>
-      <c r="AB68" t="inlineStr"/>
+      <c r="AB68" s="1" t="n">
+        <v>46133</v>
+      </c>
       <c r="AC68" t="inlineStr"/>
       <c r="AD68" t="inlineStr"/>
       <c r="AE68" t="inlineStr"/>
@@ -9581,8 +9599,16 @@
       <c r="BT68" t="inlineStr"/>
       <c r="BU68" t="inlineStr"/>
       <c r="BV68" t="inlineStr"/>
-      <c r="BW68" t="inlineStr"/>
-      <c r="BX68" t="inlineStr"/>
+      <c r="BW68" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="BX68" t="inlineStr">
+        <is>
+          <t>30/06/2026 19:31:03</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Pedro martinez, 30/06/2026 19:31)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9521,12 +9521,12 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S68" t="inlineStr"/>
@@ -9548,13 +9548,25 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="Z68" t="inlineStr"/>
-      <c r="AA68" t="inlineStr"/>
+      <c r="Z68" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>Pedro martinez</t>
+        </is>
+      </c>
       <c r="AB68" s="1" t="n">
         <v>46133</v>
       </c>
-      <c r="AC68" t="inlineStr"/>
-      <c r="AD68" t="inlineStr"/>
+      <c r="AC68" t="n">
+        <v>77</v>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE68" t="inlineStr"/>
       <c r="AF68" t="inlineStr"/>
       <c r="AG68" t="inlineStr"/>
@@ -9601,12 +9613,12 @@
       <c r="BV68" t="inlineStr"/>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>Juan Martinez</t>
+          <t>Pedro martinez</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>30/06/2026 19:31:03</t>
+          <t>30/06/2026 19:31:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Yolanda, 01/07/2026 00:23)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1789,24 +1789,54 @@
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
+      <c r="V7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="X7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="Z7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AB7" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>48</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
@@ -1851,8 +1881,16 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="inlineStr"/>
-      <c r="BW7" t="inlineStr"/>
-      <c r="BX7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>01/07/2026 00:23:48</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB018: Avance en Gestión (por Yolanda, 01/07/2026 00:25)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,7 +1791,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1799,7 +1799,11 @@
           <t>Gestión</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" s="1" t="n">
@@ -1839,14 +1843,36 @@
       </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
+      <c r="AG7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AM7" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AN7" s="1" t="n">
+        <v>46193</v>
+      </c>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
@@ -1888,7 +1914,7 @@
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:23:48</t>
+          <t>01/07/2026 00:25:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Yolanda, 01/07/2026 00:26)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,12 +1791,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1842,7 +1842,11 @@
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Se acuerda con el proveedor recoger el producto el día indicado</t>
+        </is>
+      </c>
       <c r="AG7" s="1" t="n">
         <v>46204</v>
       </c>
@@ -1868,13 +1872,19 @@
         </is>
       </c>
       <c r="AM7" s="1" t="n">
-        <v>46204</v>
+        <v>46220</v>
       </c>
       <c r="AN7" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
+      <c r="AO7" t="n">
+        <v>41</v>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
@@ -1888,7 +1898,11 @@
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
       <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="inlineStr"/>
@@ -1905,7 +1919,9 @@
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
-      <c r="BU7" t="inlineStr"/>
+      <c r="BU7" s="1" t="n">
+        <v>46224</v>
+      </c>
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="inlineStr">
         <is>
@@ -1914,7 +1930,7 @@
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:25:20</t>
+          <t>01/07/2026 00:26:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 'Reporte de reclamo' reactivada (por Reactivación, 01/07/2026 00:27)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,12 +1791,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
@@ -1925,12 +1925,12 @@
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:26:07</t>
+          <t>01/07/2026 00:27:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Juan Perez, 01/07/2026 00:28)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,12 +1791,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1805,7 +1805,11 @@
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Pruebas mal hechas</t>
+        </is>
+      </c>
       <c r="V7" s="1" t="n">
         <v>46204</v>
       </c>
@@ -1838,7 +1842,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
@@ -1925,12 +1929,12 @@
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Juan Perez</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:27:37</t>
+          <t>01/07/2026 00:28:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 'Reporte de reclamo' reactivada (por Reactivación, 01/07/2026 00:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,12 +1791,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
@@ -1929,12 +1929,12 @@
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Juan Perez</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:28:11</t>
+          <t>01/07/2026 00:29:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Juan perez, 01/07/2026 00:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1791,12 +1791,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr"/>
@@ -1929,12 +1929,12 @@
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Juan perez</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:29:08</t>
+          <t>01/07/2026 00:29:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ029: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Fernando Treviño, 01/07/2026 01:06)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10147,12 +10147,12 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión</t>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -10219,16 +10219,28 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="AK72" t="inlineStr"/>
-      <c r="AL72" t="inlineStr"/>
+      <c r="AK72" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AL72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
       <c r="AM72" s="1" t="n">
-        <v>46203</v>
+        <v>46220</v>
       </c>
       <c r="AN72" s="1" t="n">
         <v>46163</v>
       </c>
-      <c r="AO72" t="inlineStr"/>
-      <c r="AP72" t="inlineStr"/>
+      <c r="AO72" t="n">
+        <v>71</v>
+      </c>
+      <c r="AP72" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ72" t="inlineStr"/>
       <c r="AR72" t="inlineStr"/>
       <c r="AS72" t="inlineStr"/>
@@ -10242,7 +10254,11 @@
       <c r="BA72" t="inlineStr"/>
       <c r="BB72" t="inlineStr"/>
       <c r="BC72" t="inlineStr"/>
-      <c r="BD72" t="inlineStr"/>
+      <c r="BD72" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE72" t="inlineStr"/>
       <c r="BF72" t="inlineStr"/>
       <c r="BG72" t="inlineStr"/>
@@ -10259,7 +10275,9 @@
       <c r="BR72" t="inlineStr"/>
       <c r="BS72" t="inlineStr"/>
       <c r="BT72" t="inlineStr"/>
-      <c r="BU72" t="inlineStr"/>
+      <c r="BU72" s="1" t="n">
+        <v>46224</v>
+      </c>
       <c r="BV72" t="inlineStr"/>
       <c r="BW72" t="inlineStr">
         <is>
@@ -10268,7 +10286,7 @@
       </c>
       <c r="BX72" t="inlineStr">
         <is>
-          <t>30/06/2026 19:30:36</t>
+          <t>01/07/2026 01:06:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar (por Yolanda, 01/07/2026 01:07)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9605,15 +9605,19 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S68" t="inlineStr"/>
+          <t>Cuentas por pagar</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
       <c r="V68" s="1" t="n">
@@ -9653,16 +9657,42 @@
       </c>
       <c r="AE68" t="inlineStr"/>
       <c r="AF68" t="inlineStr"/>
-      <c r="AG68" t="inlineStr"/>
-      <c r="AH68" t="inlineStr"/>
-      <c r="AI68" t="inlineStr"/>
-      <c r="AJ68" t="inlineStr"/>
-      <c r="AK68" t="inlineStr"/>
-      <c r="AL68" t="inlineStr"/>
+      <c r="AG68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AH68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AL68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM68" t="inlineStr"/>
-      <c r="AN68" t="inlineStr"/>
-      <c r="AO68" t="inlineStr"/>
-      <c r="AP68" t="inlineStr"/>
+      <c r="AN68" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="AO68" t="n">
+        <v>71</v>
+      </c>
+      <c r="AP68" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
       <c r="AS68" t="inlineStr"/>
@@ -9676,7 +9706,11 @@
       <c r="BA68" t="inlineStr"/>
       <c r="BB68" t="inlineStr"/>
       <c r="BC68" t="inlineStr"/>
-      <c r="BD68" t="inlineStr"/>
+      <c r="BD68" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE68" t="inlineStr"/>
       <c r="BF68" t="inlineStr"/>
       <c r="BG68" t="inlineStr"/>
@@ -9697,12 +9731,12 @@
       <c r="BV68" t="inlineStr"/>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>Pedro martinez</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>30/06/2026 19:31:21</t>
+          <t>01/07/2026 01:07:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final (por Yolanda, 01/07/2026 01:07)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9605,12 +9605,12 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -9695,17 +9695,49 @@
       </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
-      <c r="AS68" t="inlineStr"/>
-      <c r="AT68" t="inlineStr"/>
-      <c r="AU68" t="inlineStr"/>
-      <c r="AV68" t="inlineStr"/>
-      <c r="AW68" t="inlineStr"/>
-      <c r="AX68" t="inlineStr"/>
-      <c r="AY68" t="inlineStr"/>
-      <c r="AZ68" t="inlineStr"/>
-      <c r="BA68" t="inlineStr"/>
-      <c r="BB68" t="inlineStr"/>
-      <c r="BC68" t="inlineStr"/>
+      <c r="AS68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AU68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AW68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AY68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AZ68" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BA68" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="BB68" t="n">
+        <v>41</v>
+      </c>
+      <c r="BC68" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD68" t="inlineStr">
         <is>
           <t>Destrucción</t>
@@ -9736,7 +9768,7 @@
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>01/07/2026 01:07:25</t>
+          <t>01/07/2026 01:07:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ029: Etapa 'Gestión' reactivada (por Reactivación, 01/07/2026 01:08)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10213,12 +10213,12 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 01:08 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -10269,30 +10269,12 @@
       </c>
       <c r="AE72" t="inlineStr"/>
       <c r="AF72" t="inlineStr"/>
-      <c r="AG72" s="1" t="n">
-        <v>46203</v>
-      </c>
-      <c r="AH72" t="inlineStr">
-        <is>
-          <t>Fernando Treviño</t>
-        </is>
-      </c>
-      <c r="AI72" s="1" t="n">
-        <v>46203</v>
-      </c>
-      <c r="AJ72" t="inlineStr">
-        <is>
-          <t>Fernando Treviño</t>
-        </is>
-      </c>
-      <c r="AK72" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AL72" t="inlineStr">
-        <is>
-          <t>Fernando Treviño</t>
-        </is>
-      </c>
+      <c r="AG72" t="inlineStr"/>
+      <c r="AH72" t="inlineStr"/>
+      <c r="AI72" t="inlineStr"/>
+      <c r="AJ72" t="inlineStr"/>
+      <c r="AK72" t="inlineStr"/>
+      <c r="AL72" t="inlineStr"/>
       <c r="AM72" s="1" t="n">
         <v>46220</v>
       </c>
@@ -10304,7 +10286,7 @@
       </c>
       <c r="AP72" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ72" t="inlineStr"/>
@@ -10319,7 +10301,11 @@
       <c r="AZ72" t="inlineStr"/>
       <c r="BA72" t="inlineStr"/>
       <c r="BB72" t="inlineStr"/>
-      <c r="BC72" t="inlineStr"/>
+      <c r="BC72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD72" t="inlineStr">
         <is>
           <t>Recolección</t>
@@ -10344,15 +10330,19 @@
       <c r="BU72" s="1" t="n">
         <v>46224</v>
       </c>
-      <c r="BV72" t="inlineStr"/>
+      <c r="BV72" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW72" t="inlineStr">
         <is>
-          <t>Fernando Treviño</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX72" t="inlineStr">
         <is>
-          <t>01/07/2026 01:06:26</t>
+          <t>01/07/2026 01:08:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ029: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Fernando Treviño, 01/07/2026 01:08)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10213,12 +10213,12 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 01:08 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 01:08 · Reactivación] Etapa 'Gestión' reactivada | [01/07/2026 01:08 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -10268,15 +10268,37 @@
         </is>
       </c>
       <c r="AE72" t="inlineStr"/>
-      <c r="AF72" t="inlineStr"/>
-      <c r="AG72" t="inlineStr"/>
-      <c r="AH72" t="inlineStr"/>
-      <c r="AI72" t="inlineStr"/>
-      <c r="AJ72" t="inlineStr"/>
-      <c r="AK72" t="inlineStr"/>
-      <c r="AL72" t="inlineStr"/>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>Retraso en fecha de recoleccion</t>
+        </is>
+      </c>
+      <c r="AG72" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AH72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="AI72" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
+      <c r="AK72" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AL72" t="inlineStr">
+        <is>
+          <t>Fernando Treviño</t>
+        </is>
+      </c>
       <c r="AM72" s="1" t="n">
-        <v>46220</v>
+        <v>46228</v>
       </c>
       <c r="AN72" s="1" t="n">
         <v>46163</v>
@@ -10286,7 +10308,7 @@
       </c>
       <c r="AP72" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ72" t="inlineStr"/>
@@ -10337,12 +10359,12 @@
       </c>
       <c r="BW72" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Fernando Treviño</t>
         </is>
       </c>
       <c r="BX72" t="inlineStr">
         <is>
-          <t>01/07/2026 01:08:16</t>
+          <t>01/07/2026 01:08:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 'Cuentas por pagar' reactivada (por Reactivación, 01/07/2026 01:10)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9605,12 +9605,12 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:10 · Reactivación] Etapa 'Cuentas por pagar' reactivada</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -9695,38 +9695,14 @@
       </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
-      <c r="AS68" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AT68" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AU68" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AV68" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AW68" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AX68" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AY68" s="1" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AZ68" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AS68" t="inlineStr"/>
+      <c r="AT68" t="inlineStr"/>
+      <c r="AU68" t="inlineStr"/>
+      <c r="AV68" t="inlineStr"/>
+      <c r="AW68" t="inlineStr"/>
+      <c r="AX68" t="inlineStr"/>
+      <c r="AY68" t="inlineStr"/>
+      <c r="AZ68" t="inlineStr"/>
       <c r="BA68" s="1" t="n">
         <v>46216</v>
       </c>
@@ -9735,7 +9711,7 @@
       </c>
       <c r="BC68" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BD68" t="inlineStr">
@@ -9760,15 +9736,19 @@
       <c r="BS68" t="inlineStr"/>
       <c r="BT68" t="inlineStr"/>
       <c r="BU68" t="inlineStr"/>
-      <c r="BV68" t="inlineStr"/>
+      <c r="BV68" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>01/07/2026 01:07:49</t>
+          <t>01/07/2026 01:10:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final (por YOlanda, 01/07/2026 01:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9605,12 +9605,12 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:10 · Reactivación] Etapa 'Cuentas por pagar' reactivada</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:10 · Reactivación] Etapa 'Cuentas por pagar' reactivada | [01/07/2026 01:11 · YOlanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -9695,14 +9695,38 @@
       </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
-      <c r="AS68" t="inlineStr"/>
-      <c r="AT68" t="inlineStr"/>
-      <c r="AU68" t="inlineStr"/>
-      <c r="AV68" t="inlineStr"/>
-      <c r="AW68" t="inlineStr"/>
-      <c r="AX68" t="inlineStr"/>
-      <c r="AY68" t="inlineStr"/>
-      <c r="AZ68" t="inlineStr"/>
+      <c r="AS68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>YOlanda</t>
+        </is>
+      </c>
+      <c r="AU68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>YOlanda</t>
+        </is>
+      </c>
+      <c r="AW68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t>YOlanda</t>
+        </is>
+      </c>
+      <c r="AY68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AZ68" t="inlineStr">
+        <is>
+          <t>YOlanda</t>
+        </is>
+      </c>
       <c r="BA68" s="1" t="n">
         <v>46216</v>
       </c>
@@ -9711,7 +9735,7 @@
       </c>
       <c r="BC68" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD68" t="inlineStr">
@@ -9743,12 +9767,12 @@
       </c>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>YOlanda</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>01/07/2026 01:10:57</t>
+          <t>01/07/2026 01:11:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ038: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Juan Perez, 01/07/2026 01:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -9605,12 +9605,12 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:10 · Reactivación] Etapa 'Cuentas por pagar' reactivada | [01/07/2026 01:11 · YOlanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
+          <t>[30/06/2026 19:31 · Juan Martinez] Avance en Reporte de reclamo | [30/06/2026 19:31 · Pedro martinez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 01:07 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [01/07/2026 01:07 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:10 · Reactivación] Etapa 'Cuentas por pagar' reactivada | [01/07/2026 01:11 · YOlanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [01/07/2026 01:11 · Juan Perez] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -9744,15 +9744,37 @@
         </is>
       </c>
       <c r="BE68" t="inlineStr"/>
-      <c r="BF68" t="inlineStr"/>
-      <c r="BG68" t="inlineStr"/>
-      <c r="BH68" t="inlineStr"/>
+      <c r="BF68" t="inlineStr">
+        <is>
+          <t>Folio 76565</t>
+        </is>
+      </c>
+      <c r="BG68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="BH68" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
       <c r="BI68" t="inlineStr"/>
       <c r="BJ68" t="inlineStr"/>
-      <c r="BK68" t="inlineStr"/>
-      <c r="BL68" t="inlineStr"/>
-      <c r="BM68" t="inlineStr"/>
-      <c r="BN68" t="inlineStr"/>
+      <c r="BK68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="BL68" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="BM68" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="BN68" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
       <c r="BO68" t="inlineStr"/>
       <c r="BP68" t="inlineStr"/>
       <c r="BQ68" t="inlineStr"/>
@@ -9762,17 +9784,17 @@
       <c r="BU68" t="inlineStr"/>
       <c r="BV68" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>YOlanda</t>
+          <t>Juan Perez</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
         <is>
-          <t>01/07/2026 01:11:18</t>
+          <t>01/07/2026 01:11:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB006: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Yolanda, 30/06/2026 19:22)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -832,7 +835,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I2" s="1" t="n">
@@ -884,7 +887,7 @@
           <t>Se envía la carta reclamación y se informa al comprador SILVINO</t>
         </is>
       </c>
-      <c r="V2" s="1" t="n">
+      <c r="V2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="W2" t="inlineStr">
@@ -892,7 +895,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="X2" s="1" t="n">
+      <c r="X2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="Y2" t="inlineStr">
@@ -900,7 +903,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="Z2" s="1" t="n">
+      <c r="Z2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AA2" t="inlineStr">
@@ -908,7 +911,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AB2" s="1" t="n">
+      <c r="AB2" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AC2" t="n">
@@ -925,7 +928,7 @@
           <t>Se debe proceder a destruccion el proveedor se compromete a enviar la nota de credito el 20 de junio</t>
         </is>
       </c>
-      <c r="AG2" s="1" t="n">
+      <c r="AG2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AH2" t="inlineStr">
@@ -933,7 +936,7 @@
           <t>Silvino</t>
         </is>
       </c>
-      <c r="AI2" s="1" t="n">
+      <c r="AI2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -941,7 +944,7 @@
           <t>Silvino</t>
         </is>
       </c>
-      <c r="AK2" s="1" t="n">
+      <c r="AK2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AL2" t="inlineStr">
@@ -949,10 +952,10 @@
           <t>Silvino</t>
         </is>
       </c>
-      <c r="AM2" s="1" t="n">
+      <c r="AM2" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="AN2" s="1" t="n">
+      <c r="AN2" s="2" t="n">
         <v>46193</v>
       </c>
       <c r="AO2" t="n">
@@ -995,7 +998,7 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" s="1" t="n">
+      <c r="BO2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BP2" t="inlineStr">
@@ -1003,7 +1006,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="BQ2" s="1" t="n">
+      <c r="BQ2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BR2" t="inlineStr">
@@ -1011,7 +1014,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="BS2" s="1" t="n">
+      <c r="BS2" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BT2" t="inlineStr">
@@ -1019,7 +1022,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="BU2" s="1" t="n">
+      <c r="BU2" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="BV2" t="inlineStr">
@@ -1068,7 +1071,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I3" s="1" t="n">
@@ -1120,7 +1123,7 @@
           <t>Se recibe el folio 153025, se envia al comprador Juan Martinez</t>
         </is>
       </c>
-      <c r="V3" s="1" t="n">
+      <c r="V3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="W3" t="inlineStr">
@@ -1128,7 +1131,7 @@
           <t>Juan Perez</t>
         </is>
       </c>
-      <c r="X3" s="1" t="n">
+      <c r="X3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="Y3" t="inlineStr">
@@ -1136,7 +1139,7 @@
           <t>Juan Perez</t>
         </is>
       </c>
-      <c r="Z3" s="1" t="n">
+      <c r="Z3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AA3" t="inlineStr">
@@ -1144,7 +1147,7 @@
           <t>Juan Perez</t>
         </is>
       </c>
-      <c r="AB3" s="1" t="n">
+      <c r="AB3" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AC3" t="n">
@@ -1161,7 +1164,7 @@
           <t>El proveedor enviara la unidad de Transportes juanito a recogerlo el 26/06</t>
         </is>
       </c>
-      <c r="AG3" s="1" t="n">
+      <c r="AG3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AH3" t="inlineStr">
@@ -1169,7 +1172,7 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="AI3" s="1" t="n">
+      <c r="AI3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AJ3" t="inlineStr">
@@ -1177,7 +1180,7 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="AK3" s="1" t="n">
+      <c r="AK3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AL3" t="inlineStr">
@@ -1185,10 +1188,10 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="AM3" s="1" t="n">
+      <c r="AM3" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="AN3" s="1" t="n">
+      <c r="AN3" s="2" t="n">
         <v>46193</v>
       </c>
       <c r="AO3" t="n">
@@ -1231,7 +1234,7 @@
       <c r="BL3" t="inlineStr"/>
       <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="inlineStr"/>
-      <c r="BO3" s="1" t="n">
+      <c r="BO3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BP3" t="inlineStr">
@@ -1239,7 +1242,7 @@
           <t>Pedro perez</t>
         </is>
       </c>
-      <c r="BQ3" s="1" t="n">
+      <c r="BQ3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BR3" t="inlineStr">
@@ -1247,7 +1250,7 @@
           <t>Pedro perez</t>
         </is>
       </c>
-      <c r="BS3" s="1" t="n">
+      <c r="BS3" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="BT3" t="inlineStr">
@@ -1255,7 +1258,7 @@
           <t>Martin martinez</t>
         </is>
       </c>
-      <c r="BU3" s="1" t="n">
+      <c r="BU3" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="BV3" t="inlineStr">
@@ -1304,7 +1307,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I4" s="1" t="n">
@@ -1352,7 +1355,7 @@
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" s="1" t="n">
+      <c r="V4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="W4" t="inlineStr">
@@ -1360,7 +1363,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="X4" s="1" t="n">
+      <c r="X4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1368,7 +1371,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="Z4" s="1" t="n">
+      <c r="Z4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AA4" t="inlineStr">
@@ -1376,7 +1379,7 @@
           <t>yolanda</t>
         </is>
       </c>
-      <c r="AB4" s="1" t="n">
+      <c r="AB4" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AC4" t="n">
@@ -1389,7 +1392,7 @@
       </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" s="1" t="n">
+      <c r="AG4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AH4" t="inlineStr">
@@ -1397,7 +1400,7 @@
           <t>juanuito</t>
         </is>
       </c>
-      <c r="AI4" s="1" t="n">
+      <c r="AI4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1405,7 +1408,7 @@
           <t>juanuito</t>
         </is>
       </c>
-      <c r="AK4" s="1" t="n">
+      <c r="AK4" s="2" t="n">
         <v>46186</v>
       </c>
       <c r="AL4" t="inlineStr">
@@ -1413,10 +1416,10 @@
           <t>juanuito</t>
         </is>
       </c>
-      <c r="AM4" s="1" t="n">
+      <c r="AM4" s="2" t="n">
         <v>46200</v>
       </c>
-      <c r="AN4" s="1" t="n">
+      <c r="AN4" s="2" t="n">
         <v>46193</v>
       </c>
       <c r="AO4" t="n">
@@ -1461,7 +1464,7 @@
       <c r="BR4" t="inlineStr"/>
       <c r="BS4" t="inlineStr"/>
       <c r="BT4" t="inlineStr"/>
-      <c r="BU4" s="1" t="n">
+      <c r="BU4" s="2" t="n">
         <v>46206</v>
       </c>
       <c r="BV4" t="inlineStr"/>
@@ -1506,7 +1509,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I5" s="1" t="n">
@@ -1632,7 +1635,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I6" s="1" t="n">
@@ -1758,7 +1761,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I7" s="1" t="n">
@@ -1810,7 +1813,7 @@
           <t>Pruebas mal hechas</t>
         </is>
       </c>
-      <c r="V7" s="1" t="n">
+      <c r="V7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="W7" t="inlineStr">
@@ -1818,7 +1821,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="X7" s="1" t="n">
+      <c r="X7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1826,7 +1829,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="Z7" s="1" t="n">
+      <c r="Z7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1834,7 +1837,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AB7" s="1" t="n">
+      <c r="AB7" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AC7" t="n">
@@ -1851,7 +1854,7 @@
           <t>Se acuerda con el proveedor recoger el producto el día indicado</t>
         </is>
       </c>
-      <c r="AG7" s="1" t="n">
+      <c r="AG7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AH7" t="inlineStr">
@@ -1859,7 +1862,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AI7" s="1" t="n">
+      <c r="AI7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AJ7" t="inlineStr">
@@ -1867,7 +1870,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AK7" s="1" t="n">
+      <c r="AK7" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AL7" t="inlineStr">
@@ -1875,10 +1878,10 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AM7" s="1" t="n">
+      <c r="AM7" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="AN7" s="1" t="n">
+      <c r="AN7" s="2" t="n">
         <v>46193</v>
       </c>
       <c r="AO7" t="n">
@@ -1923,7 +1926,7 @@
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
-      <c r="BU7" s="1" t="n">
+      <c r="BU7" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="BV7" t="inlineStr"/>
@@ -1968,7 +1971,7 @@
           <t>LEONELA</t>
         </is>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I8" s="1" t="n">
@@ -2001,26 +2004,52 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OTROS INGRESOS</t>
+          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
+      <c r="V8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="n">
+        <v>46163</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>47</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
@@ -2065,8 +2094,16 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
-      <c r="BW8" t="inlineStr"/>
-      <c r="BX8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>30/06/2026 19:22:38</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -2098,7 +2135,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I9" s="1" t="n">
@@ -2224,7 +2261,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I10" s="1" t="n">
@@ -2350,7 +2387,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I11" s="1" t="n">
@@ -2476,7 +2513,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I12" s="1" t="n">
@@ -2602,7 +2639,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I13" s="1" t="n">
@@ -2728,7 +2765,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I14" s="1" t="n">
@@ -2858,7 +2895,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I15" s="1" t="n">
@@ -2984,7 +3021,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I16" s="1" t="n">
@@ -3110,7 +3147,7 @@
           <t>VICTORIA</t>
         </is>
       </c>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I17" s="1" t="n">
@@ -3236,7 +3273,7 @@
           <t>JISHELL</t>
         </is>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I18" s="1" t="n">
@@ -3362,7 +3399,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I19" s="1" t="n">
@@ -3488,7 +3525,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I20" s="1" t="n">
@@ -3614,7 +3651,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I21" s="1" t="n">
@@ -3740,7 +3777,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I22" s="1" t="n">
@@ -3866,7 +3903,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I23" s="1" t="n">
@@ -3992,7 +4029,7 @@
           <t>ESTELA</t>
         </is>
       </c>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I24" s="1" t="n">
@@ -4118,7 +4155,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I25" s="1" t="n">
@@ -4244,7 +4281,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I26" s="1" t="n">
@@ -4370,7 +4407,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I27" s="1" t="n">
@@ -4496,7 +4533,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I28" s="1" t="n">
@@ -4622,7 +4659,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I29" s="1" t="n">
@@ -4748,7 +4785,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I30" s="1" t="n">
@@ -4878,7 +4915,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I31" s="1" t="n">
@@ -5004,7 +5041,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I32" s="1" t="n">
@@ -5130,7 +5167,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I33" s="1" t="n">
@@ -5256,7 +5293,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I34" s="1" t="n">
@@ -5382,7 +5419,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I35" s="1" t="n">
@@ -5512,7 +5549,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I36" s="1" t="n">
@@ -5642,7 +5679,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I37" s="1" t="n">
@@ -5768,7 +5805,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I38" s="1" t="n">
@@ -5894,7 +5931,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I39" s="1" t="n">
@@ -6020,7 +6057,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I40" s="1" t="n">
@@ -6146,7 +6183,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I41" s="1" t="n">
@@ -6272,7 +6309,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="I42" s="1" t="n">
@@ -6398,7 +6435,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I43" s="1" t="n">
@@ -6528,7 +6565,7 @@
           <t>LEONELA</t>
         </is>
       </c>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I44" s="1" t="n">
@@ -6658,7 +6695,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I45" s="1" t="n">
@@ -6784,7 +6821,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I46" s="1" t="n">
@@ -6910,7 +6947,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I47" s="1" t="n">
@@ -7036,7 +7073,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I48" s="1" t="n">
@@ -7162,7 +7199,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I49" s="1" t="n">
@@ -7288,7 +7325,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I50" s="1" t="n">
@@ -7418,7 +7455,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I51" s="1" t="n">
@@ -7548,7 +7585,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I52" s="1" t="n">
@@ -7674,7 +7711,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I53" s="1" t="n">
@@ -7800,7 +7837,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I54" s="1" t="n">
@@ -7926,7 +7963,7 @@
           <t>VICTORIA</t>
         </is>
       </c>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I55" s="1" t="n">
@@ -8052,7 +8089,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I56" s="1" t="n">
@@ -8178,7 +8215,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I57" s="1" t="n">
@@ -8308,7 +8345,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I58" s="1" t="n">
@@ -8434,7 +8471,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I59" s="1" t="n">
@@ -8564,7 +8601,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I60" s="1" t="n">
@@ -8690,7 +8727,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I61" s="1" t="n">
@@ -8816,7 +8853,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I62" s="1" t="n">
@@ -8942,7 +8979,7 @@
           <t>JISHELL</t>
         </is>
       </c>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I63" s="1" t="n">
@@ -9068,7 +9105,7 @@
           <t>VICTORIA</t>
         </is>
       </c>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I64" s="1" t="n">
@@ -9194,7 +9231,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I65" s="1" t="n">
@@ -9320,7 +9357,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I66" s="1" t="n">
@@ -9446,7 +9483,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I67" s="1" t="n">
@@ -9572,7 +9609,7 @@
           <t>KARLA ANAID</t>
         </is>
       </c>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I68" s="1" t="n">
@@ -9620,7 +9657,7 @@
       </c>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
-      <c r="V68" s="1" t="n">
+      <c r="V68" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="W68" t="inlineStr">
@@ -9628,7 +9665,7 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="X68" s="1" t="n">
+      <c r="X68" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="Y68" t="inlineStr">
@@ -9636,7 +9673,7 @@
           <t>Juan Martinez</t>
         </is>
       </c>
-      <c r="Z68" s="1" t="n">
+      <c r="Z68" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="AA68" t="inlineStr">
@@ -9644,7 +9681,7 @@
           <t>Pedro martinez</t>
         </is>
       </c>
-      <c r="AB68" s="1" t="n">
+      <c r="AB68" s="2" t="n">
         <v>46133</v>
       </c>
       <c r="AC68" t="n">
@@ -9657,7 +9694,7 @@
       </c>
       <c r="AE68" t="inlineStr"/>
       <c r="AF68" t="inlineStr"/>
-      <c r="AG68" s="1" t="n">
+      <c r="AG68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AH68" t="inlineStr">
@@ -9665,7 +9702,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AI68" s="1" t="n">
+      <c r="AI68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AJ68" t="inlineStr">
@@ -9673,7 +9710,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AK68" s="1" t="n">
+      <c r="AK68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AL68" t="inlineStr">
@@ -9682,7 +9719,7 @@
         </is>
       </c>
       <c r="AM68" t="inlineStr"/>
-      <c r="AN68" s="1" t="n">
+      <c r="AN68" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AO68" t="n">
@@ -9695,7 +9732,7 @@
       </c>
       <c r="AQ68" t="inlineStr"/>
       <c r="AR68" t="inlineStr"/>
-      <c r="AS68" s="1" t="n">
+      <c r="AS68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AT68" t="inlineStr">
@@ -9703,7 +9740,7 @@
           <t>YOlanda</t>
         </is>
       </c>
-      <c r="AU68" s="1" t="n">
+      <c r="AU68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AV68" t="inlineStr">
@@ -9711,7 +9748,7 @@
           <t>YOlanda</t>
         </is>
       </c>
-      <c r="AW68" s="1" t="n">
+      <c r="AW68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AX68" t="inlineStr">
@@ -9719,7 +9756,7 @@
           <t>YOlanda</t>
         </is>
       </c>
-      <c r="AY68" s="1" t="n">
+      <c r="AY68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AZ68" t="inlineStr">
@@ -9727,7 +9764,7 @@
           <t>YOlanda</t>
         </is>
       </c>
-      <c r="BA68" s="1" t="n">
+      <c r="BA68" s="2" t="n">
         <v>46216</v>
       </c>
       <c r="BB68" t="n">
@@ -9749,7 +9786,7 @@
           <t>Folio 76565</t>
         </is>
       </c>
-      <c r="BG68" s="1" t="n">
+      <c r="BG68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="BH68" t="inlineStr">
@@ -9759,7 +9796,7 @@
       </c>
       <c r="BI68" t="inlineStr"/>
       <c r="BJ68" t="inlineStr"/>
-      <c r="BK68" s="1" t="n">
+      <c r="BK68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="BL68" t="inlineStr">
@@ -9767,7 +9804,7 @@
           <t>Juan Perez</t>
         </is>
       </c>
-      <c r="BM68" s="1" t="n">
+      <c r="BM68" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="BN68" t="inlineStr">
@@ -9828,7 +9865,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I69" s="1" t="n">
@@ -9954,7 +9991,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I70" s="1" t="n">
@@ -10080,7 +10117,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I71" s="1" t="n">
@@ -10206,7 +10243,7 @@
           <t>KARLA ANAID</t>
         </is>
       </c>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I72" s="1" t="n">
@@ -10258,7 +10295,7 @@
           <t>Se envio al comprador la informacion para su seguimiento</t>
         </is>
       </c>
-      <c r="V72" s="1" t="n">
+      <c r="V72" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="W72" t="inlineStr">
@@ -10266,7 +10303,7 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="X72" s="1" t="n">
+      <c r="X72" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="Y72" t="inlineStr">
@@ -10274,7 +10311,7 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="Z72" s="1" t="n">
+      <c r="Z72" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="AA72" t="inlineStr">
@@ -10282,7 +10319,7 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="AB72" s="1" t="n">
+      <c r="AB72" s="2" t="n">
         <v>46133</v>
       </c>
       <c r="AC72" t="n">
@@ -10299,7 +10336,7 @@
           <t>Retraso en fecha de recoleccion</t>
         </is>
       </c>
-      <c r="AG72" s="1" t="n">
+      <c r="AG72" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AH72" t="inlineStr">
@@ -10307,7 +10344,7 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="AI72" s="1" t="n">
+      <c r="AI72" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AJ72" t="inlineStr">
@@ -10315,7 +10352,7 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="AK72" s="1" t="n">
+      <c r="AK72" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="AL72" t="inlineStr">
@@ -10323,10 +10360,10 @@
           <t>Fernando Treviño</t>
         </is>
       </c>
-      <c r="AM72" s="1" t="n">
+      <c r="AM72" s="2" t="n">
         <v>46228</v>
       </c>
-      <c r="AN72" s="1" t="n">
+      <c r="AN72" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="AO72" t="n">
@@ -10375,7 +10412,7 @@
       <c r="BR72" t="inlineStr"/>
       <c r="BS72" t="inlineStr"/>
       <c r="BT72" t="inlineStr"/>
-      <c r="BU72" s="1" t="n">
+      <c r="BU72" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="BV72" t="inlineStr">
@@ -10424,7 +10461,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I73" s="1" t="n">
@@ -10550,7 +10587,7 @@
           <t>FRANCISCO</t>
         </is>
       </c>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I74" s="1" t="n">
@@ -10680,7 +10717,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I75" s="1" t="n">
@@ -10810,7 +10847,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I76" s="1" t="n">
@@ -10936,7 +10973,7 @@
           <t>ESTELA</t>
         </is>
       </c>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I77" s="1" t="n">
@@ -11062,7 +11099,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I78" s="1" t="n">
@@ -11188,7 +11225,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I79" s="1" t="n">
@@ -11314,7 +11351,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H80" s="1" t="n">
+      <c r="H80" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I80" s="1" t="n">
@@ -11444,7 +11481,7 @@
           <t>JISHELL</t>
         </is>
       </c>
-      <c r="H81" s="1" t="n">
+      <c r="H81" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I81" s="1" t="n">
@@ -11570,7 +11607,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H82" s="1" t="n">
+      <c r="H82" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I82" s="1" t="n">
@@ -11696,7 +11733,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H83" s="1" t="n">
+      <c r="H83" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I83" s="1" t="n">
@@ -11822,7 +11859,7 @@
           <t>SILVINO</t>
         </is>
       </c>
-      <c r="H84" s="1" t="n">
+      <c r="H84" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I84" s="1" t="n">
@@ -11948,7 +11985,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H85" s="1" t="n">
+      <c r="H85" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I85" s="1" t="n">
@@ -12074,7 +12111,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H86" s="1" t="n">
+      <c r="H86" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I86" s="1" t="n">
@@ -12200,7 +12237,7 @@
           <t>MYRIAM</t>
         </is>
       </c>
-      <c r="H87" s="1" t="n">
+      <c r="H87" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I87" s="1" t="n">
@@ -12326,7 +12363,7 @@
           <t>ARICELIA</t>
         </is>
       </c>
-      <c r="H88" s="1" t="n">
+      <c r="H88" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I88" s="1" t="n">
@@ -12370,7 +12407,7 @@
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
-      <c r="V88" s="1" t="n">
+      <c r="V88" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="W88" t="inlineStr">
@@ -12382,7 +12419,7 @@
       <c r="Y88" t="inlineStr"/>
       <c r="Z88" t="inlineStr"/>
       <c r="AA88" t="inlineStr"/>
-      <c r="AB88" s="1" t="n">
+      <c r="AB88" s="2" t="n">
         <v>46133</v>
       </c>
       <c r="AC88" t="inlineStr"/>
@@ -12472,7 +12509,7 @@
           <t>LUCIA</t>
         </is>
       </c>
-      <c r="H89" s="1" t="n">
+      <c r="H89" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I89" s="1" t="n">
@@ -12598,7 +12635,7 @@
           <t>SARA</t>
         </is>
       </c>
-      <c r="H90" s="1" t="n">
+      <c r="H90" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="I90" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB006: Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar (por Yolanda, 30/06/2026 19:23)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2004,15 +2004,19 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:23 · Yolanda] Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>Cuentas por pagar</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" s="2" t="n">
@@ -2051,17 +2055,47 @@
         </is>
       </c>
       <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Se procedera aseguir negociando</t>
+        </is>
+      </c>
+      <c r="AG8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
+      <c r="AN8" s="2" t="n">
+        <v>46193</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>40</v>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
@@ -2075,7 +2109,11 @@
       <c r="BA8" t="inlineStr"/>
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="inlineStr"/>
@@ -2101,7 +2139,7 @@
       </c>
       <c r="BX8" t="inlineStr">
         <is>
-          <t>30/06/2026 19:22:38</t>
+          <t>30/06/2026 19:23:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 'Gestión' reactivada (por Reactivación, 30/06/2026 19:24)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1794,7 +1794,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:24 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1854,30 +1854,12 @@
           <t>Se acuerda con el proveedor recoger el producto el día indicado</t>
         </is>
       </c>
-      <c r="AG7" s="2" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI7" s="2" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK7" s="2" t="n">
-        <v>46204</v>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
       <c r="AM7" s="2" t="n">
         <v>46220</v>
       </c>
@@ -1889,7 +1871,7 @@
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr"/>
@@ -1904,7 +1886,11 @@
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD7" t="inlineStr">
         <is>
           <t>Recolección</t>
@@ -1929,15 +1915,19 @@
       <c r="BU7" s="2" t="n">
         <v>46224</v>
       </c>
-      <c r="BV7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Juan perez</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>01/07/2026 00:29:30</t>
+          <t>30/06/2026 19:24:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 2 TERMINADA · Recolección → pasa a Destino final (por Yolanda, 30/06/2026 19:25)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1794,12 +1794,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:24 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:24 · Reactivación] Etapa 'Gestión' reactivada | [30/06/2026 19:25 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1854,24 +1854,42 @@
           <t>Se acuerda con el proveedor recoger el producto el día indicado</t>
         </is>
       </c>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
+      <c r="AG7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM7" s="2" t="n">
-        <v>46220</v>
+        <v>46243</v>
       </c>
       <c r="AN7" s="2" t="n">
         <v>46193</v>
       </c>
       <c r="AO7" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr"/>
@@ -1913,7 +1931,7 @@
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" s="2" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="BV7" t="inlineStr">
         <is>
@@ -1922,12 +1940,12 @@
       </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>30/06/2026 19:24:31</t>
+          <t>30/06/2026 19:25:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB006: Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final (por Pedro perez, 30/06/2026 19:25)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2012,12 +2012,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:23 · Yolanda] Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar</t>
+          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:23 · Yolanda] Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar | [30/06/2026 19:25 · Pedro perez] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2106,17 +2106,49 @@
       </c>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
+      <c r="AS8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
+      <c r="AU8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
+      <c r="AW8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
+      <c r="AY8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Pedro perez</t>
+        </is>
+      </c>
+      <c r="BA8" s="2" t="n">
+        <v>46246</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>10</v>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD8" t="inlineStr">
         <is>
           <t>Destrucción</t>
@@ -2142,12 +2174,12 @@
       <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Pedro perez</t>
         </is>
       </c>
       <c r="BX8" t="inlineStr">
         <is>
-          <t>30/06/2026 19:23:25</t>
+          <t>30/06/2026 19:25:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB006: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Juan poerez, 30/06/2026 19:26)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2012,12 +2012,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:23 · Yolanda] Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar | [30/06/2026 19:25 · Pedro perez] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
+          <t>OTROS INGRESOS | [30/06/2026 19:22 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:23 · Yolanda] Etapa 2 TERMINADA · Sin respuesta → pasa a Cuentas por pagar | [30/06/2026 19:25 · Pedro perez] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [30/06/2026 19:26 · Juan poerez] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2156,14 +2156,38 @@
       </c>
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="inlineStr"/>
+      <c r="BG8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>Juan poerez</t>
+        </is>
+      </c>
+      <c r="BI8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Juan poerez</t>
+        </is>
+      </c>
+      <c r="BK8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>Juan poerez</t>
+        </is>
+      </c>
+      <c r="BM8" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>Juan poerez</t>
+        </is>
+      </c>
       <c r="BO8" t="inlineStr"/>
       <c r="BP8" t="inlineStr"/>
       <c r="BQ8" t="inlineStr"/>
@@ -2171,15 +2195,19 @@
       <c r="BS8" t="inlineStr"/>
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW8" t="inlineStr">
         <is>
-          <t>Pedro perez</t>
+          <t>Juan poerez</t>
         </is>
       </c>
       <c r="BX8" t="inlineStr">
         <is>
-          <t>30/06/2026 19:25:31</t>
+          <t>30/06/2026 19:26:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB026: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Juanito, 30/06/2026 19:26)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1340,12 +1340,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>[13/06/2026 16:40 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 16:41 · juanuito] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[13/06/2026 16:40 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [13/06/2026 16:41 · juanuito] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [30/06/2026 19:26 · Juanito] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1449,7 +1449,11 @@
         </is>
       </c>
       <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>asas</t>
+        </is>
+      </c>
       <c r="BG4" t="inlineStr"/>
       <c r="BH4" t="inlineStr"/>
       <c r="BI4" t="inlineStr"/>
@@ -1458,24 +1462,46 @@
       <c r="BL4" t="inlineStr"/>
       <c r="BM4" t="inlineStr"/>
       <c r="BN4" t="inlineStr"/>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
+      <c r="BO4" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>Juanito</t>
+        </is>
+      </c>
+      <c r="BQ4" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BR4" t="inlineStr">
+        <is>
+          <t>Juanito</t>
+        </is>
+      </c>
+      <c r="BS4" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BT4" t="inlineStr">
+        <is>
+          <t>Juanito</t>
+        </is>
+      </c>
       <c r="BU4" s="2" t="n">
         <v>46206</v>
       </c>
-      <c r="BV4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW4" t="inlineStr">
         <is>
-          <t>juanuito</t>
+          <t>Juanito</t>
         </is>
       </c>
       <c r="BX4" t="inlineStr">
         <is>
-          <t>13/06/2026 16:41:55</t>
+          <t>30/06/2026 19:26:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ029: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Alberto, 30/06/2026 19:26)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10408,12 +10408,12 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 01:08 · Reactivación] Etapa 'Gestión' reactivada | [01/07/2026 01:08 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[30/06/2026 19:29 · Fernando Treviño] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:30 · Fernando Treviño] Avance en Gestión | [01/07/2026 01:06 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 01:08 · Reactivación] Etapa 'Gestión' reactivada | [01/07/2026 01:08 · Fernando Treviño] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [30/06/2026 19:26 · Alberto] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -10529,7 +10529,11 @@
         </is>
       </c>
       <c r="BE72" t="inlineStr"/>
-      <c r="BF72" t="inlineStr"/>
+      <c r="BF72" t="inlineStr">
+        <is>
+          <t>Devolucion 45563</t>
+        </is>
+      </c>
       <c r="BG72" t="inlineStr"/>
       <c r="BH72" t="inlineStr"/>
       <c r="BI72" t="inlineStr"/>
@@ -10538,28 +10542,46 @@
       <c r="BL72" t="inlineStr"/>
       <c r="BM72" t="inlineStr"/>
       <c r="BN72" t="inlineStr"/>
-      <c r="BO72" t="inlineStr"/>
-      <c r="BP72" t="inlineStr"/>
-      <c r="BQ72" t="inlineStr"/>
-      <c r="BR72" t="inlineStr"/>
-      <c r="BS72" t="inlineStr"/>
-      <c r="BT72" t="inlineStr"/>
+      <c r="BO72" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BP72" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
+      <c r="BQ72" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BR72" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
+      <c r="BS72" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BT72" t="inlineStr">
+        <is>
+          <t>Alberto</t>
+        </is>
+      </c>
       <c r="BU72" s="2" t="n">
         <v>46224</v>
       </c>
       <c r="BV72" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW72" t="inlineStr">
         <is>
-          <t>Fernando Treviño</t>
+          <t>Alberto</t>
         </is>
       </c>
       <c r="BX72" t="inlineStr">
         <is>
-          <t>01/07/2026 01:08:51</t>
+          <t>30/06/2026 19:26:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB018: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Alberto matinez, 30/06/2026 19:27)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1820,12 +1820,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:24 · Reactivación] Etapa 'Gestión' reactivada | [30/06/2026 19:25 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final</t>
+          <t>[01/07/2026 00:23 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:25 · Yolanda] Avance en Gestión | [01/07/2026 00:26 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [01/07/2026 00:27 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:28 · Juan Perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/07/2026 00:29 · Reactivación] Etapa 'Reporte de reclamo' reactivada | [01/07/2026 00:29 · Juan perez] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [30/06/2026 19:24 · Reactivación] Etapa 'Gestión' reactivada | [30/06/2026 19:25 · Yolanda] Etapa 2 TERMINADA · Recolección → pasa a Destino final | [30/06/2026 19:27 · Alberto matinez] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1941,7 +1941,11 @@
         </is>
       </c>
       <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>7654</t>
+        </is>
+      </c>
       <c r="BG7" t="inlineStr"/>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1950,28 +1954,46 @@
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="inlineStr"/>
       <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
+      <c r="BO7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>Alberto matinez</t>
+        </is>
+      </c>
+      <c r="BQ7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>Alberto matinez</t>
+        </is>
+      </c>
+      <c r="BS7" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>Alberto matinez</t>
+        </is>
+      </c>
       <c r="BU7" s="2" t="n">
         <v>46223</v>
       </c>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Alberto matinez</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>30/06/2026 19:25:00</t>
+          <t>30/06/2026 19:27:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ016: Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 (por Yolanda, 13/07/2026 13:23)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +51,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -828,7 +831,7 @@
         <v>7497</v>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I2" s="1" t="n">
@@ -861,22 +864,52 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HIZO CAMBIO FISICO </t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Gestión</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
+      <c r="V2" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
@@ -921,8 +954,16 @@
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:23:01</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -950,7 +991,7 @@
         <v>5618.42</v>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I3" s="1" t="n">
@@ -986,7 +1027,11 @@
           <t>VALIDANDO CON EL PROVEEDOR  (FERREMOVIL)</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -1072,7 +1117,7 @@
         <v>4995.7</v>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I4" s="1" t="n">
@@ -1104,7 +1149,11 @@
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1190,7 +1239,7 @@
         <v>4141.53</v>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I5" s="1" t="n">
@@ -1226,7 +1275,11 @@
           <t>RECOLECTO</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1312,7 +1365,7 @@
         <v>3798</v>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I6" s="1" t="n">
@@ -1344,7 +1397,11 @@
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1430,7 +1487,7 @@
         <v>2929.58</v>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I7" s="1" t="n">
@@ -1466,7 +1523,11 @@
           <t>SE SOLICITO DESTRUCCION YA SE TIENE NOTA DE CREDITO</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1552,7 +1613,7 @@
         <v>2380.56</v>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I8" s="1" t="n">
@@ -1584,7 +1645,11 @@
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1670,7 +1735,7 @@
         <v>2370.73</v>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I9" s="1" t="n">
@@ -1706,7 +1771,11 @@
           <t>SE REALIZO DESTRUCCION EN ESPERA DE LA NOTA DE CREDITO</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -1792,7 +1861,7 @@
         <v>2366.06</v>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I10" s="1" t="n">
@@ -1828,7 +1897,11 @@
           <t xml:space="preserve">GARANTIAS DE REGADERAS  SE REALIZA AJUSTE INTERNO </t>
         </is>
       </c>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -1914,7 +1987,7 @@
         <v>1949.96</v>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I11" s="1" t="n">
@@ -1950,7 +2023,11 @@
           <t>RECOLECTA  09/07/2026</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2036,7 +2113,7 @@
         <v>1290.88</v>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I12" s="1" t="n">
@@ -2072,7 +2149,11 @@
           <t>DEL COBRE 10/07</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2158,7 +2239,7 @@
         <v>1265.55</v>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I13" s="1" t="n">
@@ -2194,7 +2275,11 @@
           <t>DEL COBRE 10/07</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2268,7 +2353,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEACERO S.A.P.I. DE C.V.  </t>
+          <t>DEACERO S.A.P.I. DE C.V.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2280,7 +2365,7 @@
         <v>1192.9</v>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I14" s="1" t="n">
@@ -2316,7 +2401,11 @@
           <t>PENDIENTE FECHA DE RECOLECCION</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -2402,7 +2491,7 @@
         <v>853.4400000000001</v>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I15" s="1" t="n">
@@ -2438,7 +2527,11 @@
           <t>DEL COBRE 10/07</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -2524,7 +2617,7 @@
         <v>837.99</v>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I16" s="1" t="n">
@@ -2556,7 +2649,11 @@
         </is>
       </c>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -2642,7 +2739,7 @@
         <v>755.48</v>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I17" s="1" t="n">
@@ -2678,7 +2775,11 @@
           <t>REALIZARA NOTA DE CREDITO PARA LA SALIDA</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -2764,7 +2865,7 @@
         <v>647.5599999999999</v>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I18" s="1" t="n">
@@ -2796,7 +2897,11 @@
         </is>
       </c>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -2882,7 +2987,7 @@
         <v>605.48</v>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I19" s="1" t="n">
@@ -2918,7 +3023,11 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3004,7 +3113,7 @@
         <v>576.46</v>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I20" s="1" t="n">
@@ -3040,7 +3149,11 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -3126,7 +3239,7 @@
         <v>570.6799999999999</v>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I21" s="1" t="n">
@@ -3158,7 +3271,11 @@
         </is>
       </c>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -3244,7 +3361,7 @@
         <v>570</v>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I22" s="1" t="n">
@@ -3280,7 +3397,11 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -3366,7 +3487,7 @@
         <v>564.62</v>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I23" s="1" t="n">
@@ -3402,7 +3523,11 @@
           <t>RECOLECTA  07/07/2026</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -3488,7 +3613,7 @@
         <v>547.5700000000001</v>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I24" s="1" t="n">
@@ -3524,7 +3649,11 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
@@ -3610,7 +3739,7 @@
         <v>539.33</v>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I25" s="1" t="n">
@@ -3642,7 +3771,11 @@
         </is>
       </c>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
@@ -3728,7 +3861,7 @@
         <v>504.4</v>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I26" s="1" t="n">
@@ -3760,7 +3893,11 @@
         </is>
       </c>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
@@ -3846,7 +3983,7 @@
         <v>494</v>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I27" s="1" t="n">
@@ -3882,7 +4019,11 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
@@ -3968,7 +4109,7 @@
         <v>301.48</v>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" s="1" t="n">
+      <c r="H28" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I28" s="1" t="n">
@@ -4004,7 +4145,11 @@
           <t>RECOLECTA  07/07/2026</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
@@ -4090,7 +4235,7 @@
         <v>293.64</v>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" s="1" t="n">
+      <c r="H29" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I29" s="1" t="n">
@@ -4122,7 +4267,11 @@
         </is>
       </c>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
@@ -4208,7 +4357,7 @@
         <v>289.76</v>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I30" s="1" t="n">
@@ -4240,7 +4389,11 @@
         </is>
       </c>
       <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
@@ -4326,7 +4479,7 @@
         <v>251.16</v>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" s="1" t="n">
+      <c r="H31" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I31" s="1" t="n">
@@ -4358,7 +4511,11 @@
         </is>
       </c>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
@@ -4444,7 +4601,7 @@
         <v>227.54</v>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" s="1" t="n">
+      <c r="H32" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I32" s="1" t="n">
@@ -4476,7 +4633,11 @@
         </is>
       </c>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
@@ -4562,7 +4723,7 @@
         <v>172</v>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I33" s="1" t="n">
@@ -4594,7 +4755,11 @@
         </is>
       </c>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
@@ -4680,7 +4845,7 @@
         <v>149.02</v>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" s="1" t="n">
+      <c r="H34" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I34" s="1" t="n">
@@ -4712,7 +4877,11 @@
         </is>
       </c>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
@@ -4798,7 +4967,7 @@
         <v>139</v>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" s="1" t="n">
+      <c r="H35" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I35" s="1" t="n">
@@ -4830,7 +4999,11 @@
         </is>
       </c>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
@@ -4916,7 +5089,7 @@
         <v>134.89</v>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" s="1" t="n">
+      <c r="H36" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I36" s="1" t="n">
@@ -4948,7 +5121,11 @@
         </is>
       </c>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
@@ -5034,7 +5211,7 @@
         <v>116</v>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I37" s="1" t="n">
@@ -5066,7 +5243,11 @@
         </is>
       </c>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
@@ -5152,7 +5333,7 @@
         <v>89.20999999999999</v>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" s="1" t="n">
+      <c r="H38" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I38" s="1" t="n">
@@ -5184,7 +5365,11 @@
         </is>
       </c>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
@@ -5270,7 +5455,7 @@
         <v>72.20999999999999</v>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" s="1" t="n">
+      <c r="H39" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I39" s="1" t="n">
@@ -5306,7 +5491,11 @@
           <t>RECOLECTA  SEMANA  18-23</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
@@ -5392,7 +5581,7 @@
         <v>70.66</v>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" s="1" t="n">
+      <c r="H40" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I40" s="1" t="n">
@@ -5424,7 +5613,11 @@
         </is>
       </c>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
@@ -5510,7 +5703,7 @@
         <v>68.77</v>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" s="1" t="n">
+      <c r="H41" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I41" s="1" t="n">
@@ -5542,7 +5735,11 @@
         </is>
       </c>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
@@ -5628,7 +5825,7 @@
         <v>55.15</v>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" s="1" t="n">
+      <c r="H42" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I42" s="1" t="n">
@@ -5660,7 +5857,11 @@
         </is>
       </c>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
@@ -5746,7 +5947,7 @@
         <v>35.53</v>
       </c>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" s="1" t="n">
+      <c r="H43" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I43" s="1" t="n">
@@ -5778,7 +5979,11 @@
         </is>
       </c>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
@@ -5864,7 +6069,7 @@
         <v>35.06</v>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" s="1" t="n">
+      <c r="H44" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I44" s="1" t="n">
@@ -5896,7 +6101,11 @@
         </is>
       </c>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
@@ -5982,7 +6191,7 @@
         <v>27.8</v>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" s="1" t="n">
+      <c r="H45" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I45" s="1" t="n">
@@ -6014,7 +6223,11 @@
         </is>
       </c>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr"/>
@@ -6100,7 +6313,7 @@
         <v>19.21</v>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" s="1" t="n">
+      <c r="H46" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I46" s="1" t="n">
@@ -6136,7 +6349,11 @@
           <t xml:space="preserve">HIZO CAMBIO FISICO </t>
         </is>
       </c>
-      <c r="R46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr"/>
@@ -6222,7 +6439,7 @@
         <v>15.84</v>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" s="1" t="n">
+      <c r="H47" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I47" s="1" t="n">
@@ -6254,7 +6471,11 @@
         </is>
       </c>
       <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr"/>
@@ -6340,7 +6561,7 @@
         <v>3.45</v>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" s="1" t="n">
+      <c r="H48" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I48" s="1" t="n">
@@ -6372,7 +6593,11 @@
         </is>
       </c>
       <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr"/>
@@ -6458,7 +6683,7 @@
         <v>2.12</v>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" s="1" t="n">
+      <c r="H49" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="I49" s="1" t="n">
@@ -6490,7 +6715,11 @@
         </is>
       </c>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr"/>
@@ -6576,7 +6805,7 @@
         <v>6834.93</v>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" s="1" t="n">
+      <c r="H50" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I50" s="1" t="n">
@@ -6604,7 +6833,11 @@
         </is>
       </c>
       <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr"/>
@@ -6690,7 +6923,7 @@
         <v>5102.08</v>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" s="1" t="n">
+      <c r="H51" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I51" s="1" t="n">
@@ -6718,7 +6951,11 @@
         </is>
       </c>
       <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr"/>
@@ -6804,7 +7041,7 @@
         <v>4098.87</v>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" s="1" t="n">
+      <c r="H52" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I52" s="1" t="n">
@@ -6832,7 +7069,11 @@
         </is>
       </c>
       <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr"/>
@@ -6918,7 +7159,7 @@
         <v>4012.47</v>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" s="1" t="n">
+      <c r="H53" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I53" s="1" t="n">
@@ -6946,7 +7187,11 @@
         </is>
       </c>
       <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
@@ -7032,7 +7277,7 @@
         <v>3566.47</v>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" s="1" t="n">
+      <c r="H54" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I54" s="1" t="n">
@@ -7060,7 +7305,11 @@
         </is>
       </c>
       <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
@@ -7146,7 +7395,7 @@
         <v>3401.75</v>
       </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" s="1" t="n">
+      <c r="H55" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I55" s="1" t="n">
@@ -7174,7 +7423,11 @@
         </is>
       </c>
       <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
@@ -7260,7 +7513,7 @@
         <v>3361.58</v>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" s="1" t="n">
+      <c r="H56" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I56" s="1" t="n">
@@ -7292,7 +7545,11 @@
           <t>SE CANCELA LA DEVOLUCION, OTROS INGRESOS</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
@@ -7378,7 +7635,7 @@
         <v>3271.75</v>
       </c>
       <c r="G57" t="inlineStr"/>
-      <c r="H57" s="1" t="n">
+      <c r="H57" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I57" s="1" t="n">
@@ -7406,7 +7663,11 @@
         </is>
       </c>
       <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr"/>
       <c r="U57" t="inlineStr"/>
@@ -7492,7 +7753,7 @@
         <v>3099.14</v>
       </c>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" s="1" t="n">
+      <c r="H58" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I58" s="1" t="n">
@@ -7524,7 +7785,11 @@
           <t>DA % MERMA</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr"/>
@@ -7610,7 +7875,7 @@
         <v>2804.54</v>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" s="1" t="n">
+      <c r="H59" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I59" s="1" t="n">
@@ -7638,7 +7903,11 @@
         </is>
       </c>
       <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr"/>
       <c r="U59" t="inlineStr"/>
@@ -7724,7 +7993,7 @@
         <v>2462.15</v>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" s="1" t="n">
+      <c r="H60" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I60" s="1" t="n">
@@ -7752,7 +8021,11 @@
         </is>
       </c>
       <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
       <c r="U60" t="inlineStr"/>
@@ -7838,7 +8111,7 @@
         <v>2397.88</v>
       </c>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" s="1" t="n">
+      <c r="H61" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I61" s="1" t="n">
@@ -7870,7 +8143,11 @@
           <t>REALIZARA NOTA</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr"/>
@@ -7956,7 +8233,7 @@
         <v>1453.44</v>
       </c>
       <c r="G62" t="inlineStr"/>
-      <c r="H62" s="1" t="n">
+      <c r="H62" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I62" s="1" t="n">
@@ -7988,7 +8265,11 @@
           <t xml:space="preserve">SE CANCELO DEVOLUCION ,SE INGRESO A ALMACEN </t>
         </is>
       </c>
-      <c r="R62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
@@ -8074,7 +8355,7 @@
         <v>1068.05</v>
       </c>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" s="1" t="n">
+      <c r="H63" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I63" s="1" t="n">
@@ -8102,7 +8383,11 @@
         </is>
       </c>
       <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
@@ -8188,7 +8473,7 @@
         <v>1041.48</v>
       </c>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" s="1" t="n">
+      <c r="H64" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I64" s="1" t="n">
@@ -8216,7 +8501,11 @@
         </is>
       </c>
       <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
@@ -8302,7 +8591,7 @@
         <v>1032</v>
       </c>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" s="1" t="n">
+      <c r="H65" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I65" s="1" t="n">
@@ -8330,7 +8619,11 @@
         </is>
       </c>
       <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
@@ -8416,7 +8709,7 @@
         <v>998.87</v>
       </c>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" s="1" t="n">
+      <c r="H66" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I66" s="1" t="n">
@@ -8444,7 +8737,11 @@
         </is>
       </c>
       <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr"/>
       <c r="U66" t="inlineStr"/>
@@ -8530,7 +8827,7 @@
         <v>820.8</v>
       </c>
       <c r="G67" t="inlineStr"/>
-      <c r="H67" s="1" t="n">
+      <c r="H67" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I67" s="1" t="n">
@@ -8558,7 +8855,11 @@
         </is>
       </c>
       <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr"/>
       <c r="U67" t="inlineStr"/>
@@ -8644,7 +8945,7 @@
         <v>778.08</v>
       </c>
       <c r="G68" t="inlineStr"/>
-      <c r="H68" s="1" t="n">
+      <c r="H68" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I68" s="1" t="n">
@@ -8672,7 +8973,11 @@
         </is>
       </c>
       <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
@@ -8758,7 +9063,7 @@
         <v>659.72</v>
       </c>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" s="1" t="n">
+      <c r="H69" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I69" s="1" t="n">
@@ -8786,7 +9091,11 @@
         </is>
       </c>
       <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr"/>
@@ -8872,7 +9181,7 @@
         <v>645.7</v>
       </c>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" s="1" t="n">
+      <c r="H70" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I70" s="1" t="n">
@@ -8900,7 +9209,11 @@
         </is>
       </c>
       <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S70" t="inlineStr"/>
       <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr"/>
@@ -8986,7 +9299,7 @@
         <v>576.46</v>
       </c>
       <c r="G71" t="inlineStr"/>
-      <c r="H71" s="1" t="n">
+      <c r="H71" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I71" s="1" t="n">
@@ -9014,7 +9327,11 @@
         </is>
       </c>
       <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S71" t="inlineStr"/>
       <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr"/>
@@ -9100,7 +9417,7 @@
         <v>576.42</v>
       </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" s="1" t="n">
+      <c r="H72" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I72" s="1" t="n">
@@ -9128,7 +9445,11 @@
         </is>
       </c>
       <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr"/>
@@ -9214,7 +9535,7 @@
         <v>557.26</v>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" s="1" t="n">
+      <c r="H73" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I73" s="1" t="n">
@@ -9242,7 +9563,11 @@
         </is>
       </c>
       <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr"/>
@@ -9328,7 +9653,7 @@
         <v>546.28</v>
       </c>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" s="1" t="n">
+      <c r="H74" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I74" s="1" t="n">
@@ -9356,7 +9681,11 @@
         </is>
       </c>
       <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S74" t="inlineStr"/>
       <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr"/>
@@ -9442,7 +9771,7 @@
         <v>500</v>
       </c>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" s="1" t="n">
+      <c r="H75" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I75" s="1" t="n">
@@ -9470,7 +9799,11 @@
         </is>
       </c>
       <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr"/>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr"/>
@@ -9556,7 +9889,7 @@
         <v>325.4</v>
       </c>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" s="1" t="n">
+      <c r="H76" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I76" s="1" t="n">
@@ -9584,7 +9917,11 @@
         </is>
       </c>
       <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr"/>
@@ -9670,7 +10007,7 @@
         <v>277.14</v>
       </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" s="1" t="n">
+      <c r="H77" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I77" s="1" t="n">
@@ -9698,7 +10035,11 @@
         </is>
       </c>
       <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr"/>
@@ -9784,7 +10125,7 @@
         <v>260.04</v>
       </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" s="1" t="n">
+      <c r="H78" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I78" s="1" t="n">
@@ -9816,7 +10157,11 @@
           <t>DESTRUCCION</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr"/>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr"/>
@@ -9902,7 +10247,7 @@
         <v>258.23</v>
       </c>
       <c r="G79" t="inlineStr"/>
-      <c r="H79" s="1" t="n">
+      <c r="H79" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I79" s="1" t="n">
@@ -9930,7 +10275,11 @@
         </is>
       </c>
       <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr"/>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr"/>
       <c r="U79" t="inlineStr"/>
@@ -10016,7 +10365,7 @@
         <v>252.37</v>
       </c>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" s="1" t="n">
+      <c r="H80" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I80" s="1" t="n">
@@ -10044,7 +10393,11 @@
         </is>
       </c>
       <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr"/>
@@ -10130,7 +10483,7 @@
         <v>220.8</v>
       </c>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" s="1" t="n">
+      <c r="H81" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I81" s="1" t="n">
@@ -10158,7 +10511,11 @@
         </is>
       </c>
       <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr"/>
@@ -10244,7 +10601,7 @@
         <v>145.34</v>
       </c>
       <c r="G82" t="inlineStr"/>
-      <c r="H82" s="1" t="n">
+      <c r="H82" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I82" s="1" t="n">
@@ -10272,7 +10629,11 @@
         </is>
       </c>
       <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr"/>
@@ -10358,7 +10719,7 @@
         <v>82.09999999999999</v>
       </c>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" s="1" t="n">
+      <c r="H83" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I83" s="1" t="n">
@@ -10390,7 +10751,11 @@
           <t xml:space="preserve">NO PROCEDE,APLICA A OPERACIONES </t>
         </is>
       </c>
-      <c r="R83" t="inlineStr"/>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr"/>
@@ -10476,7 +10841,7 @@
         <v>81.55</v>
       </c>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" s="1" t="n">
+      <c r="H84" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I84" s="1" t="n">
@@ -10504,7 +10869,11 @@
         </is>
       </c>
       <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr"/>
@@ -10590,7 +10959,7 @@
         <v>64.54000000000001</v>
       </c>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" s="1" t="n">
+      <c r="H85" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I85" s="1" t="n">
@@ -10618,7 +10987,11 @@
         </is>
       </c>
       <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr"/>
@@ -10704,7 +11077,7 @@
         <v>50.65</v>
       </c>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" s="1" t="n">
+      <c r="H86" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I86" s="1" t="n">
@@ -10732,7 +11105,11 @@
         </is>
       </c>
       <c r="Q86" t="inlineStr"/>
-      <c r="R86" t="inlineStr"/>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr"/>
       <c r="U86" t="inlineStr"/>
@@ -10818,7 +11195,7 @@
         <v>22.24</v>
       </c>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" s="1" t="n">
+      <c r="H87" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I87" s="1" t="n">
@@ -10846,7 +11223,11 @@
         </is>
       </c>
       <c r="Q87" t="inlineStr"/>
-      <c r="R87" t="inlineStr"/>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="inlineStr"/>
       <c r="U87" t="inlineStr"/>
@@ -10932,7 +11313,7 @@
         <v>16.43</v>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" s="1" t="n">
+      <c r="H88" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I88" s="1" t="n">
@@ -10960,7 +11341,11 @@
         </is>
       </c>
       <c r="Q88" t="inlineStr"/>
-      <c r="R88" t="inlineStr"/>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
@@ -11046,7 +11431,7 @@
         <v>5.09</v>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" s="1" t="n">
+      <c r="H89" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I89" s="1" t="n">
@@ -11074,7 +11459,11 @@
         </is>
       </c>
       <c r="Q89" t="inlineStr"/>
-      <c r="R89" t="inlineStr"/>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S89" t="inlineStr"/>
       <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr"/>
@@ -11160,7 +11549,7 @@
         <v>0.01</v>
       </c>
       <c r="G90" t="inlineStr"/>
-      <c r="H90" s="1" t="n">
+      <c r="H90" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="I90" s="1" t="n">
@@ -11188,7 +11577,11 @@
         </is>
       </c>
       <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr"/>
@@ -11274,7 +11667,7 @@
         <v>21853.63</v>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" s="1" t="n">
+      <c r="H91" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I91" s="1" t="n">
@@ -11302,7 +11695,11 @@
         </is>
       </c>
       <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S91" t="inlineStr"/>
       <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr"/>
@@ -11388,7 +11785,7 @@
         <v>15999</v>
       </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" s="1" t="n">
+      <c r="H92" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I92" s="1" t="n">
@@ -11416,7 +11813,11 @@
         </is>
       </c>
       <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
@@ -11502,7 +11903,7 @@
         <v>4695.97</v>
       </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" s="1" t="n">
+      <c r="H93" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I93" s="1" t="n">
@@ -11530,7 +11931,11 @@
         </is>
       </c>
       <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
@@ -11616,7 +12021,7 @@
         <v>4662.52</v>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" s="1" t="n">
+      <c r="H94" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I94" s="1" t="n">
@@ -11644,7 +12049,11 @@
         </is>
       </c>
       <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S94" t="inlineStr"/>
       <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr"/>
@@ -11730,7 +12139,7 @@
         <v>4633.1</v>
       </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" s="1" t="n">
+      <c r="H95" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I95" s="1" t="n">
@@ -11758,7 +12167,11 @@
         </is>
       </c>
       <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr"/>
@@ -11844,7 +12257,7 @@
         <v>3885.21</v>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" s="1" t="n">
+      <c r="H96" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I96" s="1" t="n">
@@ -11872,7 +12285,11 @@
         </is>
       </c>
       <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S96" t="inlineStr"/>
       <c r="T96" t="inlineStr"/>
       <c r="U96" t="inlineStr"/>
@@ -11958,7 +12375,7 @@
         <v>3881.54</v>
       </c>
       <c r="G97" t="inlineStr"/>
-      <c r="H97" s="1" t="n">
+      <c r="H97" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I97" s="1" t="n">
@@ -11986,7 +12403,11 @@
         </is>
       </c>
       <c r="Q97" t="inlineStr"/>
-      <c r="R97" t="inlineStr"/>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S97" t="inlineStr"/>
       <c r="T97" t="inlineStr"/>
       <c r="U97" t="inlineStr"/>
@@ -12072,7 +12493,7 @@
         <v>2348.73</v>
       </c>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" s="1" t="n">
+      <c r="H98" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I98" s="1" t="n">
@@ -12100,7 +12521,11 @@
         </is>
       </c>
       <c r="Q98" t="inlineStr"/>
-      <c r="R98" t="inlineStr"/>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S98" t="inlineStr"/>
       <c r="T98" t="inlineStr"/>
       <c r="U98" t="inlineStr"/>
@@ -12186,7 +12611,7 @@
         <v>2283.03</v>
       </c>
       <c r="G99" t="inlineStr"/>
-      <c r="H99" s="1" t="n">
+      <c r="H99" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I99" s="1" t="n">
@@ -12214,7 +12639,11 @@
         </is>
       </c>
       <c r="Q99" t="inlineStr"/>
-      <c r="R99" t="inlineStr"/>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S99" t="inlineStr"/>
       <c r="T99" t="inlineStr"/>
       <c r="U99" t="inlineStr"/>
@@ -12300,7 +12729,7 @@
         <v>2131.91</v>
       </c>
       <c r="G100" t="inlineStr"/>
-      <c r="H100" s="1" t="n">
+      <c r="H100" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I100" s="1" t="n">
@@ -12328,7 +12757,11 @@
         </is>
       </c>
       <c r="Q100" t="inlineStr"/>
-      <c r="R100" t="inlineStr"/>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S100" t="inlineStr"/>
       <c r="T100" t="inlineStr"/>
       <c r="U100" t="inlineStr"/>
@@ -12414,7 +12847,7 @@
         <v>1691.81</v>
       </c>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" s="1" t="n">
+      <c r="H101" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I101" s="1" t="n">
@@ -12442,7 +12875,11 @@
         </is>
       </c>
       <c r="Q101" t="inlineStr"/>
-      <c r="R101" t="inlineStr"/>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S101" t="inlineStr"/>
       <c r="T101" t="inlineStr"/>
       <c r="U101" t="inlineStr"/>
@@ -12528,7 +12965,7 @@
         <v>1545.38</v>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" s="1" t="n">
+      <c r="H102" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I102" s="1" t="n">
@@ -12560,7 +12997,11 @@
           <t>RECOLECTA 22-26</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr"/>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S102" t="inlineStr"/>
       <c r="T102" t="inlineStr"/>
       <c r="U102" t="inlineStr"/>
@@ -12646,7 +13087,7 @@
         <v>1485.15</v>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" s="1" t="n">
+      <c r="H103" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I103" s="1" t="n">
@@ -12674,7 +13115,11 @@
         </is>
       </c>
       <c r="Q103" t="inlineStr"/>
-      <c r="R103" t="inlineStr"/>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S103" t="inlineStr"/>
       <c r="T103" t="inlineStr"/>
       <c r="U103" t="inlineStr"/>
@@ -12760,7 +13205,7 @@
         <v>981.33</v>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" s="1" t="n">
+      <c r="H104" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I104" s="1" t="n">
@@ -12788,7 +13233,11 @@
         </is>
       </c>
       <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr"/>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S104" t="inlineStr"/>
       <c r="T104" t="inlineStr"/>
       <c r="U104" t="inlineStr"/>
@@ -12874,7 +13323,7 @@
         <v>883.53</v>
       </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" s="1" t="n">
+      <c r="H105" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I105" s="1" t="n">
@@ -12906,7 +13355,11 @@
           <t>RECOLECTA 3/07</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr"/>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S105" t="inlineStr"/>
       <c r="T105" t="inlineStr"/>
       <c r="U105" t="inlineStr"/>
@@ -12992,7 +13445,7 @@
         <v>728.84</v>
       </c>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" s="1" t="n">
+      <c r="H106" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I106" s="1" t="n">
@@ -13020,7 +13473,11 @@
         </is>
       </c>
       <c r="Q106" t="inlineStr"/>
-      <c r="R106" t="inlineStr"/>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S106" t="inlineStr"/>
       <c r="T106" t="inlineStr"/>
       <c r="U106" t="inlineStr"/>
@@ -13106,7 +13563,7 @@
         <v>635.38</v>
       </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" s="1" t="n">
+      <c r="H107" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I107" s="1" t="n">
@@ -13134,7 +13591,11 @@
         </is>
       </c>
       <c r="Q107" t="inlineStr"/>
-      <c r="R107" t="inlineStr"/>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S107" t="inlineStr"/>
       <c r="T107" t="inlineStr"/>
       <c r="U107" t="inlineStr"/>
@@ -13220,7 +13681,7 @@
         <v>539.02</v>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" s="1" t="n">
+      <c r="H108" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I108" s="1" t="n">
@@ -13248,7 +13709,11 @@
         </is>
       </c>
       <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S108" t="inlineStr"/>
       <c r="T108" t="inlineStr"/>
       <c r="U108" t="inlineStr"/>
@@ -13334,7 +13799,7 @@
         <v>527.83</v>
       </c>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" s="1" t="n">
+      <c r="H109" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I109" s="1" t="n">
@@ -13362,7 +13827,11 @@
         </is>
       </c>
       <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S109" t="inlineStr"/>
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
@@ -13448,7 +13917,7 @@
         <v>507.16</v>
       </c>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" s="1" t="n">
+      <c r="H110" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I110" s="1" t="n">
@@ -13476,7 +13945,11 @@
         </is>
       </c>
       <c r="Q110" t="inlineStr"/>
-      <c r="R110" t="inlineStr"/>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S110" t="inlineStr"/>
       <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr"/>
@@ -13562,7 +14035,7 @@
         <v>274.26</v>
       </c>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" s="1" t="n">
+      <c r="H111" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I111" s="1" t="n">
@@ -13590,7 +14063,11 @@
         </is>
       </c>
       <c r="Q111" t="inlineStr"/>
-      <c r="R111" t="inlineStr"/>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S111" t="inlineStr"/>
       <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr"/>
@@ -13676,7 +14153,7 @@
         <v>237.04</v>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" s="1" t="n">
+      <c r="H112" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I112" s="1" t="n">
@@ -13704,7 +14181,11 @@
         </is>
       </c>
       <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr"/>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S112" t="inlineStr"/>
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
@@ -13790,7 +14271,7 @@
         <v>89.34</v>
       </c>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" s="1" t="n">
+      <c r="H113" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I113" s="1" t="n">
@@ -13818,7 +14299,11 @@
         </is>
       </c>
       <c r="Q113" t="inlineStr"/>
-      <c r="R113" t="inlineStr"/>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S113" t="inlineStr"/>
       <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr"/>
@@ -13904,7 +14389,7 @@
         <v>64.54000000000001</v>
       </c>
       <c r="G114" t="inlineStr"/>
-      <c r="H114" s="1" t="n">
+      <c r="H114" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I114" s="1" t="n">
@@ -13932,7 +14417,11 @@
         </is>
       </c>
       <c r="Q114" t="inlineStr"/>
-      <c r="R114" t="inlineStr"/>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S114" t="inlineStr"/>
       <c r="T114" t="inlineStr"/>
       <c r="U114" t="inlineStr"/>
@@ -14018,7 +14507,7 @@
         <v>51.82</v>
       </c>
       <c r="G115" t="inlineStr"/>
-      <c r="H115" s="1" t="n">
+      <c r="H115" s="2" t="n">
         <v>46195</v>
       </c>
       <c r="I115" s="1" t="n">
@@ -14046,7 +14535,11 @@
         </is>
       </c>
       <c r="Q115" t="inlineStr"/>
-      <c r="R115" t="inlineStr"/>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S115" t="inlineStr"/>
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
@@ -14132,7 +14625,7 @@
         <v>38560.57</v>
       </c>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" s="1" t="n">
+      <c r="H116" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I116" s="1" t="n">
@@ -14160,7 +14653,11 @@
         </is>
       </c>
       <c r="Q116" t="inlineStr"/>
-      <c r="R116" t="inlineStr"/>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S116" t="inlineStr"/>
       <c r="T116" t="inlineStr"/>
       <c r="U116" t="inlineStr"/>
@@ -14246,7 +14743,7 @@
         <v>21834.52</v>
       </c>
       <c r="G117" t="inlineStr"/>
-      <c r="H117" s="1" t="n">
+      <c r="H117" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I117" s="1" t="n">
@@ -14274,7 +14771,11 @@
         </is>
       </c>
       <c r="Q117" t="inlineStr"/>
-      <c r="R117" t="inlineStr"/>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S117" t="inlineStr"/>
       <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr"/>
@@ -14360,7 +14861,7 @@
         <v>11325.83</v>
       </c>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" s="1" t="n">
+      <c r="H118" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I118" s="1" t="n">
@@ -14388,7 +14889,11 @@
         </is>
       </c>
       <c r="Q118" t="inlineStr"/>
-      <c r="R118" t="inlineStr"/>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S118" t="inlineStr"/>
       <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr"/>
@@ -14474,7 +14979,7 @@
         <v>7228.8</v>
       </c>
       <c r="G119" t="inlineStr"/>
-      <c r="H119" s="1" t="n">
+      <c r="H119" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I119" s="1" t="n">
@@ -14502,7 +15007,11 @@
         </is>
       </c>
       <c r="Q119" t="inlineStr"/>
-      <c r="R119" t="inlineStr"/>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S119" t="inlineStr"/>
       <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr"/>
@@ -14588,7 +15097,7 @@
         <v>6373.29</v>
       </c>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" s="1" t="n">
+      <c r="H120" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I120" s="1" t="n">
@@ -14616,7 +15125,11 @@
         </is>
       </c>
       <c r="Q120" t="inlineStr"/>
-      <c r="R120" t="inlineStr"/>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S120" t="inlineStr"/>
       <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
@@ -14702,7 +15215,7 @@
         <v>3752.4</v>
       </c>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" s="1" t="n">
+      <c r="H121" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I121" s="1" t="n">
@@ -14730,7 +15243,11 @@
         </is>
       </c>
       <c r="Q121" t="inlineStr"/>
-      <c r="R121" t="inlineStr"/>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S121" t="inlineStr"/>
       <c r="T121" t="inlineStr"/>
       <c r="U121" t="inlineStr"/>
@@ -14816,7 +15333,7 @@
         <v>3299.01</v>
       </c>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" s="1" t="n">
+      <c r="H122" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I122" s="1" t="n">
@@ -14844,7 +15361,11 @@
         </is>
       </c>
       <c r="Q122" t="inlineStr"/>
-      <c r="R122" t="inlineStr"/>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S122" t="inlineStr"/>
       <c r="T122" t="inlineStr"/>
       <c r="U122" t="inlineStr"/>
@@ -14930,7 +15451,7 @@
         <v>2995</v>
       </c>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" s="1" t="n">
+      <c r="H123" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I123" s="1" t="n">
@@ -14958,7 +15479,11 @@
         </is>
       </c>
       <c r="Q123" t="inlineStr"/>
-      <c r="R123" t="inlineStr"/>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S123" t="inlineStr"/>
       <c r="T123" t="inlineStr"/>
       <c r="U123" t="inlineStr"/>
@@ -15044,7 +15569,7 @@
         <v>2532</v>
       </c>
       <c r="G124" t="inlineStr"/>
-      <c r="H124" s="1" t="n">
+      <c r="H124" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I124" s="1" t="n">
@@ -15072,7 +15597,11 @@
         </is>
       </c>
       <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr"/>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S124" t="inlineStr"/>
       <c r="T124" t="inlineStr"/>
       <c r="U124" t="inlineStr"/>
@@ -15158,7 +15687,7 @@
         <v>2503.69</v>
       </c>
       <c r="G125" t="inlineStr"/>
-      <c r="H125" s="1" t="n">
+      <c r="H125" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I125" s="1" t="n">
@@ -15186,7 +15715,11 @@
         </is>
       </c>
       <c r="Q125" t="inlineStr"/>
-      <c r="R125" t="inlineStr"/>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S125" t="inlineStr"/>
       <c r="T125" t="inlineStr"/>
       <c r="U125" t="inlineStr"/>
@@ -15272,7 +15805,7 @@
         <v>2341.66</v>
       </c>
       <c r="G126" t="inlineStr"/>
-      <c r="H126" s="1" t="n">
+      <c r="H126" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I126" s="1" t="n">
@@ -15300,7 +15833,11 @@
         </is>
       </c>
       <c r="Q126" t="inlineStr"/>
-      <c r="R126" t="inlineStr"/>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S126" t="inlineStr"/>
       <c r="T126" t="inlineStr"/>
       <c r="U126" t="inlineStr"/>
@@ -15386,7 +15923,7 @@
         <v>1577.8</v>
       </c>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" s="1" t="n">
+      <c r="H127" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I127" s="1" t="n">
@@ -15414,7 +15951,11 @@
         </is>
       </c>
       <c r="Q127" t="inlineStr"/>
-      <c r="R127" t="inlineStr"/>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S127" t="inlineStr"/>
       <c r="T127" t="inlineStr"/>
       <c r="U127" t="inlineStr"/>
@@ -15500,7 +16041,7 @@
         <v>1346.32</v>
       </c>
       <c r="G128" t="inlineStr"/>
-      <c r="H128" s="1" t="n">
+      <c r="H128" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I128" s="1" t="n">
@@ -15528,7 +16069,11 @@
         </is>
       </c>
       <c r="Q128" t="inlineStr"/>
-      <c r="R128" t="inlineStr"/>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S128" t="inlineStr"/>
       <c r="T128" t="inlineStr"/>
       <c r="U128" t="inlineStr"/>
@@ -15614,7 +16159,7 @@
         <v>1334.58</v>
       </c>
       <c r="G129" t="inlineStr"/>
-      <c r="H129" s="1" t="n">
+      <c r="H129" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I129" s="1" t="n">
@@ -15642,7 +16187,11 @@
         </is>
       </c>
       <c r="Q129" t="inlineStr"/>
-      <c r="R129" t="inlineStr"/>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S129" t="inlineStr"/>
       <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr"/>
@@ -15728,7 +16277,7 @@
         <v>1033.53</v>
       </c>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" s="1" t="n">
+      <c r="H130" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I130" s="1" t="n">
@@ -15756,7 +16305,11 @@
         </is>
       </c>
       <c r="Q130" t="inlineStr"/>
-      <c r="R130" t="inlineStr"/>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S130" t="inlineStr"/>
       <c r="T130" t="inlineStr"/>
       <c r="U130" t="inlineStr"/>
@@ -15842,7 +16395,7 @@
         <v>843.91</v>
       </c>
       <c r="G131" t="inlineStr"/>
-      <c r="H131" s="1" t="n">
+      <c r="H131" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I131" s="1" t="n">
@@ -15870,7 +16423,11 @@
         </is>
       </c>
       <c r="Q131" t="inlineStr"/>
-      <c r="R131" t="inlineStr"/>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S131" t="inlineStr"/>
       <c r="T131" t="inlineStr"/>
       <c r="U131" t="inlineStr"/>
@@ -15956,7 +16513,7 @@
         <v>727.2</v>
       </c>
       <c r="G132" t="inlineStr"/>
-      <c r="H132" s="1" t="n">
+      <c r="H132" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I132" s="1" t="n">
@@ -15984,7 +16541,11 @@
         </is>
       </c>
       <c r="Q132" t="inlineStr"/>
-      <c r="R132" t="inlineStr"/>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S132" t="inlineStr"/>
       <c r="T132" t="inlineStr"/>
       <c r="U132" t="inlineStr"/>
@@ -16070,7 +16631,7 @@
         <v>638.3200000000001</v>
       </c>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" s="1" t="n">
+      <c r="H133" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I133" s="1" t="n">
@@ -16098,7 +16659,11 @@
         </is>
       </c>
       <c r="Q133" t="inlineStr"/>
-      <c r="R133" t="inlineStr"/>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S133" t="inlineStr"/>
       <c r="T133" t="inlineStr"/>
       <c r="U133" t="inlineStr"/>
@@ -16184,7 +16749,7 @@
         <v>592.72</v>
       </c>
       <c r="G134" t="inlineStr"/>
-      <c r="H134" s="1" t="n">
+      <c r="H134" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I134" s="1" t="n">
@@ -16212,7 +16777,11 @@
         </is>
       </c>
       <c r="Q134" t="inlineStr"/>
-      <c r="R134" t="inlineStr"/>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S134" t="inlineStr"/>
       <c r="T134" t="inlineStr"/>
       <c r="U134" t="inlineStr"/>
@@ -16298,7 +16867,7 @@
         <v>391.45</v>
       </c>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" s="1" t="n">
+      <c r="H135" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I135" s="1" t="n">
@@ -16326,7 +16895,11 @@
         </is>
       </c>
       <c r="Q135" t="inlineStr"/>
-      <c r="R135" t="inlineStr"/>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S135" t="inlineStr"/>
       <c r="T135" t="inlineStr"/>
       <c r="U135" t="inlineStr"/>
@@ -16412,7 +16985,7 @@
         <v>348</v>
       </c>
       <c r="G136" t="inlineStr"/>
-      <c r="H136" s="1" t="n">
+      <c r="H136" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I136" s="1" t="n">
@@ -16440,7 +17013,11 @@
         </is>
       </c>
       <c r="Q136" t="inlineStr"/>
-      <c r="R136" t="inlineStr"/>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S136" t="inlineStr"/>
       <c r="T136" t="inlineStr"/>
       <c r="U136" t="inlineStr"/>
@@ -16526,7 +17103,7 @@
         <v>328.93</v>
       </c>
       <c r="G137" t="inlineStr"/>
-      <c r="H137" s="1" t="n">
+      <c r="H137" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I137" s="1" t="n">
@@ -16554,7 +17131,11 @@
         </is>
       </c>
       <c r="Q137" t="inlineStr"/>
-      <c r="R137" t="inlineStr"/>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S137" t="inlineStr"/>
       <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr"/>
@@ -16640,7 +17221,7 @@
         <v>222.82</v>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" s="1" t="n">
+      <c r="H138" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I138" s="1" t="n">
@@ -16668,7 +17249,11 @@
         </is>
       </c>
       <c r="Q138" t="inlineStr"/>
-      <c r="R138" t="inlineStr"/>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S138" t="inlineStr"/>
       <c r="T138" t="inlineStr"/>
       <c r="U138" t="inlineStr"/>
@@ -16754,7 +17339,7 @@
         <v>209.05</v>
       </c>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" s="1" t="n">
+      <c r="H139" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I139" s="1" t="n">
@@ -16782,7 +17367,11 @@
         </is>
       </c>
       <c r="Q139" t="inlineStr"/>
-      <c r="R139" t="inlineStr"/>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S139" t="inlineStr"/>
       <c r="T139" t="inlineStr"/>
       <c r="U139" t="inlineStr"/>
@@ -16868,7 +17457,7 @@
         <v>119.7</v>
       </c>
       <c r="G140" t="inlineStr"/>
-      <c r="H140" s="1" t="n">
+      <c r="H140" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I140" s="1" t="n">
@@ -16896,7 +17485,11 @@
         </is>
       </c>
       <c r="Q140" t="inlineStr"/>
-      <c r="R140" t="inlineStr"/>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S140" t="inlineStr"/>
       <c r="T140" t="inlineStr"/>
       <c r="U140" t="inlineStr"/>
@@ -16982,7 +17575,7 @@
         <v>96</v>
       </c>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" s="1" t="n">
+      <c r="H141" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I141" s="1" t="n">
@@ -17010,7 +17603,11 @@
         </is>
       </c>
       <c r="Q141" t="inlineStr"/>
-      <c r="R141" t="inlineStr"/>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S141" t="inlineStr"/>
       <c r="T141" t="inlineStr"/>
       <c r="U141" t="inlineStr"/>
@@ -17096,7 +17693,7 @@
         <v>68.77</v>
       </c>
       <c r="G142" t="inlineStr"/>
-      <c r="H142" s="1" t="n">
+      <c r="H142" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I142" s="1" t="n">
@@ -17124,7 +17721,11 @@
         </is>
       </c>
       <c r="Q142" t="inlineStr"/>
-      <c r="R142" t="inlineStr"/>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S142" t="inlineStr"/>
       <c r="T142" t="inlineStr"/>
       <c r="U142" t="inlineStr"/>
@@ -17210,7 +17811,7 @@
         <v>64.54000000000001</v>
       </c>
       <c r="G143" t="inlineStr"/>
-      <c r="H143" s="1" t="n">
+      <c r="H143" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I143" s="1" t="n">
@@ -17238,7 +17839,11 @@
         </is>
       </c>
       <c r="Q143" t="inlineStr"/>
-      <c r="R143" t="inlineStr"/>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S143" t="inlineStr"/>
       <c r="T143" t="inlineStr"/>
       <c r="U143" t="inlineStr"/>
@@ -17324,7 +17929,7 @@
         <v>32</v>
       </c>
       <c r="G144" t="inlineStr"/>
-      <c r="H144" s="1" t="n">
+      <c r="H144" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I144" s="1" t="n">
@@ -17352,7 +17957,11 @@
         </is>
       </c>
       <c r="Q144" t="inlineStr"/>
-      <c r="R144" t="inlineStr"/>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S144" t="inlineStr"/>
       <c r="T144" t="inlineStr"/>
       <c r="U144" t="inlineStr"/>
@@ -17438,7 +18047,7 @@
         <v>1.36</v>
       </c>
       <c r="G145" t="inlineStr"/>
-      <c r="H145" s="1" t="n">
+      <c r="H145" s="2" t="n">
         <v>46213</v>
       </c>
       <c r="I145" s="1" t="n">
@@ -17466,7 +18075,11 @@
         </is>
       </c>
       <c r="Q145" t="inlineStr"/>
-      <c r="R145" t="inlineStr"/>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Reporte de reclamo</t>
+        </is>
+      </c>
       <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr"/>
       <c r="U145" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ016: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 (por Yolanda, 13/07/2026 13:41)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -864,15 +864,19 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026</t>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>Destino final</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
@@ -912,16 +916,42 @@
       </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
+      <c r="AG2" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
+      <c r="AN2" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
@@ -935,7 +965,11 @@
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
@@ -952,7 +986,9 @@
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
+      <c r="BU2" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr">
         <is>
@@ -961,7 +997,7 @@
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/07/2026 13:23:01</t>
+          <t>13/07/2026 13:41:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ016: Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 (por Yolanda, 13/07/2026 13:43)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -864,12 +864,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -980,16 +980,38 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
+      <c r="BO2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU2" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="BV2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW2" t="inlineStr">
         <is>
           <t>Yolanda</t>
@@ -997,7 +1019,7 @@
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/07/2026 13:41:51</t>
+          <t>13/07/2026 13:43:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ016: Etapa 'Destino final' reactivada (por Reactivación, 13/07/2026 13:55)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -864,12 +864,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026</t>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 | [13/07/2026 13:55 · Reactivación] Etapa 'Destino final' reactivada</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>FINALIZADO</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -980,46 +980,28 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BQ2" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BS2" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BT2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
       <c r="BU2" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>13/07/2026 13:55:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ016: Avance en Destino final (por Yolanda, 13/07/2026 13:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -864,7 +864,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 | [13/07/2026 13:55 · Reactivación] Etapa 'Destino final' reactivada</t>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 | [13/07/2026 13:55 · Reactivación] Etapa 'Destino final' reactivada | [13/07/2026 13:56 · Yolanda] Avance en Destino final</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -971,7 +971,11 @@
         </is>
       </c>
       <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>folio de devolución 34298</t>
+        </is>
+      </c>
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
@@ -996,12 +1000,12 @@
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/07/2026 13:55:27</t>
+          <t>13/07/2026 13:56:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ016: Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 (por Yolanda, 13/07/2026 13:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -864,12 +864,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 | [13/07/2026 13:55 · Reactivación] Etapa 'Destino final' reactivada | [13/07/2026 13:56 · Yolanda] Avance en Destino final</t>
+          <t>HIZO CAMBIO FISICO | [13/07/2026 13:23 · Yolanda] Ajuste manual de fechas en 'Reporte de reclamo' · etapa TERMINADA con fecha 07/05/2026 | [13/07/2026 13:41 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [13/07/2026 13:43 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026 | [13/07/2026 13:55 · Reactivación] Etapa 'Destino final' reactivada | [13/07/2026 13:56 · Yolanda] Avance en Destino final | [13/07/2026 13:56 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 26/06/2026</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -984,18 +984,36 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
+      <c r="BO2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU2" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
@@ -1005,7 +1023,7 @@
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>13/07/2026 13:56:19</t>
+          <t>13/07/2026 13:56:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 14:33)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -866,7 +866,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2162,7 +2162,7 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -4196,7 +4196,7 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -4544,7 +4544,7 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -4714,7 +4714,7 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -4884,7 +4884,7 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
@@ -5054,7 +5054,7 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
@@ -5224,7 +5224,7 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
@@ -5394,7 +5394,7 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
@@ -5564,7 +5564,7 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -5734,7 +5734,7 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
@@ -5904,7 +5904,7 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
@@ -6074,7 +6074,7 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
@@ -6244,7 +6244,7 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
@@ -6414,7 +6414,7 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
@@ -6584,7 +6584,7 @@
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
@@ -6760,7 +6760,7 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
@@ -6930,7 +6930,7 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S36" t="inlineStr"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 14:42)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -963,9 +963,17 @@
       <c r="AX2" t="inlineStr"/>
       <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
+      <c r="BA2" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD2" t="inlineStr"/>
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
@@ -1370,7 +1378,7 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr">
         <is>
-          <t>Se autorizo destuccion recibida Nota de credito</t>
+          <t>Se autorizo destruccion recibida Nota de credito</t>
         </is>
       </c>
       <c r="BG4" t="inlineStr"/>
@@ -1825,9 +1833,17 @@
       <c r="AX7" t="inlineStr"/>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
+      <c r="BA7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
@@ -2223,9 +2239,17 @@
       <c r="AX9" t="inlineStr"/>
       <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="inlineStr"/>
-      <c r="BB9" t="inlineStr"/>
-      <c r="BC9" t="inlineStr"/>
+      <c r="BA9" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD9" t="inlineStr"/>
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
@@ -2531,9 +2555,17 @@
       <c r="AX11" t="inlineStr"/>
       <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="inlineStr"/>
-      <c r="BB11" t="inlineStr"/>
-      <c r="BC11" t="inlineStr"/>
+      <c r="BA11" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD11" t="inlineStr"/>
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
@@ -2841,9 +2873,17 @@
       <c r="AX13" t="inlineStr"/>
       <c r="AY13" t="inlineStr"/>
       <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
-      <c r="BB13" t="inlineStr"/>
-      <c r="BC13" t="inlineStr"/>
+      <c r="BA13" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD13" t="inlineStr"/>
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
@@ -3023,9 +3063,17 @@
       <c r="AX14" t="inlineStr"/>
       <c r="AY14" t="inlineStr"/>
       <c r="AZ14" t="inlineStr"/>
-      <c r="BA14" t="inlineStr"/>
-      <c r="BB14" t="inlineStr"/>
-      <c r="BC14" t="inlineStr"/>
+      <c r="BA14" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD14" t="inlineStr"/>
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
@@ -3677,9 +3725,17 @@
       <c r="AX18" t="inlineStr"/>
       <c r="AY18" t="inlineStr"/>
       <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="inlineStr"/>
-      <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
+      <c r="BA18" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD18" t="inlineStr"/>
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
@@ -4217,9 +4273,17 @@
       <c r="AX22" t="inlineStr"/>
       <c r="AY22" t="inlineStr"/>
       <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" t="inlineStr"/>
-      <c r="BB22" t="inlineStr"/>
-      <c r="BC22" t="inlineStr"/>
+      <c r="BA22" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB22" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC22" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD22" t="inlineStr"/>
       <c r="BE22" t="inlineStr"/>
       <c r="BF22" t="inlineStr"/>
@@ -4527,9 +4591,17 @@
       <c r="AX24" t="inlineStr"/>
       <c r="AY24" t="inlineStr"/>
       <c r="AZ24" t="inlineStr"/>
-      <c r="BA24" t="inlineStr"/>
-      <c r="BB24" t="inlineStr"/>
-      <c r="BC24" t="inlineStr"/>
+      <c r="BA24" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC24" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD24" t="inlineStr"/>
       <c r="BE24" t="inlineStr"/>
       <c r="BF24" t="inlineStr"/>
@@ -4919,9 +4991,17 @@
       <c r="AX26" t="inlineStr"/>
       <c r="AY26" t="inlineStr"/>
       <c r="AZ26" t="inlineStr"/>
-      <c r="BA26" t="inlineStr"/>
-      <c r="BB26" t="inlineStr"/>
-      <c r="BC26" t="inlineStr"/>
+      <c r="BA26" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC26" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD26" t="inlineStr"/>
       <c r="BE26" t="inlineStr"/>
       <c r="BF26" t="inlineStr"/>
@@ -5525,9 +5605,17 @@
       <c r="AX29" t="inlineStr"/>
       <c r="AY29" t="inlineStr"/>
       <c r="AZ29" t="inlineStr"/>
-      <c r="BA29" t="inlineStr"/>
-      <c r="BB29" t="inlineStr"/>
-      <c r="BC29" t="inlineStr"/>
+      <c r="BA29" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC29" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD29" t="inlineStr"/>
       <c r="BE29" t="inlineStr"/>
       <c r="BF29" t="inlineStr"/>
@@ -5833,9 +5921,17 @@
       <c r="AX31" t="inlineStr"/>
       <c r="AY31" t="inlineStr"/>
       <c r="AZ31" t="inlineStr"/>
-      <c r="BA31" t="inlineStr"/>
-      <c r="BB31" t="inlineStr"/>
-      <c r="BC31" t="inlineStr"/>
+      <c r="BA31" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC31" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD31" t="inlineStr"/>
       <c r="BE31" t="inlineStr"/>
       <c r="BF31" t="inlineStr"/>
@@ -6021,9 +6117,17 @@
       <c r="AX32" t="inlineStr"/>
       <c r="AY32" t="inlineStr"/>
       <c r="AZ32" t="inlineStr"/>
-      <c r="BA32" t="inlineStr"/>
-      <c r="BB32" t="inlineStr"/>
-      <c r="BC32" t="inlineStr"/>
+      <c r="BA32" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC32" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD32" t="inlineStr"/>
       <c r="BE32" t="inlineStr"/>
       <c r="BF32" t="inlineStr"/>
@@ -6417,9 +6521,17 @@
       <c r="AX34" t="inlineStr"/>
       <c r="AY34" t="inlineStr"/>
       <c r="AZ34" t="inlineStr"/>
-      <c r="BA34" t="inlineStr"/>
-      <c r="BB34" t="inlineStr"/>
-      <c r="BC34" t="inlineStr"/>
+      <c r="BA34" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB34" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC34" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD34" t="inlineStr"/>
       <c r="BE34" t="inlineStr"/>
       <c r="BF34" t="inlineStr"/>
@@ -7267,9 +7379,17 @@
       <c r="AX39" t="inlineStr"/>
       <c r="AY39" t="inlineStr"/>
       <c r="AZ39" t="inlineStr"/>
-      <c r="BA39" t="inlineStr"/>
-      <c r="BB39" t="inlineStr"/>
-      <c r="BC39" t="inlineStr"/>
+      <c r="BA39" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB39" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC39" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD39" t="inlineStr"/>
       <c r="BE39" t="inlineStr"/>
       <c r="BF39" t="inlineStr"/>
@@ -7453,9 +7573,17 @@
       <c r="AX40" t="inlineStr"/>
       <c r="AY40" t="inlineStr"/>
       <c r="AZ40" t="inlineStr"/>
-      <c r="BA40" t="inlineStr"/>
-      <c r="BB40" t="inlineStr"/>
-      <c r="BC40" t="inlineStr"/>
+      <c r="BA40" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB40" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC40" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD40" t="inlineStr"/>
       <c r="BE40" t="inlineStr"/>
       <c r="BF40" t="inlineStr"/>
@@ -7641,9 +7769,17 @@
       <c r="AX41" t="inlineStr"/>
       <c r="AY41" t="inlineStr"/>
       <c r="AZ41" t="inlineStr"/>
-      <c r="BA41" t="inlineStr"/>
-      <c r="BB41" t="inlineStr"/>
-      <c r="BC41" t="inlineStr"/>
+      <c r="BA41" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB41" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC41" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD41" t="inlineStr"/>
       <c r="BE41" t="inlineStr"/>
       <c r="BF41" t="inlineStr"/>
@@ -7829,9 +7965,17 @@
       <c r="AX42" t="inlineStr"/>
       <c r="AY42" t="inlineStr"/>
       <c r="AZ42" t="inlineStr"/>
-      <c r="BA42" t="inlineStr"/>
-      <c r="BB42" t="inlineStr"/>
-      <c r="BC42" t="inlineStr"/>
+      <c r="BA42" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB42" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD42" t="inlineStr"/>
       <c r="BE42" t="inlineStr"/>
       <c r="BF42" t="inlineStr"/>
@@ -8003,9 +8147,17 @@
       <c r="AX43" t="inlineStr"/>
       <c r="AY43" t="inlineStr"/>
       <c r="AZ43" t="inlineStr"/>
-      <c r="BA43" t="inlineStr"/>
-      <c r="BB43" t="inlineStr"/>
-      <c r="BC43" t="inlineStr"/>
+      <c r="BA43" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB43" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC43" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD43" t="inlineStr"/>
       <c r="BE43" t="inlineStr"/>
       <c r="BF43" t="inlineStr"/>
@@ -9625,9 +9777,17 @@
       <c r="AX52" t="inlineStr"/>
       <c r="AY52" t="inlineStr"/>
       <c r="AZ52" t="inlineStr"/>
-      <c r="BA52" t="inlineStr"/>
-      <c r="BB52" t="inlineStr"/>
-      <c r="BC52" t="inlineStr"/>
+      <c r="BA52" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB52" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC52" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD52" t="inlineStr"/>
       <c r="BE52" t="inlineStr"/>
       <c r="BF52" t="inlineStr"/>
@@ -10160,8 +10320,14 @@
       <c r="AY55" t="inlineStr"/>
       <c r="AZ55" t="inlineStr"/>
       <c r="BA55" t="inlineStr"/>
-      <c r="BB55" t="inlineStr"/>
-      <c r="BC55" t="inlineStr"/>
+      <c r="BB55" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC55" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD55" t="inlineStr"/>
       <c r="BE55" t="inlineStr"/>
       <c r="BF55" t="inlineStr">
@@ -10777,9 +10943,17 @@
       <c r="AX58" t="inlineStr"/>
       <c r="AY58" t="inlineStr"/>
       <c r="AZ58" t="inlineStr"/>
-      <c r="BA58" t="inlineStr"/>
-      <c r="BB58" t="inlineStr"/>
-      <c r="BC58" t="inlineStr"/>
+      <c r="BA58" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB58" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC58" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD58" t="inlineStr"/>
       <c r="BE58" t="inlineStr"/>
       <c r="BF58" t="inlineStr"/>
@@ -10947,9 +11121,17 @@
       <c r="AX59" t="inlineStr"/>
       <c r="AY59" t="inlineStr"/>
       <c r="AZ59" t="inlineStr"/>
-      <c r="BA59" t="inlineStr"/>
-      <c r="BB59" t="inlineStr"/>
-      <c r="BC59" t="inlineStr"/>
+      <c r="BA59" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB59" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC59" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD59" t="inlineStr"/>
       <c r="BE59" t="inlineStr"/>
       <c r="BF59" t="inlineStr"/>
@@ -11323,9 +11505,17 @@
       <c r="AX61" t="inlineStr"/>
       <c r="AY61" t="inlineStr"/>
       <c r="AZ61" t="inlineStr"/>
-      <c r="BA61" t="inlineStr"/>
-      <c r="BB61" t="inlineStr"/>
-      <c r="BC61" t="inlineStr"/>
+      <c r="BA61" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB61" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC61" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD61" t="inlineStr"/>
       <c r="BE61" t="inlineStr"/>
       <c r="BF61" t="inlineStr"/>
@@ -11877,9 +12067,17 @@
       <c r="AX64" t="inlineStr"/>
       <c r="AY64" t="inlineStr"/>
       <c r="AZ64" t="inlineStr"/>
-      <c r="BA64" t="inlineStr"/>
-      <c r="BB64" t="inlineStr"/>
-      <c r="BC64" t="inlineStr"/>
+      <c r="BA64" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB64" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC64" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD64" t="inlineStr"/>
       <c r="BE64" t="inlineStr"/>
       <c r="BF64" t="inlineStr"/>
@@ -13023,9 +13221,17 @@
       <c r="AX70" t="inlineStr"/>
       <c r="AY70" t="inlineStr"/>
       <c r="AZ70" t="inlineStr"/>
-      <c r="BA70" t="inlineStr"/>
-      <c r="BB70" t="inlineStr"/>
-      <c r="BC70" t="inlineStr"/>
+      <c r="BA70" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB70" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC70" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD70" t="inlineStr"/>
       <c r="BE70" t="inlineStr"/>
       <c r="BF70" t="inlineStr"/>
@@ -13791,9 +13997,17 @@
       <c r="AX75" t="inlineStr"/>
       <c r="AY75" t="inlineStr"/>
       <c r="AZ75" t="inlineStr"/>
-      <c r="BA75" t="inlineStr"/>
-      <c r="BB75" t="inlineStr"/>
-      <c r="BC75" t="inlineStr"/>
+      <c r="BA75" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB75" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC75" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD75" t="inlineStr"/>
       <c r="BE75" t="inlineStr"/>
       <c r="BF75" t="inlineStr"/>
@@ -13961,9 +14175,17 @@
       <c r="AX76" t="inlineStr"/>
       <c r="AY76" t="inlineStr"/>
       <c r="AZ76" t="inlineStr"/>
-      <c r="BA76" t="inlineStr"/>
-      <c r="BB76" t="inlineStr"/>
-      <c r="BC76" t="inlineStr"/>
+      <c r="BA76" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB76" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC76" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD76" t="inlineStr"/>
       <c r="BE76" t="inlineStr"/>
       <c r="BF76" t="inlineStr"/>
@@ -14131,9 +14353,17 @@
       <c r="AX77" t="inlineStr"/>
       <c r="AY77" t="inlineStr"/>
       <c r="AZ77" t="inlineStr"/>
-      <c r="BA77" t="inlineStr"/>
-      <c r="BB77" t="inlineStr"/>
-      <c r="BC77" t="inlineStr"/>
+      <c r="BA77" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB77" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC77" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD77" t="inlineStr"/>
       <c r="BE77" t="inlineStr"/>
       <c r="BF77" t="inlineStr"/>
@@ -14301,9 +14531,17 @@
       <c r="AX78" t="inlineStr"/>
       <c r="AY78" t="inlineStr"/>
       <c r="AZ78" t="inlineStr"/>
-      <c r="BA78" t="inlineStr"/>
-      <c r="BB78" t="inlineStr"/>
-      <c r="BC78" t="inlineStr"/>
+      <c r="BA78" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB78" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC78" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD78" t="inlineStr"/>
       <c r="BE78" t="inlineStr"/>
       <c r="BF78" t="inlineStr"/>
@@ -14471,9 +14709,17 @@
       <c r="AX79" t="inlineStr"/>
       <c r="AY79" t="inlineStr"/>
       <c r="AZ79" t="inlineStr"/>
-      <c r="BA79" t="inlineStr"/>
-      <c r="BB79" t="inlineStr"/>
-      <c r="BC79" t="inlineStr"/>
+      <c r="BA79" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB79" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC79" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD79" t="inlineStr"/>
       <c r="BE79" t="inlineStr"/>
       <c r="BF79" t="inlineStr"/>
@@ -14641,9 +14887,17 @@
       <c r="AX80" t="inlineStr"/>
       <c r="AY80" t="inlineStr"/>
       <c r="AZ80" t="inlineStr"/>
-      <c r="BA80" t="inlineStr"/>
-      <c r="BB80" t="inlineStr"/>
-      <c r="BC80" t="inlineStr"/>
+      <c r="BA80" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB80" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC80" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD80" t="inlineStr"/>
       <c r="BE80" t="inlineStr"/>
       <c r="BF80" t="inlineStr"/>
@@ -14933,9 +15187,17 @@
       <c r="AX82" t="inlineStr"/>
       <c r="AY82" t="inlineStr"/>
       <c r="AZ82" t="inlineStr"/>
-      <c r="BA82" t="inlineStr"/>
-      <c r="BB82" t="inlineStr"/>
-      <c r="BC82" t="inlineStr"/>
+      <c r="BA82" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB82" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC82" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD82" t="inlineStr"/>
       <c r="BE82" t="inlineStr"/>
       <c r="BF82" t="inlineStr">
@@ -15139,9 +15401,17 @@
       <c r="AX83" t="inlineStr"/>
       <c r="AY83" t="inlineStr"/>
       <c r="AZ83" t="inlineStr"/>
-      <c r="BA83" t="inlineStr"/>
-      <c r="BB83" t="inlineStr"/>
-      <c r="BC83" t="inlineStr"/>
+      <c r="BA83" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB83" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC83" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD83" t="inlineStr"/>
       <c r="BE83" t="inlineStr"/>
       <c r="BF83" t="inlineStr"/>
@@ -15315,9 +15585,17 @@
       <c r="AX84" t="inlineStr"/>
       <c r="AY84" t="inlineStr"/>
       <c r="AZ84" t="inlineStr"/>
-      <c r="BA84" t="inlineStr"/>
-      <c r="BB84" t="inlineStr"/>
-      <c r="BC84" t="inlineStr"/>
+      <c r="BA84" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB84" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC84" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD84" t="inlineStr"/>
       <c r="BE84" t="inlineStr"/>
       <c r="BF84" t="inlineStr"/>
@@ -15603,9 +15881,17 @@
       <c r="AX86" t="inlineStr"/>
       <c r="AY86" t="inlineStr"/>
       <c r="AZ86" t="inlineStr"/>
-      <c r="BA86" t="inlineStr"/>
-      <c r="BB86" t="inlineStr"/>
-      <c r="BC86" t="inlineStr"/>
+      <c r="BA86" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB86" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC86" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD86" t="inlineStr"/>
       <c r="BE86" t="inlineStr"/>
       <c r="BF86" t="inlineStr"/>
@@ -15967,14 +16253,8 @@
       </c>
       <c r="AE89" t="inlineStr"/>
       <c r="AF89" t="inlineStr"/>
-      <c r="AG89" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH89" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG89" t="inlineStr"/>
+      <c r="AH89" t="inlineStr"/>
       <c r="AI89" s="1" t="n">
         <v>46199</v>
       </c>
@@ -16013,14 +16293,22 @@
       <c r="AX89" t="inlineStr"/>
       <c r="AY89" t="inlineStr"/>
       <c r="AZ89" t="inlineStr"/>
-      <c r="BA89" t="inlineStr"/>
-      <c r="BB89" t="inlineStr"/>
-      <c r="BC89" t="inlineStr"/>
+      <c r="BA89" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB89" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC89" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD89" t="inlineStr"/>
       <c r="BE89" t="inlineStr"/>
       <c r="BF89" t="inlineStr">
         <is>
-          <t>No procede aplica a operaciones</t>
+          <t>CANCELADA No procede aplica a operaciones</t>
         </is>
       </c>
       <c r="BG89" t="inlineStr"/>
@@ -16173,14 +16461,8 @@
       </c>
       <c r="AE90" t="inlineStr"/>
       <c r="AF90" t="inlineStr"/>
-      <c r="AG90" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH90" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG90" t="inlineStr"/>
+      <c r="AH90" t="inlineStr"/>
       <c r="AI90" s="1" t="n">
         <v>46199</v>
       </c>
@@ -16219,9 +16501,17 @@
       <c r="AX90" t="inlineStr"/>
       <c r="AY90" t="inlineStr"/>
       <c r="AZ90" t="inlineStr"/>
-      <c r="BA90" t="inlineStr"/>
-      <c r="BB90" t="inlineStr"/>
-      <c r="BC90" t="inlineStr"/>
+      <c r="BA90" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB90" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC90" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD90" t="inlineStr"/>
       <c r="BE90" t="inlineStr"/>
       <c r="BF90" t="inlineStr"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 14:46)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4184,7 +4184,7 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -4227,42 +4227,16 @@
       </c>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
-      <c r="AG22" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AH22" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI22" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AJ22" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK22" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AL22" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
       <c r="AM22" t="inlineStr"/>
-      <c r="AN22" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
       <c r="AQ22" t="inlineStr"/>
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
@@ -4273,17 +4247,9 @@
       <c r="AX22" t="inlineStr"/>
       <c r="AY22" t="inlineStr"/>
       <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB22" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC22" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
       <c r="BD22" t="inlineStr"/>
       <c r="BE22" t="inlineStr"/>
       <c r="BF22" t="inlineStr"/>
@@ -8058,7 +8024,7 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
@@ -8101,42 +8067,16 @@
       </c>
       <c r="AE43" t="inlineStr"/>
       <c r="AF43" t="inlineStr"/>
-      <c r="AG43" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AH43" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI43" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AJ43" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK43" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AL43" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr"/>
+      <c r="AK43" t="inlineStr"/>
+      <c r="AL43" t="inlineStr"/>
       <c r="AM43" t="inlineStr"/>
-      <c r="AN43" s="1" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AO43" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP43" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN43" t="inlineStr"/>
+      <c r="AO43" t="inlineStr"/>
+      <c r="AP43" t="inlineStr"/>
       <c r="AQ43" t="inlineStr"/>
       <c r="AR43" t="inlineStr"/>
       <c r="AS43" t="inlineStr"/>
@@ -8147,17 +8087,9 @@
       <c r="AX43" t="inlineStr"/>
       <c r="AY43" t="inlineStr"/>
       <c r="AZ43" t="inlineStr"/>
-      <c r="BA43" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB43" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC43" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA43" t="inlineStr"/>
+      <c r="BB43" t="inlineStr"/>
+      <c r="BC43" t="inlineStr"/>
       <c r="BD43" t="inlineStr"/>
       <c r="BE43" t="inlineStr"/>
       <c r="BF43" t="inlineStr"/>
@@ -10854,7 +10786,7 @@
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S58" t="inlineStr"/>
@@ -10897,42 +10829,16 @@
       </c>
       <c r="AE58" t="inlineStr"/>
       <c r="AF58" t="inlineStr"/>
-      <c r="AG58" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH58" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI58" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ58" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK58" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL58" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
+      <c r="AJ58" t="inlineStr"/>
+      <c r="AK58" t="inlineStr"/>
+      <c r="AL58" t="inlineStr"/>
       <c r="AM58" t="inlineStr"/>
-      <c r="AN58" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO58" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP58" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN58" t="inlineStr"/>
+      <c r="AO58" t="inlineStr"/>
+      <c r="AP58" t="inlineStr"/>
       <c r="AQ58" t="inlineStr"/>
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
@@ -10943,17 +10849,9 @@
       <c r="AX58" t="inlineStr"/>
       <c r="AY58" t="inlineStr"/>
       <c r="AZ58" t="inlineStr"/>
-      <c r="BA58" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB58" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC58" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA58" t="inlineStr"/>
+      <c r="BB58" t="inlineStr"/>
+      <c r="BC58" t="inlineStr"/>
       <c r="BD58" t="inlineStr"/>
       <c r="BE58" t="inlineStr"/>
       <c r="BF58" t="inlineStr"/>
@@ -11032,7 +10930,7 @@
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
@@ -11075,42 +10973,16 @@
       </c>
       <c r="AE59" t="inlineStr"/>
       <c r="AF59" t="inlineStr"/>
-      <c r="AG59" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH59" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI59" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ59" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK59" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL59" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
+      <c r="AJ59" t="inlineStr"/>
+      <c r="AK59" t="inlineStr"/>
+      <c r="AL59" t="inlineStr"/>
       <c r="AM59" t="inlineStr"/>
-      <c r="AN59" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO59" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP59" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN59" t="inlineStr"/>
+      <c r="AO59" t="inlineStr"/>
+      <c r="AP59" t="inlineStr"/>
       <c r="AQ59" t="inlineStr"/>
       <c r="AR59" t="inlineStr"/>
       <c r="AS59" t="inlineStr"/>
@@ -11121,17 +10993,9 @@
       <c r="AX59" t="inlineStr"/>
       <c r="AY59" t="inlineStr"/>
       <c r="AZ59" t="inlineStr"/>
-      <c r="BA59" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB59" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC59" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA59" t="inlineStr"/>
+      <c r="BB59" t="inlineStr"/>
+      <c r="BC59" t="inlineStr"/>
       <c r="BD59" t="inlineStr"/>
       <c r="BE59" t="inlineStr"/>
       <c r="BF59" t="inlineStr"/>
@@ -11416,7 +11280,7 @@
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S61" t="inlineStr"/>
@@ -11459,42 +11323,16 @@
       </c>
       <c r="AE61" t="inlineStr"/>
       <c r="AF61" t="inlineStr"/>
-      <c r="AG61" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH61" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI61" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ61" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK61" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL61" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
+      <c r="AJ61" t="inlineStr"/>
+      <c r="AK61" t="inlineStr"/>
+      <c r="AL61" t="inlineStr"/>
       <c r="AM61" t="inlineStr"/>
-      <c r="AN61" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO61" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP61" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN61" t="inlineStr"/>
+      <c r="AO61" t="inlineStr"/>
+      <c r="AP61" t="inlineStr"/>
       <c r="AQ61" t="inlineStr"/>
       <c r="AR61" t="inlineStr"/>
       <c r="AS61" t="inlineStr"/>
@@ -11505,17 +11343,9 @@
       <c r="AX61" t="inlineStr"/>
       <c r="AY61" t="inlineStr"/>
       <c r="AZ61" t="inlineStr"/>
-      <c r="BA61" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB61" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC61" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA61" t="inlineStr"/>
+      <c r="BB61" t="inlineStr"/>
+      <c r="BC61" t="inlineStr"/>
       <c r="BD61" t="inlineStr"/>
       <c r="BE61" t="inlineStr"/>
       <c r="BF61" t="inlineStr"/>
@@ -11978,7 +11808,7 @@
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S64" t="inlineStr"/>
@@ -12021,42 +11851,16 @@
       </c>
       <c r="AE64" t="inlineStr"/>
       <c r="AF64" t="inlineStr"/>
-      <c r="AG64" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH64" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI64" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ64" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK64" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL64" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
+      <c r="AJ64" t="inlineStr"/>
+      <c r="AK64" t="inlineStr"/>
+      <c r="AL64" t="inlineStr"/>
       <c r="AM64" t="inlineStr"/>
-      <c r="AN64" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO64" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP64" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN64" t="inlineStr"/>
+      <c r="AO64" t="inlineStr"/>
+      <c r="AP64" t="inlineStr"/>
       <c r="AQ64" t="inlineStr"/>
       <c r="AR64" t="inlineStr"/>
       <c r="AS64" t="inlineStr"/>
@@ -12067,17 +11871,9 @@
       <c r="AX64" t="inlineStr"/>
       <c r="AY64" t="inlineStr"/>
       <c r="AZ64" t="inlineStr"/>
-      <c r="BA64" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB64" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC64" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA64" t="inlineStr"/>
+      <c r="BB64" t="inlineStr"/>
+      <c r="BC64" t="inlineStr"/>
       <c r="BD64" t="inlineStr"/>
       <c r="BE64" t="inlineStr"/>
       <c r="BF64" t="inlineStr"/>
@@ -13132,7 +12928,7 @@
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S70" t="inlineStr"/>
@@ -13175,42 +12971,16 @@
       </c>
       <c r="AE70" t="inlineStr"/>
       <c r="AF70" t="inlineStr"/>
-      <c r="AG70" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH70" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI70" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ70" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK70" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL70" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr"/>
+      <c r="AJ70" t="inlineStr"/>
+      <c r="AK70" t="inlineStr"/>
+      <c r="AL70" t="inlineStr"/>
       <c r="AM70" t="inlineStr"/>
-      <c r="AN70" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO70" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP70" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN70" t="inlineStr"/>
+      <c r="AO70" t="inlineStr"/>
+      <c r="AP70" t="inlineStr"/>
       <c r="AQ70" t="inlineStr"/>
       <c r="AR70" t="inlineStr"/>
       <c r="AS70" t="inlineStr"/>
@@ -13221,17 +12991,9 @@
       <c r="AX70" t="inlineStr"/>
       <c r="AY70" t="inlineStr"/>
       <c r="AZ70" t="inlineStr"/>
-      <c r="BA70" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB70" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC70" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA70" t="inlineStr"/>
+      <c r="BB70" t="inlineStr"/>
+      <c r="BC70" t="inlineStr"/>
       <c r="BD70" t="inlineStr"/>
       <c r="BE70" t="inlineStr"/>
       <c r="BF70" t="inlineStr"/>
@@ -13908,7 +13670,7 @@
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S75" t="inlineStr"/>
@@ -13951,42 +13713,16 @@
       </c>
       <c r="AE75" t="inlineStr"/>
       <c r="AF75" t="inlineStr"/>
-      <c r="AG75" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH75" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI75" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ75" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK75" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL75" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG75" t="inlineStr"/>
+      <c r="AH75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr"/>
+      <c r="AJ75" t="inlineStr"/>
+      <c r="AK75" t="inlineStr"/>
+      <c r="AL75" t="inlineStr"/>
       <c r="AM75" t="inlineStr"/>
-      <c r="AN75" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO75" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP75" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN75" t="inlineStr"/>
+      <c r="AO75" t="inlineStr"/>
+      <c r="AP75" t="inlineStr"/>
       <c r="AQ75" t="inlineStr"/>
       <c r="AR75" t="inlineStr"/>
       <c r="AS75" t="inlineStr"/>
@@ -13997,17 +13733,9 @@
       <c r="AX75" t="inlineStr"/>
       <c r="AY75" t="inlineStr"/>
       <c r="AZ75" t="inlineStr"/>
-      <c r="BA75" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB75" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC75" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA75" t="inlineStr"/>
+      <c r="BB75" t="inlineStr"/>
+      <c r="BC75" t="inlineStr"/>
       <c r="BD75" t="inlineStr"/>
       <c r="BE75" t="inlineStr"/>
       <c r="BF75" t="inlineStr"/>
@@ -14086,7 +13814,7 @@
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S76" t="inlineStr"/>
@@ -14129,42 +13857,16 @@
       </c>
       <c r="AE76" t="inlineStr"/>
       <c r="AF76" t="inlineStr"/>
-      <c r="AG76" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH76" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI76" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ76" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK76" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL76" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG76" t="inlineStr"/>
+      <c r="AH76" t="inlineStr"/>
+      <c r="AI76" t="inlineStr"/>
+      <c r="AJ76" t="inlineStr"/>
+      <c r="AK76" t="inlineStr"/>
+      <c r="AL76" t="inlineStr"/>
       <c r="AM76" t="inlineStr"/>
-      <c r="AN76" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO76" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP76" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN76" t="inlineStr"/>
+      <c r="AO76" t="inlineStr"/>
+      <c r="AP76" t="inlineStr"/>
       <c r="AQ76" t="inlineStr"/>
       <c r="AR76" t="inlineStr"/>
       <c r="AS76" t="inlineStr"/>
@@ -14175,17 +13877,9 @@
       <c r="AX76" t="inlineStr"/>
       <c r="AY76" t="inlineStr"/>
       <c r="AZ76" t="inlineStr"/>
-      <c r="BA76" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB76" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC76" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA76" t="inlineStr"/>
+      <c r="BB76" t="inlineStr"/>
+      <c r="BC76" t="inlineStr"/>
       <c r="BD76" t="inlineStr"/>
       <c r="BE76" t="inlineStr"/>
       <c r="BF76" t="inlineStr"/>
@@ -14264,7 +13958,7 @@
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S77" t="inlineStr"/>
@@ -14307,42 +14001,16 @@
       </c>
       <c r="AE77" t="inlineStr"/>
       <c r="AF77" t="inlineStr"/>
-      <c r="AG77" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH77" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI77" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ77" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK77" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL77" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG77" t="inlineStr"/>
+      <c r="AH77" t="inlineStr"/>
+      <c r="AI77" t="inlineStr"/>
+      <c r="AJ77" t="inlineStr"/>
+      <c r="AK77" t="inlineStr"/>
+      <c r="AL77" t="inlineStr"/>
       <c r="AM77" t="inlineStr"/>
-      <c r="AN77" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO77" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP77" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN77" t="inlineStr"/>
+      <c r="AO77" t="inlineStr"/>
+      <c r="AP77" t="inlineStr"/>
       <c r="AQ77" t="inlineStr"/>
       <c r="AR77" t="inlineStr"/>
       <c r="AS77" t="inlineStr"/>
@@ -14353,17 +14021,9 @@
       <c r="AX77" t="inlineStr"/>
       <c r="AY77" t="inlineStr"/>
       <c r="AZ77" t="inlineStr"/>
-      <c r="BA77" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB77" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC77" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA77" t="inlineStr"/>
+      <c r="BB77" t="inlineStr"/>
+      <c r="BC77" t="inlineStr"/>
       <c r="BD77" t="inlineStr"/>
       <c r="BE77" t="inlineStr"/>
       <c r="BF77" t="inlineStr"/>
@@ -14442,7 +14102,7 @@
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S78" t="inlineStr"/>
@@ -14485,42 +14145,16 @@
       </c>
       <c r="AE78" t="inlineStr"/>
       <c r="AF78" t="inlineStr"/>
-      <c r="AG78" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH78" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI78" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ78" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK78" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL78" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG78" t="inlineStr"/>
+      <c r="AH78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr"/>
+      <c r="AJ78" t="inlineStr"/>
+      <c r="AK78" t="inlineStr"/>
+      <c r="AL78" t="inlineStr"/>
       <c r="AM78" t="inlineStr"/>
-      <c r="AN78" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO78" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP78" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN78" t="inlineStr"/>
+      <c r="AO78" t="inlineStr"/>
+      <c r="AP78" t="inlineStr"/>
       <c r="AQ78" t="inlineStr"/>
       <c r="AR78" t="inlineStr"/>
       <c r="AS78" t="inlineStr"/>
@@ -14531,17 +14165,9 @@
       <c r="AX78" t="inlineStr"/>
       <c r="AY78" t="inlineStr"/>
       <c r="AZ78" t="inlineStr"/>
-      <c r="BA78" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB78" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC78" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA78" t="inlineStr"/>
+      <c r="BB78" t="inlineStr"/>
+      <c r="BC78" t="inlineStr"/>
       <c r="BD78" t="inlineStr"/>
       <c r="BE78" t="inlineStr"/>
       <c r="BF78" t="inlineStr"/>
@@ -14620,7 +14246,7 @@
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S79" t="inlineStr"/>
@@ -14663,42 +14289,16 @@
       </c>
       <c r="AE79" t="inlineStr"/>
       <c r="AF79" t="inlineStr"/>
-      <c r="AG79" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH79" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI79" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ79" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK79" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL79" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG79" t="inlineStr"/>
+      <c r="AH79" t="inlineStr"/>
+      <c r="AI79" t="inlineStr"/>
+      <c r="AJ79" t="inlineStr"/>
+      <c r="AK79" t="inlineStr"/>
+      <c r="AL79" t="inlineStr"/>
       <c r="AM79" t="inlineStr"/>
-      <c r="AN79" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO79" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP79" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN79" t="inlineStr"/>
+      <c r="AO79" t="inlineStr"/>
+      <c r="AP79" t="inlineStr"/>
       <c r="AQ79" t="inlineStr"/>
       <c r="AR79" t="inlineStr"/>
       <c r="AS79" t="inlineStr"/>
@@ -14709,17 +14309,9 @@
       <c r="AX79" t="inlineStr"/>
       <c r="AY79" t="inlineStr"/>
       <c r="AZ79" t="inlineStr"/>
-      <c r="BA79" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB79" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC79" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA79" t="inlineStr"/>
+      <c r="BB79" t="inlineStr"/>
+      <c r="BC79" t="inlineStr"/>
       <c r="BD79" t="inlineStr"/>
       <c r="BE79" t="inlineStr"/>
       <c r="BF79" t="inlineStr"/>
@@ -14798,7 +14390,7 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S80" t="inlineStr"/>
@@ -14841,42 +14433,16 @@
       </c>
       <c r="AE80" t="inlineStr"/>
       <c r="AF80" t="inlineStr"/>
-      <c r="AG80" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH80" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI80" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ80" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK80" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL80" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr"/>
+      <c r="AJ80" t="inlineStr"/>
+      <c r="AK80" t="inlineStr"/>
+      <c r="AL80" t="inlineStr"/>
       <c r="AM80" t="inlineStr"/>
-      <c r="AN80" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO80" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP80" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN80" t="inlineStr"/>
+      <c r="AO80" t="inlineStr"/>
+      <c r="AP80" t="inlineStr"/>
       <c r="AQ80" t="inlineStr"/>
       <c r="AR80" t="inlineStr"/>
       <c r="AS80" t="inlineStr"/>
@@ -14887,17 +14453,9 @@
       <c r="AX80" t="inlineStr"/>
       <c r="AY80" t="inlineStr"/>
       <c r="AZ80" t="inlineStr"/>
-      <c r="BA80" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB80" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC80" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA80" t="inlineStr"/>
+      <c r="BB80" t="inlineStr"/>
+      <c r="BC80" t="inlineStr"/>
       <c r="BD80" t="inlineStr"/>
       <c r="BE80" t="inlineStr"/>
       <c r="BF80" t="inlineStr"/>
@@ -15312,7 +14870,7 @@
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S83" t="inlineStr"/>
@@ -15355,42 +14913,16 @@
       </c>
       <c r="AE83" t="inlineStr"/>
       <c r="AF83" t="inlineStr"/>
-      <c r="AG83" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH83" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI83" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ83" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK83" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL83" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG83" t="inlineStr"/>
+      <c r="AH83" t="inlineStr"/>
+      <c r="AI83" t="inlineStr"/>
+      <c r="AJ83" t="inlineStr"/>
+      <c r="AK83" t="inlineStr"/>
+      <c r="AL83" t="inlineStr"/>
       <c r="AM83" t="inlineStr"/>
-      <c r="AN83" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO83" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP83" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN83" t="inlineStr"/>
+      <c r="AO83" t="inlineStr"/>
+      <c r="AP83" t="inlineStr"/>
       <c r="AQ83" t="inlineStr"/>
       <c r="AR83" t="inlineStr"/>
       <c r="AS83" t="inlineStr"/>
@@ -15401,17 +14933,9 @@
       <c r="AX83" t="inlineStr"/>
       <c r="AY83" t="inlineStr"/>
       <c r="AZ83" t="inlineStr"/>
-      <c r="BA83" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB83" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC83" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA83" t="inlineStr"/>
+      <c r="BB83" t="inlineStr"/>
+      <c r="BC83" t="inlineStr"/>
       <c r="BD83" t="inlineStr"/>
       <c r="BE83" t="inlineStr"/>
       <c r="BF83" t="inlineStr"/>
@@ -15490,7 +15014,7 @@
       <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S84" t="inlineStr"/>
@@ -15537,44 +15061,16 @@
           <t>RECOLECTA 3 /07</t>
         </is>
       </c>
-      <c r="AG84" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH84" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI84" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ84" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK84" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL84" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AM84" s="1" t="n">
-        <v>46206</v>
-      </c>
-      <c r="AN84" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO84" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP84" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AG84" t="inlineStr"/>
+      <c r="AH84" t="inlineStr"/>
+      <c r="AI84" t="inlineStr"/>
+      <c r="AJ84" t="inlineStr"/>
+      <c r="AK84" t="inlineStr"/>
+      <c r="AL84" t="inlineStr"/>
+      <c r="AM84" t="inlineStr"/>
+      <c r="AN84" t="inlineStr"/>
+      <c r="AO84" t="inlineStr"/>
+      <c r="AP84" t="inlineStr"/>
       <c r="AQ84" t="inlineStr"/>
       <c r="AR84" t="inlineStr"/>
       <c r="AS84" t="inlineStr"/>
@@ -15585,17 +15081,9 @@
       <c r="AX84" t="inlineStr"/>
       <c r="AY84" t="inlineStr"/>
       <c r="AZ84" t="inlineStr"/>
-      <c r="BA84" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB84" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC84" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA84" t="inlineStr"/>
+      <c r="BB84" t="inlineStr"/>
+      <c r="BC84" t="inlineStr"/>
       <c r="BD84" t="inlineStr"/>
       <c r="BE84" t="inlineStr"/>
       <c r="BF84" t="inlineStr"/>
@@ -15792,7 +15280,7 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S86" t="inlineStr"/>
@@ -15835,42 +15323,16 @@
       </c>
       <c r="AE86" t="inlineStr"/>
       <c r="AF86" t="inlineStr"/>
-      <c r="AG86" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH86" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI86" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ86" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK86" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL86" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG86" t="inlineStr"/>
+      <c r="AH86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr"/>
+      <c r="AJ86" t="inlineStr"/>
+      <c r="AK86" t="inlineStr"/>
+      <c r="AL86" t="inlineStr"/>
       <c r="AM86" t="inlineStr"/>
-      <c r="AN86" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO86" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP86" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN86" t="inlineStr"/>
+      <c r="AO86" t="inlineStr"/>
+      <c r="AP86" t="inlineStr"/>
       <c r="AQ86" t="inlineStr"/>
       <c r="AR86" t="inlineStr"/>
       <c r="AS86" t="inlineStr"/>
@@ -15881,17 +15343,9 @@
       <c r="AX86" t="inlineStr"/>
       <c r="AY86" t="inlineStr"/>
       <c r="AZ86" t="inlineStr"/>
-      <c r="BA86" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB86" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC86" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA86" t="inlineStr"/>
+      <c r="BB86" t="inlineStr"/>
+      <c r="BC86" t="inlineStr"/>
       <c r="BD86" t="inlineStr"/>
       <c r="BE86" t="inlineStr"/>
       <c r="BF86" t="inlineStr"/>
@@ -16418,7 +15872,7 @@
       <c r="Q90" t="inlineStr"/>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestion</t>
         </is>
       </c>
       <c r="S90" t="inlineStr"/>
@@ -16463,34 +15917,14 @@
       <c r="AF90" t="inlineStr"/>
       <c r="AG90" t="inlineStr"/>
       <c r="AH90" t="inlineStr"/>
-      <c r="AI90" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ90" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK90" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL90" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AI90" t="inlineStr"/>
+      <c r="AJ90" t="inlineStr"/>
+      <c r="AK90" t="inlineStr"/>
+      <c r="AL90" t="inlineStr"/>
       <c r="AM90" t="inlineStr"/>
-      <c r="AN90" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AO90" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP90" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="AN90" t="inlineStr"/>
+      <c r="AO90" t="inlineStr"/>
+      <c r="AP90" t="inlineStr"/>
       <c r="AQ90" t="inlineStr"/>
       <c r="AR90" t="inlineStr"/>
       <c r="AS90" t="inlineStr"/>
@@ -16501,17 +15935,9 @@
       <c r="AX90" t="inlineStr"/>
       <c r="AY90" t="inlineStr"/>
       <c r="AZ90" t="inlineStr"/>
-      <c r="BA90" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB90" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC90" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA90" t="inlineStr"/>
+      <c r="BB90" t="inlineStr"/>
+      <c r="BC90" t="inlineStr"/>
       <c r="BD90" t="inlineStr"/>
       <c r="BE90" t="inlineStr"/>
       <c r="BF90" t="inlineStr"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 14:51)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2025,14 +2025,38 @@
           <t>Folio de dev  7984</t>
         </is>
       </c>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="inlineStr"/>
-      <c r="BK8" t="inlineStr"/>
-      <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
-      <c r="BN8" t="inlineStr"/>
+      <c r="BG8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO8" s="1" t="n">
         <v>46199</v>
       </c>
@@ -3511,14 +3535,38 @@
           <t>Folio de  devolucion 34298</t>
         </is>
       </c>
-      <c r="BG17" t="inlineStr"/>
-      <c r="BH17" t="inlineStr"/>
-      <c r="BI17" t="inlineStr"/>
-      <c r="BJ17" t="inlineStr"/>
-      <c r="BK17" t="inlineStr"/>
-      <c r="BL17" t="inlineStr"/>
-      <c r="BM17" t="inlineStr"/>
-      <c r="BN17" t="inlineStr"/>
+      <c r="BG17" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI17" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK17" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM17" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN17" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO17" s="1" t="n">
         <v>46199</v>
       </c>
@@ -4749,14 +4797,38 @@
           <t xml:space="preserve">  Folio de dev 8302</t>
         </is>
       </c>
-      <c r="BG25" t="inlineStr"/>
-      <c r="BH25" t="inlineStr"/>
-      <c r="BI25" t="inlineStr"/>
-      <c r="BJ25" t="inlineStr"/>
-      <c r="BK25" t="inlineStr"/>
-      <c r="BL25" t="inlineStr"/>
-      <c r="BM25" t="inlineStr"/>
-      <c r="BN25" t="inlineStr"/>
+      <c r="BG25" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH25" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI25" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ25" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK25" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL25" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM25" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN25" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO25" s="1" t="n">
         <v>46199</v>
       </c>
@@ -5149,14 +5221,38 @@
           <t>Folio de dev 8341</t>
         </is>
       </c>
-      <c r="BG27" t="inlineStr"/>
-      <c r="BH27" t="inlineStr"/>
-      <c r="BI27" t="inlineStr"/>
-      <c r="BJ27" t="inlineStr"/>
-      <c r="BK27" t="inlineStr"/>
-      <c r="BL27" t="inlineStr"/>
-      <c r="BM27" t="inlineStr"/>
-      <c r="BN27" t="inlineStr"/>
+      <c r="BG27" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH27" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI27" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ27" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK27" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL27" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM27" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN27" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO27" s="1" t="n">
         <v>46199</v>
       </c>
@@ -5363,16 +5459,40 @@
           <t>Folio de dev 35811, se hizo cambio Fisico</t>
         </is>
       </c>
-      <c r="BG28" t="inlineStr"/>
-      <c r="BH28" t="inlineStr"/>
-      <c r="BI28" t="inlineStr"/>
-      <c r="BJ28" t="inlineStr"/>
-      <c r="BK28" t="inlineStr"/>
-      <c r="BL28" t="inlineStr"/>
-      <c r="BM28" t="inlineStr"/>
-      <c r="BN28" t="inlineStr"/>
+      <c r="BG28" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH28" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI28" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ28" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK28" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL28" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM28" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN28" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO28" s="1" t="n">
-        <v>46182</v>
+        <v>46199</v>
       </c>
       <c r="BP28" t="inlineStr">
         <is>
@@ -5380,7 +5500,7 @@
         </is>
       </c>
       <c r="BQ28" s="1" t="n">
-        <v>46182</v>
+        <v>46199</v>
       </c>
       <c r="BR28" t="inlineStr">
         <is>
@@ -5388,7 +5508,7 @@
         </is>
       </c>
       <c r="BS28" s="1" t="n">
-        <v>46182</v>
+        <v>46199</v>
       </c>
       <c r="BT28" t="inlineStr">
         <is>
@@ -5396,7 +5516,7 @@
         </is>
       </c>
       <c r="BU28" s="1" t="n">
-        <v>46182</v>
+        <v>46199</v>
       </c>
       <c r="BV28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 14:53)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -2005,19 +2005,57 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
+      <c r="AQ8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AS8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AU8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AW8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AY8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BA8" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD8" t="inlineStr"/>
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr">

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 15:04)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1907,27 +1907,31 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
+      <c r="AQ7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
+      <c r="AU7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
@@ -5237,27 +5241,31 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ26" t="inlineStr"/>
-      <c r="AR26" t="inlineStr"/>
+      <c r="AQ26" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AS26" t="inlineStr"/>
       <c r="AT26" t="inlineStr"/>
-      <c r="AU26" t="inlineStr"/>
-      <c r="AV26" t="inlineStr"/>
+      <c r="AU26" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AW26" t="inlineStr"/>
       <c r="AX26" t="inlineStr"/>
       <c r="AY26" t="inlineStr"/>
       <c r="AZ26" t="inlineStr"/>
-      <c r="BA26" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB26" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC26" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
       <c r="BD26" t="inlineStr"/>
       <c r="BE26" t="inlineStr"/>
       <c r="BF26" t="inlineStr"/>
@@ -5987,27 +5995,31 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ29" t="inlineStr"/>
-      <c r="AR29" t="inlineStr"/>
+      <c r="AQ29" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AS29" t="inlineStr"/>
       <c r="AT29" t="inlineStr"/>
-      <c r="AU29" t="inlineStr"/>
-      <c r="AV29" t="inlineStr"/>
+      <c r="AU29" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV29" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AW29" t="inlineStr"/>
       <c r="AX29" t="inlineStr"/>
       <c r="AY29" t="inlineStr"/>
       <c r="AZ29" t="inlineStr"/>
-      <c r="BA29" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB29" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC29" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
       <c r="BD29" t="inlineStr"/>
       <c r="BE29" t="inlineStr"/>
       <c r="BF29" t="inlineStr"/>
@@ -10427,27 +10439,31 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ52" t="inlineStr"/>
-      <c r="AR52" t="inlineStr"/>
+      <c r="AQ52" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AS52" t="inlineStr"/>
       <c r="AT52" t="inlineStr"/>
-      <c r="AU52" t="inlineStr"/>
-      <c r="AV52" t="inlineStr"/>
+      <c r="AU52" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV52" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AW52" t="inlineStr"/>
       <c r="AX52" t="inlineStr"/>
       <c r="AY52" t="inlineStr"/>
       <c r="AZ52" t="inlineStr"/>
-      <c r="BA52" s="1" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BB52" t="n">
-        <v>30</v>
-      </c>
-      <c r="BC52" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="BA52" t="inlineStr"/>
+      <c r="BB52" t="inlineStr"/>
+      <c r="BC52" t="inlineStr"/>
       <c r="BD52" t="inlineStr"/>
       <c r="BE52" t="inlineStr"/>
       <c r="BF52" t="inlineStr"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 15:08)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -4404,7 +4404,7 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -8588,7 +8588,7 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -9988,7 +9988,7 @@
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -10170,7 +10170,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -10542,7 +10542,7 @@
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -10722,7 +10722,7 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -11650,7 +11650,7 @@
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -11798,7 +11798,7 @@
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -12194,7 +12194,7 @@
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -12590,7 +12590,7 @@
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -12768,7 +12768,7 @@
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -12916,7 +12916,7 @@
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -13094,7 +13094,7 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -14018,7 +14018,7 @@
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -14402,7 +14402,7 @@
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -14586,7 +14586,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -14764,7 +14764,7 @@
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
@@ -14912,7 +14912,7 @@
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -15060,7 +15060,7 @@
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
@@ -15208,7 +15208,7 @@
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
@@ -15356,7 +15356,7 @@
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
@@ -15504,7 +15504,7 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -16022,7 +16022,7 @@
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
@@ -16170,7 +16170,7 @@
       <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -16440,7 +16440,7 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -17070,7 +17070,7 @@
       <c r="Q90" t="inlineStr"/>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Gestion</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 15:20)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -856,7 +856,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>GESTION</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-MZ013: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 (por Yolanda, 13/07/2026 15:44)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3130,12 +3130,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>VALIDANDO CON EL PROVEEDOR  (FERREMOVIL) | [13/07/2026 15:42 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>VALIDANDO CON EL PROVEEDOR  (FERREMOVIL) | [13/07/2026 15:42 · Reactivación] Etapa 'Gestión' reactivada | [13/07/2026 15:44 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -3186,12 +3186,30 @@
           <t>VALIDANDO CON EL PROVEEDOR  (FERREMOVIL)</t>
         </is>
       </c>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
+      <c r="AG14" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI14" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK14" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" s="2" t="n">
         <v>46179</v>
@@ -3201,7 +3219,7 @@
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr"/>
@@ -3225,7 +3243,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BD14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="inlineStr"/>
@@ -3250,12 +3272,12 @@
       </c>
       <c r="BW14" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX14" t="inlineStr">
         <is>
-          <t>13/07/2026 15:42:28</t>
+          <t>13/07/2026 15:44:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 13/07/2026 16:12)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -829,7 +829,7 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" s="1" t="n">
-        <v>46082</v>
+        <v>46142</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>46149</v>
@@ -841,7 +841,7 @@
         <v>46232</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>46172</v>
+        <v>46232</v>
       </c>
       <c r="M2" t="n">
         <v>74</v>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando Treviño (144 registros, 21/07/2026 09:15)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -870,7 +870,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -3952,7 +3952,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
@@ -6428,7 +6428,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -6826,7 +6826,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -8268,7 +8268,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -8866,7 +8866,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
@@ -9156,7 +9156,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -9548,7 +9548,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -9810,7 +9810,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -10072,7 +10072,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -10330,7 +10330,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -10702,7 +10702,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -12364,7 +12364,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -12778,7 +12778,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -13036,7 +13036,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -13222,7 +13222,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -13378,7 +13378,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -14526,7 +14526,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -14682,7 +14682,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S71" t="inlineStr"/>
@@ -14808,7 +14808,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S72" t="inlineStr"/>
@@ -14934,7 +14934,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -15122,7 +15122,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -15308,7 +15308,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
@@ -15464,7 +15464,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -15620,7 +15620,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
@@ -15776,7 +15776,7 @@
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
@@ -16088,7 +16088,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -16244,7 +16244,7 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S81" t="inlineStr"/>
@@ -16628,7 +16628,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S85" t="inlineStr"/>
@@ -17070,7 +17070,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -17226,7 +17226,7 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S87" t="inlineStr"/>
@@ -17352,7 +17352,7 @@
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S88" t="inlineStr"/>
@@ -17730,7 +17730,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S91" t="inlineStr"/>
@@ -18012,7 +18012,7 @@
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S92" t="inlineStr"/>
@@ -18138,7 +18138,7 @@
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S93" t="inlineStr"/>
@@ -18264,7 +18264,7 @@
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S94" t="inlineStr"/>
@@ -18390,7 +18390,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S95" t="inlineStr"/>
@@ -18516,7 +18516,7 @@
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S96" t="inlineStr"/>
@@ -18642,7 +18642,7 @@
       </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
@@ -18768,7 +18768,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S98" t="inlineStr"/>
@@ -18894,7 +18894,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S99" t="inlineStr"/>
@@ -19020,7 +19020,7 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S100" t="inlineStr"/>
@@ -19146,7 +19146,7 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S101" t="inlineStr"/>
@@ -19272,7 +19272,7 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S102" t="inlineStr"/>
@@ -19398,7 +19398,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S103" t="inlineStr"/>
@@ -19524,7 +19524,7 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S104" t="inlineStr"/>
@@ -19650,7 +19650,7 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S105" t="inlineStr"/>
@@ -19776,7 +19776,7 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S106" t="inlineStr"/>
@@ -19902,7 +19902,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
@@ -20160,7 +20160,7 @@
       </c>
       <c r="R108" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S108" t="inlineStr"/>
@@ -20286,7 +20286,7 @@
       </c>
       <c r="R109" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S109" t="inlineStr"/>
@@ -20412,7 +20412,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
@@ -20538,7 +20538,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S111" t="inlineStr"/>
@@ -20664,7 +20664,7 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S112" t="inlineStr">
@@ -20922,7 +20922,7 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S113" t="inlineStr">
@@ -21180,7 +21180,7 @@
       </c>
       <c r="R114" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
@@ -21438,7 +21438,7 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
@@ -21696,7 +21696,7 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
@@ -21822,7 +21822,7 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S117" t="inlineStr"/>
@@ -21948,7 +21948,7 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S118" t="inlineStr"/>
@@ -22074,7 +22074,7 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S119" t="inlineStr"/>
@@ -22200,7 +22200,7 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S120" t="inlineStr"/>
@@ -22326,7 +22326,7 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S121" t="inlineStr"/>
@@ -22452,7 +22452,7 @@
       </c>
       <c r="R122" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S122" t="inlineStr"/>
@@ -22578,7 +22578,7 @@
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S123" t="inlineStr"/>
@@ -22704,7 +22704,7 @@
       </c>
       <c r="R124" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S124" t="inlineStr"/>
@@ -22956,7 +22956,7 @@
       </c>
       <c r="R126" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S126" t="inlineStr"/>
@@ -23082,7 +23082,7 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S127" t="inlineStr"/>
@@ -23208,7 +23208,7 @@
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S128" t="inlineStr"/>
@@ -23334,7 +23334,7 @@
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S129" t="inlineStr"/>
@@ -23460,7 +23460,7 @@
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S130" t="inlineStr"/>
@@ -23586,7 +23586,7 @@
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S131" t="inlineStr"/>
@@ -23712,7 +23712,7 @@
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S132" t="inlineStr"/>
@@ -23838,7 +23838,7 @@
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S133" t="inlineStr"/>
@@ -23964,7 +23964,7 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S134" t="inlineStr"/>
@@ -24090,7 +24090,7 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S135" t="inlineStr"/>
@@ -24216,7 +24216,7 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S136" t="inlineStr"/>
@@ -24342,7 +24342,7 @@
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S137" t="inlineStr"/>
@@ -24468,7 +24468,7 @@
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S138" t="inlineStr"/>
@@ -24594,7 +24594,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S139" t="inlineStr"/>
@@ -24720,7 +24720,7 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S140" t="inlineStr"/>
@@ -24846,7 +24846,7 @@
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S141" t="inlineStr"/>
@@ -24972,7 +24972,7 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S142" t="inlineStr"/>
@@ -25098,7 +25098,7 @@
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S143" t="inlineStr"/>
@@ -25224,7 +25224,7 @@
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>DESTINO FINAL</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S144" t="inlineStr"/>
@@ -25350,7 +25350,7 @@
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>REPORTE DE RECLAMO</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S145" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ028: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 (por Yolanda, 21/07/2026 10:05)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6092,17 +6092,17 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:05 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Destrucción</t>
+          <t>Recolección</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
@@ -6148,12 +6148,30 @@
           <t>REALIZARA NOTA DE CREDITO PARA LA SALIDA</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr"/>
-      <c r="AH29" t="inlineStr"/>
-      <c r="AI29" t="inlineStr"/>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
-      <c r="AL29" t="inlineStr"/>
+      <c r="AG29" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI29" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK29" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM29" t="inlineStr"/>
       <c r="AN29" s="2" t="n">
         <v>46179</v>
@@ -6163,7 +6181,7 @@
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ29" t="inlineStr">
@@ -6191,7 +6209,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BD29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE29" t="inlineStr"/>
       <c r="BF29" t="inlineStr"/>
       <c r="BG29" t="inlineStr"/>
@@ -6208,7 +6230,9 @@
       <c r="BR29" t="inlineStr"/>
       <c r="BS29" t="inlineStr"/>
       <c r="BT29" t="inlineStr"/>
-      <c r="BU29" t="inlineStr"/>
+      <c r="BU29" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="BV29" t="inlineStr">
         <is>
           <t>NO</t>
@@ -6216,12 +6240,12 @@
       </c>
       <c r="BW29" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX29" t="inlineStr">
         <is>
-          <t>21/07/2026 10:02:53</t>
+          <t>21/07/2026 10:05:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ028: Recolección vencida → cambia a destrucción (por Sistema, 21/07/2026 10:05)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6092,7 +6092,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:05 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
+          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:05 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:05 · Sistema] Recolección vencida → cambia a destrucción</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -6211,10 +6211,14 @@
       </c>
       <c r="BD29" t="inlineStr">
         <is>
-          <t>Recolección</t>
-        </is>
-      </c>
-      <c r="BE29" t="inlineStr"/>
+          <t>Destrucción</t>
+        </is>
+      </c>
+      <c r="BE29" t="inlineStr">
+        <is>
+          <t>Definición de destino final</t>
+        </is>
+      </c>
       <c r="BF29" t="inlineStr"/>
       <c r="BG29" t="inlineStr"/>
       <c r="BH29" t="inlineStr"/>
@@ -6240,12 +6244,12 @@
       </c>
       <c r="BW29" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="BX29" t="inlineStr">
         <is>
-          <t>21/07/2026 10:05:05</t>
+          <t>21/07/2026 10:05:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ028: Modalidad de Destino final corregida a 'Recolección' (por Corrección, 21/07/2026 10:06)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -6092,7 +6092,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:05 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:05 · Sistema] Recolección vencida → cambia a destrucción</t>
+          <t>DESTRUCCION | [21/07/2026 10:02 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:05 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:05 · Sistema] Recolección vencida → cambia a destrucción | [21/07/2026 10:06 · Corrección] Modalidad de Destino final corregida a 'Recolección'</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="BD29" t="inlineStr">
         <is>
-          <t>Destrucción</t>
+          <t>Recolección</t>
         </is>
       </c>
       <c r="BE29" t="inlineStr">
@@ -6244,12 +6244,12 @@
       </c>
       <c r="BW29" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Corrección</t>
         </is>
       </c>
       <c r="BX29" t="inlineStr">
         <is>
-          <t>21/07/2026 10:05:43</t>
+          <t>21/07/2026 10:06:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ039: Etapa 'Gestión' reactivada (por Reactivación, 21/07/2026 10:07)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8286,12 +8286,12 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [21/07/2026 10:07 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -8342,30 +8342,12 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="AG40" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AH40" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI40" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AJ40" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK40" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AL40" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
+      <c r="AJ40" t="inlineStr"/>
+      <c r="AK40" t="inlineStr"/>
+      <c r="AL40" t="inlineStr"/>
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" s="2" t="n">
         <v>46179</v>
@@ -8375,7 +8357,7 @@
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ40" t="inlineStr"/>
@@ -8396,7 +8378,7 @@
       </c>
       <c r="BC40" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BD40" t="inlineStr"/>
@@ -8417,9 +8399,21 @@
       <c r="BS40" t="inlineStr"/>
       <c r="BT40" t="inlineStr"/>
       <c r="BU40" t="inlineStr"/>
-      <c r="BV40" t="inlineStr"/>
-      <c r="BW40" t="inlineStr"/>
-      <c r="BX40" t="inlineStr"/>
+      <c r="BV40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BW40" t="inlineStr">
+        <is>
+          <t>Reactivación</t>
+        </is>
+      </c>
+      <c r="BX40" t="inlineStr">
+        <is>
+          <t>21/07/2026 10:07:28</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ039: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/07/2026 (por Yolanda, 21/07/2026 10:08)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8286,12 +8286,12 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [21/07/2026 10:07 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>DEVOLUCION | [21/07/2026 10:07 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:08 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/07/2026</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -8342,22 +8342,40 @@
           <t>RECOLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="AG40" t="inlineStr"/>
-      <c r="AH40" t="inlineStr"/>
-      <c r="AI40" t="inlineStr"/>
-      <c r="AJ40" t="inlineStr"/>
-      <c r="AK40" t="inlineStr"/>
-      <c r="AL40" t="inlineStr"/>
+      <c r="AG40" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AH40" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI40" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK40" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM40" t="inlineStr"/>
       <c r="AN40" s="2" t="n">
         <v>46179</v>
       </c>
       <c r="AO40" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ40" t="inlineStr"/>
@@ -8381,7 +8399,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BD40" t="inlineStr"/>
+      <c r="BD40" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE40" t="inlineStr"/>
       <c r="BF40" t="inlineStr"/>
       <c r="BG40" t="inlineStr"/>
@@ -8398,7 +8420,9 @@
       <c r="BR40" t="inlineStr"/>
       <c r="BS40" t="inlineStr"/>
       <c r="BT40" t="inlineStr"/>
-      <c r="BU40" t="inlineStr"/>
+      <c r="BU40" s="2" t="n">
+        <v>46229</v>
+      </c>
       <c r="BV40" t="inlineStr">
         <is>
           <t>NO</t>
@@ -8406,12 +8430,12 @@
       </c>
       <c r="BW40" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX40" t="inlineStr">
         <is>
-          <t>21/07/2026 10:07:28</t>
+          <t>21/07/2026 10:08:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB016: Etapa 'Gestión' reactivada (por Reactivación, 21/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13414,12 +13414,12 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -13470,30 +13470,12 @@
           <t>RECLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="AG65" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AH65" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI65" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AJ65" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK65" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AL65" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG65" t="inlineStr"/>
+      <c r="AH65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr"/>
+      <c r="AJ65" t="inlineStr"/>
+      <c r="AK65" t="inlineStr"/>
+      <c r="AL65" t="inlineStr"/>
       <c r="AM65" t="inlineStr"/>
       <c r="AN65" s="2" t="n">
         <v>46199</v>
@@ -13503,7 +13485,7 @@
       </c>
       <c r="AP65" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ65" t="inlineStr"/>
@@ -13518,7 +13500,11 @@
       <c r="AZ65" t="inlineStr"/>
       <c r="BA65" t="inlineStr"/>
       <c r="BB65" t="inlineStr"/>
-      <c r="BC65" t="inlineStr"/>
+      <c r="BC65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD65" t="inlineStr"/>
       <c r="BE65" t="inlineStr"/>
       <c r="BF65" t="inlineStr"/>
@@ -13537,9 +13523,21 @@
       <c r="BS65" t="inlineStr"/>
       <c r="BT65" t="inlineStr"/>
       <c r="BU65" t="inlineStr"/>
-      <c r="BV65" t="inlineStr"/>
-      <c r="BW65" t="inlineStr"/>
-      <c r="BX65" t="inlineStr"/>
+      <c r="BV65" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BW65" t="inlineStr">
+        <is>
+          <t>Reactivación</t>
+        </is>
+      </c>
+      <c r="BX65" t="inlineStr">
+        <is>
+          <t>21/07/2026 10:10:01</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB016: Ajuste manual de fechas en 'Gestión' (por Yolanda, 21/07/2026 10:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13414,7 +13414,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión'</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -13470,8 +13470,14 @@
           <t>RECLECTA EN JULIO</t>
         </is>
       </c>
-      <c r="AG65" t="inlineStr"/>
-      <c r="AH65" t="inlineStr"/>
+      <c r="AG65" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AI65" t="inlineStr"/>
       <c r="AJ65" t="inlineStr"/>
       <c r="AK65" t="inlineStr"/>
@@ -13530,12 +13536,12 @@
       </c>
       <c r="BW65" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX65" t="inlineStr">
         <is>
-          <t>21/07/2026 10:10:01</t>
+          <t>21/07/2026 10:11:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB016: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 (por Yolanda, 21/07/2026 10:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13414,12 +13414,12 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión'</t>
+          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -13487,11 +13487,11 @@
         <v>46199</v>
       </c>
       <c r="AO65" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="AP65" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ65" t="inlineStr"/>
@@ -13511,7 +13511,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BD65" t="inlineStr"/>
+      <c r="BD65" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE65" t="inlineStr"/>
       <c r="BF65" t="inlineStr"/>
       <c r="BG65" t="inlineStr"/>
@@ -13528,7 +13532,9 @@
       <c r="BR65" t="inlineStr"/>
       <c r="BS65" t="inlineStr"/>
       <c r="BT65" t="inlineStr"/>
-      <c r="BU65" t="inlineStr"/>
+      <c r="BU65" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="BV65" t="inlineStr">
         <is>
           <t>NO</t>
@@ -13541,7 +13547,7 @@
       </c>
       <c r="BX65" t="inlineStr">
         <is>
-          <t>21/07/2026 10:11:22</t>
+          <t>21/07/2026 10:11:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB016: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 (por Yolanda, 21/07/2026 10:14)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13414,7 +13414,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
+          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:14 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -13478,10 +13478,22 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AI65" t="inlineStr"/>
-      <c r="AJ65" t="inlineStr"/>
-      <c r="AK65" t="inlineStr"/>
-      <c r="AL65" t="inlineStr"/>
+      <c r="AI65" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK65" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="AL65" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM65" t="inlineStr"/>
       <c r="AN65" s="2" t="n">
         <v>46199</v>
@@ -13547,7 +13559,7 @@
       </c>
       <c r="BX65" t="inlineStr">
         <is>
-          <t>21/07/2026 10:11:50</t>
+          <t>21/07/2026 10:14:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB016: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/07/2026 (por Yolanda, 21/07/2026 10:15)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -13414,7 +13414,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:14 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026</t>
+          <t>DEVOLUCION | [21/07/2026 10:10 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' | [21/07/2026 10:11 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:14 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/06/2026 | [21/07/2026 10:15 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 06/07/2026</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -13471,7 +13471,7 @@
         </is>
       </c>
       <c r="AG65" s="2" t="n">
-        <v>46179</v>
+        <v>46209</v>
       </c>
       <c r="AH65" t="inlineStr">
         <is>
@@ -13479,7 +13479,7 @@
         </is>
       </c>
       <c r="AI65" s="2" t="n">
-        <v>46179</v>
+        <v>46209</v>
       </c>
       <c r="AJ65" t="inlineStr">
         <is>
@@ -13487,7 +13487,7 @@
         </is>
       </c>
       <c r="AK65" s="2" t="n">
-        <v>46179</v>
+        <v>46209</v>
       </c>
       <c r="AL65" t="inlineStr">
         <is>
@@ -13499,7 +13499,7 @@
         <v>46199</v>
       </c>
       <c r="AO65" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="AP65" t="inlineStr">
         <is>
@@ -13545,7 +13545,7 @@
       <c r="BS65" t="inlineStr"/>
       <c r="BT65" t="inlineStr"/>
       <c r="BU65" s="2" t="n">
-        <v>46199</v>
+        <v>46229</v>
       </c>
       <c r="BV65" t="inlineStr">
         <is>
@@ -13559,7 +13559,7 @@
       </c>
       <c r="BX65" t="inlineStr">
         <is>
-          <t>21/07/2026 10:14:21</t>
+          <t>21/07/2026 10:15:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ035: Etapa 'Destino final' reactivada (por Reactivación, 21/07/2026 10:18)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7434,7 +7434,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8345</t>
+          <t>DEVOLUCION 8345 | [21/07/2026 10:18 · Reactivación] Etapa 'Destino final' reactivada</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -7590,46 +7590,28 @@
       <c r="BL36" t="inlineStr"/>
       <c r="BM36" t="inlineStr"/>
       <c r="BN36" t="inlineStr"/>
-      <c r="BO36" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BP36" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BQ36" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BR36" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BS36" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="BT36" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="BO36" t="inlineStr"/>
+      <c r="BP36" t="inlineStr"/>
+      <c r="BQ36" t="inlineStr"/>
+      <c r="BR36" t="inlineStr"/>
+      <c r="BS36" t="inlineStr"/>
+      <c r="BT36" t="inlineStr"/>
       <c r="BU36" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="BV36" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BW36" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX36" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>21/07/2026 10:18:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ035: Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 25/06/2026 (por Yolanda, 21/07/2026 10:19)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7434,12 +7434,12 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8345 | [21/07/2026 10:18 · Reactivación] Etapa 'Destino final' reactivada</t>
+          <t>DEVOLUCION 8345 | [21/07/2026 10:18 · Reactivación] Etapa 'Destino final' reactivada | [21/07/2026 10:19 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 25/06/2026</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -7590,28 +7590,46 @@
       <c r="BL36" t="inlineStr"/>
       <c r="BM36" t="inlineStr"/>
       <c r="BN36" t="inlineStr"/>
-      <c r="BO36" t="inlineStr"/>
-      <c r="BP36" t="inlineStr"/>
-      <c r="BQ36" t="inlineStr"/>
-      <c r="BR36" t="inlineStr"/>
-      <c r="BS36" t="inlineStr"/>
-      <c r="BT36" t="inlineStr"/>
+      <c r="BO36" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="BP36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ36" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="BR36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS36" s="2" t="n">
+        <v>46198</v>
+      </c>
+      <c r="BT36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU36" s="2" t="n">
         <v>46199</v>
       </c>
       <c r="BV36" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW36" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX36" t="inlineStr">
         <is>
-          <t>21/07/2026 10:18:14</t>
+          <t>21/07/2026 10:19:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB013: Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 27/06/2026 (por Yolanda, 21/07/2026 10:20)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -12814,12 +12814,12 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8345</t>
+          <t>DEVOLUCION 8345 | [21/07/2026 10:20 · Yolanda] Ajuste manual de fechas en 'Destino final' · etapa TERMINADA con fecha 27/06/2026</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="BX62" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>21/07/2026 10:20:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ001: Avance en Destino final (por Yolanda, 21/07/2026 11:15)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -868,7 +868,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382</t>
+          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -992,16 +992,30 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
+      <c r="BO2" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BQ2" t="inlineStr"/>
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>21/07/2026 11:15:23</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ001: Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO (por Yolanda, 21/07/2026 11:16)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -868,12 +868,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final</t>
+          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -985,7 +985,7 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr">
         <is>
-          <t>SE REALIZO EL DIA 28/07/2026</t>
+          <t>SE REALIZO EL DIA 28/07/2026, FOL DEV</t>
         </is>
       </c>
       <c r="BG2" t="inlineStr"/>
@@ -1012,10 +1012,20 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
+      <c r="BS2" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW2" t="inlineStr">
         <is>
           <t>Yolanda</t>
@@ -1023,7 +1033,7 @@
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>21/07/2026 11:15:56</t>
+          <t>21/07/2026 11:16:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ002: Etapa 'Destino final' reactivada (por Reactivación, 21/07/2026 11:16)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1100,7 +1100,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>DEVOLUCION  8325</t>
+          <t>DEVOLUCION  8325 | [21/07/2026 11:16 · Reactivación] Etapa 'Destino final' reactivada</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1260,46 +1260,28 @@
       <c r="BL3" t="inlineStr"/>
       <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="inlineStr"/>
-      <c r="BO3" s="2" t="n">
-        <v>46183</v>
-      </c>
-      <c r="BP3" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BQ3" s="2" t="n">
-        <v>46183</v>
-      </c>
-      <c r="BR3" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BS3" s="2" t="n">
-        <v>46183</v>
-      </c>
-      <c r="BT3" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
       <c r="BU3" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>21/07/2026 11:16:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ006: Etapa 'Gestión' reactivada (por Reactivación, 21/07/2026 11:22)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1870,12 +1870,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>DESTRUCCION</t>
+          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1926,30 +1926,12 @@
           <t xml:space="preserve">GARANTIAS DE REGADERAS  SE REALIZA AJUSTE INTERNO </t>
         </is>
       </c>
-      <c r="AG7" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AI7" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="AK7" s="2" t="n">
-        <v>46179</v>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" s="2" t="n">
         <v>46179</v>
@@ -1959,7 +1941,7 @@
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
@@ -1974,21 +1956,19 @@
       </c>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
-      <c r="AU7" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
@@ -2007,9 +1987,21 @@
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
-      <c r="BW7" t="inlineStr"/>
-      <c r="BX7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>Reactivación</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>21/07/2026 11:22:31</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MZ006: Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar (por Yolanda, 21/07/2026 11:23)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1870,12 +1870,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada</t>
+          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 11:23 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1923,25 +1923,43 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GARANTIAS DE REGADERAS  SE REALIZA AJUSTE INTERNO </t>
-        </is>
-      </c>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
+          <t>GARANTIAS DE REGADERAS  SE REALIZA AJUSTE INTERNO</t>
+        </is>
+      </c>
+      <c r="AG7" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI7" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK7" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" s="2" t="n">
         <v>46179</v>
       </c>
       <c r="AO7" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
@@ -1969,7 +1987,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BD7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="inlineStr"/>
@@ -1994,12 +2016,12 @@
       </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>21/07/2026 11:22:31</t>
+          <t>21/07/2026 11:23:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ006: Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final (por Yolanda, 21/07/2026 11:24)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1870,12 +1870,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 11:23 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar</t>
+          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 11:23 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [21/07/2026 11:24 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>Destino final</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Se aplico a la factura xxs</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr"/>
@@ -1978,13 +1978,23 @@
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
+      <c r="AY7" s="2" t="n">
+        <v>46224</v>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BA7" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>45</v>
+      </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD7" t="inlineStr">
@@ -2021,7 +2031,7 @@
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>21/07/2026 11:23:28</t>
+          <t>21/07/2026 11:24:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ006: Etapa 'Cuentas por pagar' reactivada (por Reactivación, 21/07/2026 11:31)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1870,12 +1870,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 11:23 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [21/07/2026 11:24 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final</t>
+          <t>DESTRUCCION | [21/07/2026 11:22 · Reactivación] Etapa 'Gestión' reactivada | [21/07/2026 11:23 · Yolanda] Etapa 2 TERMINADA · Destrucción → pasa a Cuentas por pagar | [21/07/2026 11:24 · Yolanda] Etapa 3 (Cuentas por pagar) TERMINADA → pasa a Destino final | [21/07/2026 11:31 · Reactivación] Etapa 'Cuentas por pagar' reactivada</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1978,14 +1978,8 @@
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
-      <c r="AY7" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
       <c r="BA7" s="2" t="n">
         <v>46232</v>
       </c>
@@ -1994,7 +1988,7 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BD7" t="inlineStr">
@@ -2026,12 +2020,12 @@
       </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
         <is>
-          <t>21/07/2026 11:24:56</t>
+          <t>21/07/2026 11:31:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Folio DC-MZ001: Etapa 'Disposición final' reactivada (por Reactivación, 21/07/2026 12:30)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -868,12 +868,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO</t>
+          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO | [21/07/2026 12:30 · Reactivación] Etapa 'Disposición final' reactivada</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>FINALIZADO</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BD2" t="inlineStr"/>
@@ -996,44 +996,26 @@
       <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr"/>
-      <c r="BO2" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BQ2" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
-      <c r="BS2" s="2" t="n">
-        <v>46224</v>
-      </c>
-      <c r="BT2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Reactivación</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>21/07/2026 11:16:13</t>
+          <t>21/07/2026 12:30:20</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1180,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS3" s="2" t="n">
+      <c r="AS3" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT3" t="inlineStr">
@@ -1446,7 +1428,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS4" s="2" t="n">
+      <c r="AS4" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT4" t="inlineStr">
@@ -2190,7 +2172,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS8" s="2" t="n">
+      <c r="AS8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT8" t="inlineStr">
@@ -2240,7 +2222,7 @@
           <t>Folio de dev  7984</t>
         </is>
       </c>
-      <c r="BG8" s="2" t="n">
+      <c r="BG8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BH8" t="inlineStr">
@@ -2248,7 +2230,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BI8" s="2" t="n">
+      <c r="BI8" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BJ8" t="inlineStr">
@@ -3792,7 +3774,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS17" s="2" t="n">
+      <c r="AS17" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT17" t="inlineStr">
@@ -3846,7 +3828,7 @@
           <t>Folio de  devolucion 34298</t>
         </is>
       </c>
-      <c r="BG17" s="2" t="n">
+      <c r="BG17" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BH17" t="inlineStr">
@@ -3854,7 +3836,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BI17" s="2" t="n">
+      <c r="BI17" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BJ17" t="inlineStr">
@@ -5162,7 +5144,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS25" s="2" t="n">
+      <c r="AS25" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT25" t="inlineStr">
@@ -5212,7 +5194,7 @@
           <t xml:space="preserve">  Folio de dev 8302</t>
         </is>
       </c>
-      <c r="BG25" s="2" t="n">
+      <c r="BG25" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BH25" t="inlineStr">
@@ -5220,7 +5202,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BI25" s="2" t="n">
+      <c r="BI25" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BJ25" t="inlineStr">
@@ -5652,7 +5634,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS27" s="2" t="n">
+      <c r="AS27" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT27" t="inlineStr">
@@ -5702,7 +5684,7 @@
           <t>Folio de dev 8341</t>
         </is>
       </c>
-      <c r="BG27" s="2" t="n">
+      <c r="BG27" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BH27" t="inlineStr">
@@ -5710,7 +5692,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BI27" s="2" t="n">
+      <c r="BI27" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BJ27" t="inlineStr">
@@ -5938,7 +5920,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS28" s="2" t="n">
+      <c r="AS28" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT28" t="inlineStr">
@@ -5988,7 +5970,7 @@
           <t>Folio de dev 35811, se hizo cambio Fisico</t>
         </is>
       </c>
-      <c r="BG28" s="2" t="n">
+      <c r="BG28" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BH28" t="inlineStr">
@@ -5996,7 +5978,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="BI28" s="2" t="n">
+      <c r="BI28" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="BJ28" t="inlineStr">
@@ -6976,7 +6958,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS33" s="2" t="n">
+      <c r="AS33" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT33" t="inlineStr">
@@ -7566,7 +7548,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS36" s="2" t="n">
+      <c r="AS36" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT36" t="inlineStr">
@@ -7828,7 +7810,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS37" s="2" t="n">
+      <c r="AS37" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT37" t="inlineStr">
@@ -9454,7 +9436,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS46" s="2" t="n">
+      <c r="AS46" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT46" t="inlineStr">
@@ -9716,7 +9698,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS47" s="2" t="n">
+      <c r="AS47" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT47" t="inlineStr">
@@ -9978,7 +9960,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS48" s="2" t="n">
+      <c r="AS48" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT48" t="inlineStr">
@@ -10240,7 +10222,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS49" s="2" t="n">
+      <c r="AS49" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT49" t="inlineStr">
@@ -11446,7 +11428,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS55" s="2" t="n">
+      <c r="AS55" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT55" t="inlineStr">
@@ -11704,7 +11686,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS56" s="2" t="n">
+      <c r="AS56" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT56" t="inlineStr">
@@ -11962,7 +11944,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS57" s="2" t="n">
+      <c r="AS57" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT57" t="inlineStr">
@@ -12532,7 +12514,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS60" s="2" t="n">
+      <c r="AS60" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT60" t="inlineStr">
@@ -12946,7 +12928,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS62" s="2" t="n">
+      <c r="AS62" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT62" t="inlineStr">
@@ -13942,7 +13924,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS67" s="2" t="n">
+      <c r="AS67" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT67" t="inlineStr">
@@ -14200,7 +14182,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS68" s="2" t="n">
+      <c r="AS68" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT68" t="inlineStr">
@@ -14458,7 +14440,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS69" s="2" t="n">
+      <c r="AS69" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT69" t="inlineStr">
@@ -16560,7 +16542,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS82" s="2" t="n">
+      <c r="AS82" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT82" t="inlineStr">
@@ -17662,7 +17644,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS89" s="2" t="n">
+      <c r="AS89" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT89" t="inlineStr">
@@ -20092,7 +20074,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS107" s="2" t="n">
+      <c r="AS107" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT107" t="inlineStr">
@@ -20854,7 +20836,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS112" s="2" t="n">
+      <c r="AS112" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT112" t="inlineStr">
@@ -21112,7 +21094,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS113" s="2" t="n">
+      <c r="AS113" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT113" t="inlineStr">
@@ -21370,7 +21352,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS114" s="2" t="n">
+      <c r="AS114" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT114" t="inlineStr">
@@ -21628,7 +21610,7 @@
           <t>Yolanda</t>
         </is>
       </c>
-      <c r="AS115" s="2" t="n">
+      <c r="AS115" s="1" t="n">
         <v>46199</v>
       </c>
       <c r="AT115" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-MZ001: Avance en Disposición final (por Yolanda, 21/07/2026 12:32)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -868,7 +868,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO | [21/07/2026 12:30 · Reactivación] Etapa 'Disposición final' reactivada</t>
+          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO | [21/07/2026 12:30 · Reactivación] Etapa 'Disposición final' reactivada | [21/07/2026 12:32 · Yolanda] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -983,11 +983,7 @@
       </c>
       <c r="BD2" t="inlineStr"/>
       <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>SE REALIZO EL DIA 28/07/2026, FOL DEV</t>
-        </is>
-      </c>
+      <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
@@ -1010,12 +1006,12 @@
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>21/07/2026 12:30:20</t>
+          <t>21/07/2026 12:32:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 21/07/2026 15:32)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1080,7 +1080,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -7438,7 +7438,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -7591,14 +7591,38 @@
           <t>Folio de dev  8345</t>
         </is>
       </c>
-      <c r="BG36" t="inlineStr"/>
-      <c r="BH36" t="inlineStr"/>
-      <c r="BI36" t="inlineStr"/>
-      <c r="BJ36" t="inlineStr"/>
-      <c r="BK36" t="inlineStr"/>
-      <c r="BL36" t="inlineStr"/>
-      <c r="BM36" t="inlineStr"/>
-      <c r="BN36" t="inlineStr"/>
+      <c r="BG36" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI36" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK36" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM36" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN36" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO36" s="1" t="n">
         <v>46198</v>
       </c>
@@ -7710,7 +7734,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -8300,7 +8324,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -8516,7 +8540,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -9336,7 +9360,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -9598,7 +9622,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -9850,7 +9874,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -9860,7 +9884,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -10003,14 +10027,38 @@
           <t>Folio de dev 8274</t>
         </is>
       </c>
-      <c r="BG48" t="inlineStr"/>
-      <c r="BH48" t="inlineStr"/>
-      <c r="BI48" t="inlineStr"/>
-      <c r="BJ48" t="inlineStr"/>
-      <c r="BK48" t="inlineStr"/>
-      <c r="BL48" t="inlineStr"/>
-      <c r="BM48" t="inlineStr"/>
-      <c r="BN48" t="inlineStr"/>
+      <c r="BG48" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH48" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI48" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ48" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK48" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL48" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM48" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN48" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO48" s="1" t="n">
         <v>46199</v>
       </c>
@@ -10122,7 +10170,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -10380,7 +10428,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -10952,7 +11000,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -11140,7 +11188,7 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -11586,7 +11634,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -12414,7 +12462,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -12818,7 +12866,7 @@
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -12971,14 +13019,38 @@
           <t>Folio de dev 8345</t>
         </is>
       </c>
-      <c r="BG62" t="inlineStr"/>
-      <c r="BH62" t="inlineStr"/>
-      <c r="BI62" t="inlineStr"/>
-      <c r="BJ62" t="inlineStr"/>
-      <c r="BK62" t="inlineStr"/>
-      <c r="BL62" t="inlineStr"/>
-      <c r="BM62" t="inlineStr"/>
-      <c r="BN62" t="inlineStr"/>
+      <c r="BG62" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BH62" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI62" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BJ62" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK62" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BL62" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM62" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BN62" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO62" s="1" t="n">
         <v>46200</v>
       </c>
@@ -13428,7 +13500,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -13636,7 +13708,7 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -13824,7 +13896,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -14082,7 +14154,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -14330,7 +14402,7 @@
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -14340,7 +14412,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -14483,14 +14555,38 @@
           <t>Folio de dev 8330-8274</t>
         </is>
       </c>
-      <c r="BG69" t="inlineStr"/>
-      <c r="BH69" t="inlineStr"/>
-      <c r="BI69" t="inlineStr"/>
-      <c r="BJ69" t="inlineStr"/>
-      <c r="BK69" t="inlineStr"/>
-      <c r="BL69" t="inlineStr"/>
-      <c r="BM69" t="inlineStr"/>
-      <c r="BN69" t="inlineStr"/>
+      <c r="BG69" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BH69" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI69" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BJ69" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK69" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BL69" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM69" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BN69" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO69" s="1" t="n">
         <v>46200</v>
       </c>
@@ -14996,7 +15092,7 @@
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -15006,7 +15102,7 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -15054,7 +15150,7 @@
       <c r="AE73" t="inlineStr"/>
       <c r="AF73" t="inlineStr">
         <is>
-          <t>RECOLECTA  24/07</t>
+          <t>RECOLECTA  15/07</t>
         </is>
       </c>
       <c r="AG73" s="1" t="n">
@@ -15082,7 +15178,7 @@
         </is>
       </c>
       <c r="AM73" s="1" t="n">
-        <v>46227</v>
+        <v>46218</v>
       </c>
       <c r="AN73" s="1" t="n">
         <v>46199</v>
@@ -15095,40 +15191,146 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AQ73" t="inlineStr"/>
-      <c r="AR73" t="inlineStr"/>
-      <c r="AS73" t="inlineStr"/>
-      <c r="AT73" t="inlineStr"/>
-      <c r="AU73" t="inlineStr"/>
-      <c r="AV73" t="inlineStr"/>
-      <c r="AW73" t="inlineStr"/>
-      <c r="AX73" t="inlineStr"/>
-      <c r="AY73" t="inlineStr"/>
-      <c r="AZ73" t="inlineStr"/>
-      <c r="BA73" t="inlineStr"/>
-      <c r="BB73" t="inlineStr"/>
-      <c r="BC73" t="inlineStr"/>
-      <c r="BD73" t="inlineStr"/>
-      <c r="BE73" t="inlineStr"/>
-      <c r="BF73" t="inlineStr"/>
-      <c r="BG73" t="inlineStr"/>
-      <c r="BH73" t="inlineStr"/>
-      <c r="BI73" t="inlineStr"/>
-      <c r="BJ73" t="inlineStr"/>
-      <c r="BK73" t="inlineStr"/>
-      <c r="BL73" t="inlineStr"/>
-      <c r="BM73" t="inlineStr"/>
-      <c r="BN73" t="inlineStr"/>
-      <c r="BO73" t="inlineStr"/>
-      <c r="BP73" t="inlineStr"/>
-      <c r="BQ73" t="inlineStr"/>
-      <c r="BR73" t="inlineStr"/>
-      <c r="BS73" t="inlineStr"/>
-      <c r="BT73" t="inlineStr"/>
-      <c r="BU73" t="inlineStr"/>
-      <c r="BV73" t="inlineStr"/>
-      <c r="BW73" t="inlineStr"/>
-      <c r="BX73" t="inlineStr"/>
+      <c r="AQ73" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AS73" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AU73" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AV73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AW73" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AX73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AY73" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="AZ73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BA73" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BB73" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC73" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="BD73" t="inlineStr">
+        <is>
+          <t>Recoleccion</t>
+        </is>
+      </c>
+      <c r="BE73" t="inlineStr">
+        <is>
+          <t>Programada</t>
+        </is>
+      </c>
+      <c r="BF73" t="inlineStr">
+        <is>
+          <t>FOLIO DE DEV 8347</t>
+        </is>
+      </c>
+      <c r="BG73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BH73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BJ73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BL73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BN73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BP73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BR73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS73" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="BT73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BU73" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="BV73" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="BW73" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX73" s="1" t="n">
+        <v>46224</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -15194,7 +15396,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -15536,7 +15738,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -16856,7 +17058,7 @@
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -17958,7 +18160,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S91" t="inlineStr"/>
@@ -18714,7 +18916,7 @@
       </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
@@ -19470,7 +19672,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S103" t="inlineStr"/>
@@ -19848,7 +20050,7 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S106" t="inlineStr"/>
@@ -19974,7 +20176,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
@@ -20736,7 +20938,7 @@
       </c>
       <c r="R112" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S112" t="inlineStr">
@@ -20994,7 +21196,7 @@
       </c>
       <c r="R113" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S113" t="inlineStr">
@@ -21242,7 +21444,7 @@
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -21252,7 +21454,7 @@
       </c>
       <c r="R114" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S114" t="inlineStr">
@@ -21395,14 +21597,38 @@
           <t>Folio de dev  8330</t>
         </is>
       </c>
-      <c r="BG114" t="inlineStr"/>
-      <c r="BH114" t="inlineStr"/>
-      <c r="BI114" t="inlineStr"/>
-      <c r="BJ114" t="inlineStr"/>
-      <c r="BK114" t="inlineStr"/>
-      <c r="BL114" t="inlineStr"/>
-      <c r="BM114" t="inlineStr"/>
-      <c r="BN114" t="inlineStr"/>
+      <c r="BG114" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="BH114" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI114" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="BJ114" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK114" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="BL114" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM114" s="1" t="n">
+        <v>46200</v>
+      </c>
+      <c r="BN114" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO114" s="1" t="n">
         <v>46200</v>
       </c>
@@ -21510,7 +21736,7 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
@@ -22650,7 +22876,7 @@
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S123" t="inlineStr"/>
@@ -23536,7 +23762,7 @@
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S130" t="inlineStr"/>
@@ -23788,7 +24014,7 @@
       </c>
       <c r="R132" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S132" t="inlineStr"/>
@@ -25038,7 +25264,7 @@
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
         <is>
-          <t>TRANSITO</t>
+          <t>TERMINADO</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -25048,67 +25274,221 @@
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>Destino final</t>
-        </is>
-      </c>
-      <c r="S142" t="inlineStr"/>
+          <t>FINALIZADO</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T142" t="inlineStr"/>
       <c r="U142" t="inlineStr"/>
-      <c r="V142" t="inlineStr"/>
-      <c r="W142" t="inlineStr"/>
-      <c r="X142" t="inlineStr"/>
-      <c r="Y142" t="inlineStr"/>
-      <c r="Z142" t="inlineStr"/>
-      <c r="AA142" t="inlineStr"/>
-      <c r="AB142" t="inlineStr"/>
-      <c r="AC142" t="inlineStr"/>
-      <c r="AD142" t="inlineStr"/>
+      <c r="V142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="X142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="Z142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AB142" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="AC142" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD142" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE142" t="inlineStr"/>
       <c r="AF142" t="inlineStr"/>
-      <c r="AG142" t="inlineStr"/>
-      <c r="AH142" t="inlineStr"/>
-      <c r="AI142" t="inlineStr"/>
-      <c r="AJ142" t="inlineStr"/>
-      <c r="AK142" t="inlineStr"/>
-      <c r="AL142" t="inlineStr"/>
-      <c r="AM142" t="inlineStr"/>
-      <c r="AN142" t="inlineStr"/>
-      <c r="AO142" t="inlineStr"/>
-      <c r="AP142" t="inlineStr"/>
-      <c r="AQ142" t="inlineStr"/>
-      <c r="AR142" t="inlineStr"/>
-      <c r="AS142" t="inlineStr"/>
-      <c r="AT142" t="inlineStr"/>
-      <c r="AU142" t="inlineStr"/>
-      <c r="AV142" t="inlineStr"/>
-      <c r="AW142" t="inlineStr"/>
-      <c r="AX142" t="inlineStr"/>
-      <c r="AY142" t="inlineStr"/>
-      <c r="AZ142" t="inlineStr"/>
-      <c r="BA142" t="inlineStr"/>
-      <c r="BB142" t="inlineStr"/>
-      <c r="BC142" t="inlineStr"/>
+      <c r="AG142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="AH142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AI142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="AJ142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AK142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="AL142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AM142" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="AN142" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="AO142" t="n">
+        <v>30</v>
+      </c>
+      <c r="AP142" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="AQ142" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="AR142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AS142" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="AT142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AU142" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="AV142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AW142" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="AX142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AY142" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="AZ142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BA142" s="1" t="n">
+        <v>46250</v>
+      </c>
+      <c r="BB142" t="n">
+        <v>30</v>
+      </c>
+      <c r="BC142" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BD142" t="inlineStr"/>
       <c r="BE142" t="inlineStr"/>
-      <c r="BF142" t="inlineStr"/>
-      <c r="BG142" t="inlineStr"/>
-      <c r="BH142" t="inlineStr"/>
-      <c r="BI142" t="inlineStr"/>
-      <c r="BJ142" t="inlineStr"/>
-      <c r="BK142" t="inlineStr"/>
-      <c r="BL142" t="inlineStr"/>
-      <c r="BM142" t="inlineStr"/>
-      <c r="BN142" t="inlineStr"/>
-      <c r="BO142" t="inlineStr"/>
-      <c r="BP142" t="inlineStr"/>
-      <c r="BQ142" t="inlineStr"/>
-      <c r="BR142" t="inlineStr"/>
-      <c r="BS142" t="inlineStr"/>
-      <c r="BT142" t="inlineStr"/>
-      <c r="BU142" t="inlineStr"/>
-      <c r="BV142" t="inlineStr"/>
-      <c r="BW142" t="inlineStr"/>
-      <c r="BX142" t="inlineStr"/>
+      <c r="BF142" t="inlineStr">
+        <is>
+          <t>Folio de dev 8378</t>
+        </is>
+      </c>
+      <c r="BG142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="BH142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="BJ142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="BL142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM142" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="BN142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO142" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="BP142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ142" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="BR142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS142" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="BT142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BU142" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="BV142" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="BW142" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX142" s="1" t="n">
+        <v>46224.57197916666</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -25300,7 +25680,7 @@
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Destino final</t>
+          <t>Disposición final</t>
         </is>
       </c>
       <c r="S144" t="inlineStr"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por fERNANDO (144 registros, 22/07/2026 08:29)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -3721,7 +3721,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H17" s="1" t="n">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H25" s="1" t="n">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H29" s="1" t="n">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H32" s="1" t="n">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H36" s="1" t="n">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H40" s="1" t="n">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H43" s="1" t="n">
@@ -12113,7 +12113,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H57" s="1" t="n">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H62" s="1" t="n">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H65" s="1" t="n">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H73" s="1" t="n">
@@ -15639,7 +15639,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H74" s="1" t="n">
@@ -17345,7 +17345,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H84" s="1" t="n">
@@ -19229,7 +19229,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H96" s="1" t="n">
@@ -20433,7 +20433,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H104" s="1" t="n">
@@ -20689,7 +20689,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H106" s="1" t="n">
@@ -20907,7 +20907,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H107" s="1" t="n">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H122" s="1" t="n">
@@ -23911,7 +23911,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H125" s="1" t="n">
@@ -24707,7 +24707,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H130" s="1" t="n">
@@ -25529,7 +25529,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H135" s="1" t="n">
@@ -25785,7 +25785,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H137" s="1" t="n">
@@ -26837,7 +26837,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>ROLANDO</t>
+          <t>MYRIAM</t>
         </is>
       </c>
       <c r="H144" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB003: Modalidad de Disposición final corregida a 'Destrucción' (por Corrección, 27/07/2026 13:24)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10994,7 +10994,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [27/07/2026 13:24 · Corrección] Modalidad de Disposición final corregida a 'Destrucción'</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -11113,7 +11113,11 @@
       <c r="BA52" t="inlineStr"/>
       <c r="BB52" t="inlineStr"/>
       <c r="BC52" t="inlineStr"/>
-      <c r="BD52" t="inlineStr"/>
+      <c r="BD52" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE52" t="inlineStr"/>
       <c r="BF52" t="inlineStr"/>
       <c r="BG52" t="inlineStr"/>
@@ -11132,8 +11136,16 @@
       <c r="BT52" t="inlineStr"/>
       <c r="BU52" t="inlineStr"/>
       <c r="BV52" t="inlineStr"/>
-      <c r="BW52" t="inlineStr"/>
-      <c r="BX52" t="inlineStr"/>
+      <c r="BW52" t="inlineStr">
+        <is>
+          <t>Corrección</t>
+        </is>
+      </c>
+      <c r="BX52" t="inlineStr">
+        <is>
+          <t>27/07/2026 13:24:09</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-AB003: Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 26/06/2026 (por Yolanda, 27/07/2026 14:50)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -10994,7 +10994,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [27/07/2026 13:24 · Corrección] Modalidad de Disposición final corregida a 'Destrucción'</t>
+          <t>DEVOLUCION | [27/07/2026 13:24 · Corrección] Modalidad de Disposición final corregida a 'Destrucción' | [27/07/2026 14:50 · Yolanda] Ajuste manual de fechas en 'Gestión' · etapa TERMINADA con fecha 26/06/2026</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -11004,7 +11004,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Recolección</t>
+          <t>Destrucción</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
@@ -11079,7 +11079,7 @@
         <v>46199</v>
       </c>
       <c r="AO52" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="AP52" t="inlineStr">
         <is>
@@ -11138,12 +11138,12 @@
       <c r="BV52" t="inlineStr"/>
       <c r="BW52" t="inlineStr">
         <is>
-          <t>Corrección</t>
+          <t>Yolanda</t>
         </is>
       </c>
       <c r="BX52" t="inlineStr">
         <is>
-          <t>27/07/2026 13:24:09</t>
+          <t>27/07/2026 14:50:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando Treviño (144 registros, 10/08/2026 14:02)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1031,20 +1031,54 @@
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO2" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ2" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS2" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
@@ -1263,22 +1297,56 @@
       <c r="BH3" t="inlineStr"/>
       <c r="BI3" t="inlineStr"/>
       <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>21/07/2026 11:16:37</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>21/07/2026 11:16:37</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO3" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ3" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR3" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS3" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT3" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU3" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW3" t="inlineStr">
@@ -2093,24 +2161,66 @@
           <t>Destrucción</t>
         </is>
       </c>
-      <c r="BG7" t="inlineStr"/>
-      <c r="BH7" t="inlineStr"/>
-      <c r="BI7" t="inlineStr"/>
-      <c r="BJ7" t="inlineStr"/>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
+      <c r="BG7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BI7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BK7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BL7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS7" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW7" t="inlineStr">
@@ -3045,7 +3155,11 @@
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
-      <c r="BC11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD11" t="inlineStr"/>
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
@@ -3098,7 +3212,7 @@
       </c>
       <c r="BV11" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW11" t="inlineStr">
@@ -3469,20 +3583,54 @@
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
       <c r="BJ13" t="inlineStr"/>
-      <c r="BK13" t="inlineStr"/>
-      <c r="BL13" t="inlineStr"/>
-      <c r="BM13" t="inlineStr"/>
-      <c r="BN13" t="inlineStr"/>
-      <c r="BO13" t="inlineStr"/>
-      <c r="BP13" t="inlineStr"/>
-      <c r="BQ13" t="inlineStr"/>
-      <c r="BR13" t="inlineStr"/>
-      <c r="BS13" t="inlineStr"/>
-      <c r="BT13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO13" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ13" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR13" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS13" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW13" t="inlineStr">
@@ -4489,7 +4637,11 @@
       <c r="AZ18" t="inlineStr"/>
       <c r="BA18" t="inlineStr"/>
       <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD18" t="inlineStr"/>
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
@@ -4542,7 +4694,7 @@
       </c>
       <c r="BV18" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW18" t="inlineStr">
@@ -5579,20 +5731,54 @@
       <c r="BH24" t="inlineStr"/>
       <c r="BI24" t="inlineStr"/>
       <c r="BJ24" t="inlineStr"/>
-      <c r="BK24" t="inlineStr"/>
-      <c r="BL24" t="inlineStr"/>
-      <c r="BM24" t="inlineStr"/>
-      <c r="BN24" t="inlineStr"/>
-      <c r="BO24" t="inlineStr"/>
-      <c r="BP24" t="inlineStr"/>
-      <c r="BQ24" t="inlineStr"/>
-      <c r="BR24" t="inlineStr"/>
-      <c r="BS24" t="inlineStr"/>
-      <c r="BT24" t="inlineStr"/>
+      <c r="BK24" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BL24" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM24" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BN24" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO24" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP24" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ24" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR24" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS24" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT24" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU24" t="inlineStr"/>
       <c r="BV24" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW24" t="inlineStr">
@@ -6079,7 +6265,11 @@
       <c r="AZ26" t="inlineStr"/>
       <c r="BA26" t="inlineStr"/>
       <c r="BB26" t="inlineStr"/>
-      <c r="BC26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD26" t="inlineStr"/>
       <c r="BE26" t="inlineStr"/>
       <c r="BF26" t="inlineStr"/>
@@ -6132,7 +6322,7 @@
       </c>
       <c r="BV26" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW26" t="inlineStr">
@@ -6394,7 +6584,7 @@
       </c>
       <c r="BV27" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW27" t="inlineStr">
@@ -6912,7 +7102,7 @@
       <c r="BS29" t="inlineStr"/>
       <c r="BT29" t="inlineStr"/>
       <c r="BU29" s="1" t="n">
-        <v>46199</v>
+        <v>46229</v>
       </c>
       <c r="BV29" t="inlineStr">
         <is>
@@ -7259,7 +7449,11 @@
       <c r="AZ31" t="inlineStr"/>
       <c r="BA31" t="inlineStr"/>
       <c r="BB31" t="inlineStr"/>
-      <c r="BC31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD31" t="inlineStr"/>
       <c r="BE31" t="inlineStr"/>
       <c r="BF31" t="inlineStr"/>
@@ -7312,7 +7506,7 @@
       </c>
       <c r="BV31" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW31" t="inlineStr">
@@ -7531,20 +7725,54 @@
       <c r="BH32" t="inlineStr"/>
       <c r="BI32" t="inlineStr"/>
       <c r="BJ32" t="inlineStr"/>
-      <c r="BK32" t="inlineStr"/>
-      <c r="BL32" t="inlineStr"/>
-      <c r="BM32" t="inlineStr"/>
-      <c r="BN32" t="inlineStr"/>
-      <c r="BO32" t="inlineStr"/>
-      <c r="BP32" t="inlineStr"/>
-      <c r="BQ32" t="inlineStr"/>
-      <c r="BR32" t="inlineStr"/>
-      <c r="BS32" t="inlineStr"/>
-      <c r="BT32" t="inlineStr"/>
+      <c r="BK32" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BL32" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM32" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BN32" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO32" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP32" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ32" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR32" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS32" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT32" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU32" t="inlineStr"/>
       <c r="BV32" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW32" t="inlineStr">
@@ -7763,10 +7991,26 @@
       <c r="BH33" t="inlineStr"/>
       <c r="BI33" t="inlineStr"/>
       <c r="BJ33" t="inlineStr"/>
-      <c r="BK33" t="inlineStr"/>
-      <c r="BL33" t="inlineStr"/>
-      <c r="BM33" t="inlineStr"/>
-      <c r="BN33" t="inlineStr"/>
+      <c r="BK33" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL33" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM33" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN33" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO33" s="1" t="n">
         <v>46199</v>
       </c>
@@ -7796,7 +8040,7 @@
       </c>
       <c r="BV33" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW33" t="inlineStr">
@@ -8013,8 +8257,14 @@
       <c r="BR34" t="inlineStr"/>
       <c r="BS34" t="inlineStr"/>
       <c r="BT34" t="inlineStr"/>
-      <c r="BU34" t="inlineStr"/>
-      <c r="BV34" t="inlineStr"/>
+      <c r="BU34" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BV34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW34" t="inlineStr"/>
       <c r="BX34" t="inlineStr"/>
       <c r="BY34" t="inlineStr"/>
@@ -9113,8 +9363,14 @@
       <c r="BR39" t="inlineStr"/>
       <c r="BS39" t="inlineStr"/>
       <c r="BT39" t="inlineStr"/>
-      <c r="BU39" t="inlineStr"/>
-      <c r="BV39" t="inlineStr"/>
+      <c r="BU39" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="BV39" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW39" t="inlineStr"/>
       <c r="BX39" t="inlineStr"/>
       <c r="BY39" t="inlineStr"/>
@@ -9551,20 +9807,54 @@
       <c r="BH41" t="inlineStr"/>
       <c r="BI41" t="inlineStr"/>
       <c r="BJ41" t="inlineStr"/>
-      <c r="BK41" t="inlineStr"/>
-      <c r="BL41" t="inlineStr"/>
-      <c r="BM41" t="inlineStr"/>
-      <c r="BN41" t="inlineStr"/>
-      <c r="BO41" t="inlineStr"/>
-      <c r="BP41" t="inlineStr"/>
-      <c r="BQ41" t="inlineStr"/>
-      <c r="BR41" t="inlineStr"/>
-      <c r="BS41" t="inlineStr"/>
-      <c r="BT41" t="inlineStr"/>
+      <c r="BK41" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BL41" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM41" t="inlineStr">
+        <is>
+          <t>21/07/2026 12:32:17</t>
+        </is>
+      </c>
+      <c r="BN41" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO41" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP41" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ41" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR41" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS41" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT41" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU41" t="inlineStr"/>
       <c r="BV41" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW41" t="inlineStr">
@@ -9783,8 +10073,14 @@
       <c r="BR42" t="inlineStr"/>
       <c r="BS42" t="inlineStr"/>
       <c r="BT42" t="inlineStr"/>
-      <c r="BU42" t="inlineStr"/>
-      <c r="BV42" t="inlineStr"/>
+      <c r="BU42" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="BV42" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW42" t="inlineStr"/>
       <c r="BX42" t="inlineStr"/>
       <c r="BY42" t="inlineStr"/>
@@ -10477,10 +10773,26 @@
       <c r="BH46" t="inlineStr"/>
       <c r="BI46" t="inlineStr"/>
       <c r="BJ46" t="inlineStr"/>
-      <c r="BK46" t="inlineStr"/>
-      <c r="BL46" t="inlineStr"/>
-      <c r="BM46" t="inlineStr"/>
-      <c r="BN46" t="inlineStr"/>
+      <c r="BK46" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL46" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM46" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN46" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO46" s="1" t="n">
         <v>46199</v>
       </c>
@@ -10510,7 +10822,7 @@
       </c>
       <c r="BV46" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW46" t="inlineStr">
@@ -11609,20 +11921,54 @@
       <c r="BH50" t="inlineStr"/>
       <c r="BI50" t="inlineStr"/>
       <c r="BJ50" t="inlineStr"/>
-      <c r="BK50" t="inlineStr"/>
-      <c r="BL50" t="inlineStr"/>
-      <c r="BM50" t="inlineStr"/>
-      <c r="BN50" t="inlineStr"/>
-      <c r="BO50" t="inlineStr"/>
-      <c r="BP50" t="inlineStr"/>
-      <c r="BQ50" t="inlineStr"/>
-      <c r="BR50" t="inlineStr"/>
-      <c r="BS50" t="inlineStr"/>
-      <c r="BT50" t="inlineStr"/>
+      <c r="BK50" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL50" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM50" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN50" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO50" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP50" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ50" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR50" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS50" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT50" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU50" t="inlineStr"/>
       <c r="BV50" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW50" t="inlineStr">
@@ -12137,8 +12483,14 @@
       <c r="BR52" t="inlineStr"/>
       <c r="BS52" t="inlineStr"/>
       <c r="BT52" t="inlineStr"/>
-      <c r="BU52" t="inlineStr"/>
-      <c r="BV52" t="inlineStr"/>
+      <c r="BU52" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="BV52" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW52" t="inlineStr">
         <is>
           <t>Yolanda</t>
@@ -12651,20 +13003,54 @@
       <c r="BH54" t="inlineStr"/>
       <c r="BI54" t="inlineStr"/>
       <c r="BJ54" t="inlineStr"/>
-      <c r="BK54" t="inlineStr"/>
-      <c r="BL54" t="inlineStr"/>
-      <c r="BM54" t="inlineStr"/>
-      <c r="BN54" t="inlineStr"/>
-      <c r="BO54" t="inlineStr"/>
-      <c r="BP54" t="inlineStr"/>
-      <c r="BQ54" t="inlineStr"/>
-      <c r="BR54" t="inlineStr"/>
-      <c r="BS54" t="inlineStr"/>
-      <c r="BT54" t="inlineStr"/>
+      <c r="BK54" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL54" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM54" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN54" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO54" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP54" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ54" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR54" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS54" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT54" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU54" t="inlineStr"/>
       <c r="BV54" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW54" t="inlineStr">
@@ -13149,10 +13535,26 @@
       <c r="BH56" t="inlineStr"/>
       <c r="BI56" t="inlineStr"/>
       <c r="BJ56" t="inlineStr"/>
-      <c r="BK56" t="inlineStr"/>
-      <c r="BL56" t="inlineStr"/>
-      <c r="BM56" t="inlineStr"/>
-      <c r="BN56" t="inlineStr"/>
+      <c r="BK56" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL56" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM56" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN56" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO56" s="1" t="n">
         <v>46200</v>
       </c>
@@ -13182,7 +13584,7 @@
       </c>
       <c r="BV56" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW56" t="inlineStr">
@@ -13653,7 +14055,11 @@
       <c r="AZ58" t="inlineStr"/>
       <c r="BA58" t="inlineStr"/>
       <c r="BB58" t="inlineStr"/>
-      <c r="BC58" t="inlineStr"/>
+      <c r="BC58" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD58" t="inlineStr"/>
       <c r="BE58" t="inlineStr"/>
       <c r="BF58" t="inlineStr"/>
@@ -13706,7 +14112,7 @@
       </c>
       <c r="BV58" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW58" t="inlineStr">
@@ -13887,7 +14293,11 @@
       <c r="AZ59" t="inlineStr"/>
       <c r="BA59" t="inlineStr"/>
       <c r="BB59" t="inlineStr"/>
-      <c r="BC59" t="inlineStr"/>
+      <c r="BC59" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD59" t="inlineStr"/>
       <c r="BE59" t="inlineStr"/>
       <c r="BF59" t="inlineStr"/>
@@ -13940,7 +14350,7 @@
       </c>
       <c r="BV59" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW59" t="inlineStr">
@@ -14153,10 +14563,26 @@
       <c r="BH60" t="inlineStr"/>
       <c r="BI60" t="inlineStr"/>
       <c r="BJ60" t="inlineStr"/>
-      <c r="BK60" t="inlineStr"/>
-      <c r="BL60" t="inlineStr"/>
-      <c r="BM60" t="inlineStr"/>
-      <c r="BN60" t="inlineStr"/>
+      <c r="BK60" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL60" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM60" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN60" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO60" s="1" t="n">
         <v>46200</v>
       </c>
@@ -14186,7 +14612,7 @@
       </c>
       <c r="BV60" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW60" t="inlineStr">
@@ -15501,20 +15927,54 @@
       <c r="BH66" t="inlineStr"/>
       <c r="BI66" t="inlineStr"/>
       <c r="BJ66" t="inlineStr"/>
-      <c r="BK66" t="inlineStr"/>
-      <c r="BL66" t="inlineStr"/>
-      <c r="BM66" t="inlineStr"/>
-      <c r="BN66" t="inlineStr"/>
-      <c r="BO66" t="inlineStr"/>
-      <c r="BP66" t="inlineStr"/>
-      <c r="BQ66" t="inlineStr"/>
-      <c r="BR66" t="inlineStr"/>
-      <c r="BS66" t="inlineStr"/>
-      <c r="BT66" t="inlineStr"/>
+      <c r="BK66" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL66" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM66" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN66" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO66" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP66" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ66" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR66" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS66" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT66" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU66" t="inlineStr"/>
       <c r="BV66" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW66" t="inlineStr">
@@ -15729,10 +16189,26 @@
       <c r="BH67" t="inlineStr"/>
       <c r="BI67" t="inlineStr"/>
       <c r="BJ67" t="inlineStr"/>
-      <c r="BK67" t="inlineStr"/>
-      <c r="BL67" t="inlineStr"/>
-      <c r="BM67" t="inlineStr"/>
-      <c r="BN67" t="inlineStr"/>
+      <c r="BK67" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL67" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM67" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN67" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO67" s="1" t="n">
         <v>46200</v>
       </c>
@@ -15762,7 +16238,7 @@
       </c>
       <c r="BV67" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW67" t="inlineStr">
@@ -17413,8 +17889,14 @@
       <c r="BR74" t="inlineStr"/>
       <c r="BS74" t="inlineStr"/>
       <c r="BT74" t="inlineStr"/>
-      <c r="BU74" t="inlineStr"/>
-      <c r="BV74" t="inlineStr"/>
+      <c r="BU74" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="BV74" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BW74" t="inlineStr"/>
       <c r="BX74" t="inlineStr"/>
       <c r="BY74" t="inlineStr"/>
@@ -17948,7 +18430,7 @@
       </c>
       <c r="BV76" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW76" t="inlineStr">
@@ -19628,7 +20110,7 @@
       </c>
       <c r="BV84" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW84" t="inlineStr">
@@ -20935,20 +21417,54 @@
       <c r="BH91" t="inlineStr"/>
       <c r="BI91" t="inlineStr"/>
       <c r="BJ91" t="inlineStr"/>
-      <c r="BK91" t="inlineStr"/>
-      <c r="BL91" t="inlineStr"/>
-      <c r="BM91" t="inlineStr"/>
-      <c r="BN91" t="inlineStr"/>
-      <c r="BO91" t="inlineStr"/>
-      <c r="BP91" t="inlineStr"/>
-      <c r="BQ91" t="inlineStr"/>
-      <c r="BR91" t="inlineStr"/>
-      <c r="BS91" t="inlineStr"/>
-      <c r="BT91" t="inlineStr"/>
+      <c r="BK91" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL91" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM91" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN91" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO91" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP91" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ91" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR91" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS91" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT91" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU91" t="inlineStr"/>
       <c r="BV91" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW91" t="inlineStr">
@@ -21757,7 +22273,11 @@
       <c r="AZ95" t="inlineStr"/>
       <c r="BA95" t="inlineStr"/>
       <c r="BB95" t="inlineStr"/>
-      <c r="BC95" t="inlineStr"/>
+      <c r="BC95" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD95" t="inlineStr"/>
       <c r="BE95" t="inlineStr"/>
       <c r="BF95" t="inlineStr"/>
@@ -21810,7 +22330,7 @@
       </c>
       <c r="BV95" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW95" t="inlineStr">
@@ -22225,20 +22745,54 @@
       <c r="BH97" t="inlineStr"/>
       <c r="BI97" t="inlineStr"/>
       <c r="BJ97" t="inlineStr"/>
-      <c r="BK97" t="inlineStr"/>
-      <c r="BL97" t="inlineStr"/>
-      <c r="BM97" t="inlineStr"/>
-      <c r="BN97" t="inlineStr"/>
-      <c r="BO97" t="inlineStr"/>
-      <c r="BP97" t="inlineStr"/>
-      <c r="BQ97" t="inlineStr"/>
-      <c r="BR97" t="inlineStr"/>
-      <c r="BS97" t="inlineStr"/>
-      <c r="BT97" t="inlineStr"/>
+      <c r="BK97" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL97" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM97" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN97" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO97" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP97" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ97" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR97" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS97" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT97" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU97" t="inlineStr"/>
       <c r="BV97" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW97" t="inlineStr">
@@ -22627,7 +23181,11 @@
       <c r="AZ99" t="inlineStr"/>
       <c r="BA99" t="inlineStr"/>
       <c r="BB99" t="inlineStr"/>
-      <c r="BC99" t="inlineStr"/>
+      <c r="BC99" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD99" t="inlineStr"/>
       <c r="BE99" t="inlineStr"/>
       <c r="BF99" t="inlineStr"/>
@@ -22680,7 +23238,7 @@
       </c>
       <c r="BV99" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW99" t="inlineStr">
@@ -22861,7 +23419,11 @@
       <c r="AZ100" t="inlineStr"/>
       <c r="BA100" t="inlineStr"/>
       <c r="BB100" t="inlineStr"/>
-      <c r="BC100" t="inlineStr"/>
+      <c r="BC100" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD100" t="inlineStr"/>
       <c r="BE100" t="inlineStr"/>
       <c r="BF100" t="inlineStr"/>
@@ -22914,7 +23476,7 @@
       </c>
       <c r="BV100" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW100" t="inlineStr">
@@ -23095,7 +23657,11 @@
       <c r="AZ101" t="inlineStr"/>
       <c r="BA101" t="inlineStr"/>
       <c r="BB101" t="inlineStr"/>
-      <c r="BC101" t="inlineStr"/>
+      <c r="BC101" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD101" t="inlineStr"/>
       <c r="BE101" t="inlineStr"/>
       <c r="BF101" t="inlineStr"/>
@@ -23148,7 +23714,7 @@
       </c>
       <c r="BV101" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW101" t="inlineStr">
@@ -23975,7 +24541,11 @@
       <c r="AZ105" t="inlineStr"/>
       <c r="BA105" t="inlineStr"/>
       <c r="BB105" t="inlineStr"/>
-      <c r="BC105" t="inlineStr"/>
+      <c r="BC105" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="BD105" t="inlineStr"/>
       <c r="BE105" t="inlineStr"/>
       <c r="BF105" t="inlineStr"/>
@@ -24028,7 +24598,7 @@
       </c>
       <c r="BV105" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW105" t="inlineStr">
@@ -24237,20 +24807,54 @@
       <c r="BH106" t="inlineStr"/>
       <c r="BI106" t="inlineStr"/>
       <c r="BJ106" t="inlineStr"/>
-      <c r="BK106" t="inlineStr"/>
-      <c r="BL106" t="inlineStr"/>
-      <c r="BM106" t="inlineStr"/>
-      <c r="BN106" t="inlineStr"/>
-      <c r="BO106" t="inlineStr"/>
-      <c r="BP106" t="inlineStr"/>
-      <c r="BQ106" t="inlineStr"/>
-      <c r="BR106" t="inlineStr"/>
-      <c r="BS106" t="inlineStr"/>
-      <c r="BT106" t="inlineStr"/>
+      <c r="BK106" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL106" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM106" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN106" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO106" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP106" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ106" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR106" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS106" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT106" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU106" t="inlineStr"/>
       <c r="BV106" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW106" t="inlineStr">
@@ -24465,10 +25069,26 @@
       <c r="BH107" t="inlineStr"/>
       <c r="BI107" t="inlineStr"/>
       <c r="BJ107" t="inlineStr"/>
-      <c r="BK107" t="inlineStr"/>
-      <c r="BL107" t="inlineStr"/>
-      <c r="BM107" t="inlineStr"/>
-      <c r="BN107" t="inlineStr"/>
+      <c r="BK107" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL107" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM107" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN107" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO107" s="1" t="n">
         <v>46200</v>
       </c>
@@ -24498,7 +25118,7 @@
       </c>
       <c r="BV107" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW107" t="inlineStr">
@@ -25479,10 +26099,26 @@
       <c r="BH112" t="inlineStr"/>
       <c r="BI112" t="inlineStr"/>
       <c r="BJ112" t="inlineStr"/>
-      <c r="BK112" t="inlineStr"/>
-      <c r="BL112" t="inlineStr"/>
-      <c r="BM112" t="inlineStr"/>
-      <c r="BN112" t="inlineStr"/>
+      <c r="BK112" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL112" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM112" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN112" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BO112" s="1" t="n">
         <v>46200</v>
       </c>
@@ -25512,7 +26148,7 @@
       </c>
       <c r="BV112" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW112" t="inlineStr">
@@ -27921,20 +28557,54 @@
       <c r="BH123" t="inlineStr"/>
       <c r="BI123" t="inlineStr"/>
       <c r="BJ123" t="inlineStr"/>
-      <c r="BK123" t="inlineStr"/>
-      <c r="BL123" t="inlineStr"/>
-      <c r="BM123" t="inlineStr"/>
-      <c r="BN123" t="inlineStr"/>
-      <c r="BO123" t="inlineStr"/>
-      <c r="BP123" t="inlineStr"/>
-      <c r="BQ123" t="inlineStr"/>
-      <c r="BR123" t="inlineStr"/>
-      <c r="BS123" t="inlineStr"/>
-      <c r="BT123" t="inlineStr"/>
+      <c r="BK123" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL123" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM123" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN123" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO123" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP123" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ123" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR123" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS123" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT123" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU123" t="inlineStr"/>
       <c r="BV123" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW123" t="inlineStr">
@@ -29409,20 +30079,54 @@
       <c r="BH130" t="inlineStr"/>
       <c r="BI130" t="inlineStr"/>
       <c r="BJ130" t="inlineStr"/>
-      <c r="BK130" t="inlineStr"/>
-      <c r="BL130" t="inlineStr"/>
-      <c r="BM130" t="inlineStr"/>
-      <c r="BN130" t="inlineStr"/>
-      <c r="BO130" t="inlineStr"/>
-      <c r="BP130" t="inlineStr"/>
-      <c r="BQ130" t="inlineStr"/>
-      <c r="BR130" t="inlineStr"/>
-      <c r="BS130" t="inlineStr"/>
-      <c r="BT130" t="inlineStr"/>
+      <c r="BK130" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL130" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM130" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN130" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO130" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP130" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ130" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR130" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS130" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT130" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU130" t="inlineStr"/>
       <c r="BV130" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW130" t="inlineStr">
@@ -32305,20 +33009,54 @@
       <c r="BH144" t="inlineStr"/>
       <c r="BI144" t="inlineStr"/>
       <c r="BJ144" t="inlineStr"/>
-      <c r="BK144" t="inlineStr"/>
-      <c r="BL144" t="inlineStr"/>
-      <c r="BM144" t="inlineStr"/>
-      <c r="BN144" t="inlineStr"/>
-      <c r="BO144" t="inlineStr"/>
-      <c r="BP144" t="inlineStr"/>
-      <c r="BQ144" t="inlineStr"/>
-      <c r="BR144" t="inlineStr"/>
-      <c r="BS144" t="inlineStr"/>
-      <c r="BT144" t="inlineStr"/>
+      <c r="BK144" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BL144" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BM144" t="inlineStr">
+        <is>
+          <t>13/07/2026 13:43:39</t>
+        </is>
+      </c>
+      <c r="BN144" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BO144" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BP144" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BQ144" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BR144" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BS144" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="BT144" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
       <c r="BU144" t="inlineStr"/>
       <c r="BV144" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW144" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-MY034: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por yolanda, 17/08/2026 14:48)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -24730,12 +24730,12 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359</t>
+          <t>DEVOLUCION 8359 | [17/08/2026 14:48 · yolanda] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
@@ -24836,15 +24836,23 @@
       </c>
       <c r="AW106" t="inlineStr"/>
       <c r="AX106" t="inlineStr"/>
-      <c r="AY106" t="inlineStr"/>
-      <c r="AZ106" t="inlineStr"/>
+      <c r="AY106" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ106" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BA106" s="2" t="n">
         <v>46285</v>
       </c>
-      <c r="BB106" t="inlineStr"/>
+      <c r="BB106" t="n">
+        <v>19</v>
+      </c>
       <c r="BC106" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD106" t="inlineStr">
@@ -24910,12 +24918,12 @@
       </c>
       <c r="BW106" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX106" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>17/08/2026 14:48:21</t>
         </is>
       </c>
       <c r="BY106" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JN041: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 17/08/2026 14:49)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -32950,12 +32950,12 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359</t>
+          <t>DEVOLUCION 8359 | [17/08/2026 14:49 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S144" t="inlineStr">
@@ -33046,25 +33046,27 @@
       </c>
       <c r="AS144" t="inlineStr"/>
       <c r="AT144" t="inlineStr"/>
-      <c r="AU144" s="2" t="n">
-        <v>46220</v>
-      </c>
-      <c r="AV144" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU144" t="inlineStr"/>
+      <c r="AV144" t="inlineStr"/>
       <c r="AW144" t="inlineStr"/>
       <c r="AX144" t="inlineStr"/>
-      <c r="AY144" t="inlineStr"/>
-      <c r="AZ144" t="inlineStr"/>
+      <c r="AY144" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ144" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
       <c r="BA144" s="2" t="n">
         <v>46303</v>
       </c>
-      <c r="BB144" t="inlineStr"/>
+      <c r="BB144" t="n">
+        <v>1</v>
+      </c>
       <c r="BC144" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD144" t="inlineStr">
@@ -33130,12 +33132,12 @@
       </c>
       <c r="BW144" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX144" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>17/08/2026 14:49:44</t>
         </is>
       </c>
       <c r="BY144" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ001: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 17/08/2026 14:55)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -898,12 +898,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO | [21/07/2026 12:30 · Reactivación] Etapa 'Disposición final' reactivada | [21/07/2026 12:32 · Yolanda] Avance en Disposición final</t>
+          <t>DEVOLUCION 8382 | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:15 · Yolanda] Avance en Destino final | [21/07/2026 11:16 · Yolanda] Etapa 4 (Destino final) TERMINADA · PROCESO FINALIZADO | [21/07/2026 12:30 · Reactivación] Etapa 'Disposición final' reactivada | [21/07/2026 12:32 · Yolanda] Avance en Disposición final | [17/08/2026 14:55 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -998,25 +998,27 @@
       </c>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
-      <c r="AU2" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
+      <c r="AY2" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
       <c r="BA2" s="2" t="n">
         <v>46232</v>
       </c>
-      <c r="BB2" t="inlineStr"/>
+      <c r="BB2" t="n">
+        <v>72</v>
+      </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD2" t="inlineStr">
@@ -1082,12 +1084,12 @@
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>21/07/2026 12:32:17</t>
+          <t>17/08/2026 14:55:08</t>
         </is>
       </c>
       <c r="BY2" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB001: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 17/08/2026 14:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -11790,12 +11790,12 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382</t>
+          <t>DEVOLUCION 8382 | [17/08/2026 14:56 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -11890,25 +11890,27 @@
       </c>
       <c r="AS50" t="inlineStr"/>
       <c r="AT50" t="inlineStr"/>
-      <c r="AU50" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AV50" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU50" t="inlineStr"/>
+      <c r="AV50" t="inlineStr"/>
       <c r="AW50" t="inlineStr"/>
       <c r="AX50" t="inlineStr"/>
-      <c r="AY50" t="inlineStr"/>
-      <c r="AZ50" t="inlineStr"/>
+      <c r="AY50" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ50" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
       <c r="BA50" s="2" t="n">
         <v>46252</v>
       </c>
-      <c r="BB50" t="inlineStr"/>
+      <c r="BB50" t="n">
+        <v>52</v>
+      </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD50" t="inlineStr">
@@ -11974,12 +11976,12 @@
       </c>
       <c r="BW50" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX50" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>17/08/2026 14:56:19</t>
         </is>
       </c>
       <c r="BY50" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MY001: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 17/08/2026 14:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -21328,12 +21328,12 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8382</t>
+          <t>DEVOLUCION 8382 | [17/08/2026 14:56 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
@@ -21424,25 +21424,27 @@
       </c>
       <c r="AS91" t="inlineStr"/>
       <c r="AT91" t="inlineStr"/>
-      <c r="AU91" s="2" t="n">
-        <v>46220</v>
-      </c>
-      <c r="AV91" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU91" t="inlineStr"/>
+      <c r="AV91" t="inlineStr"/>
       <c r="AW91" t="inlineStr"/>
       <c r="AX91" t="inlineStr"/>
-      <c r="AY91" t="inlineStr"/>
-      <c r="AZ91" t="inlineStr"/>
+      <c r="AY91" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ91" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
       <c r="BA91" s="2" t="n">
         <v>46285</v>
       </c>
-      <c r="BB91" t="inlineStr"/>
+      <c r="BB91" t="n">
+        <v>19</v>
+      </c>
       <c r="BC91" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD91" t="inlineStr">
@@ -21508,12 +21510,12 @@
       </c>
       <c r="BW91" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX91" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>17/08/2026 14:56:53</t>
         </is>
       </c>
       <c r="BY91" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ032: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 17/08/2026 14:59)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -7872,12 +7872,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8335</t>
+          <t>DEVOLUCION 8335 | [17/08/2026 14:59 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -7972,25 +7972,27 @@
       </c>
       <c r="AS33" t="inlineStr"/>
       <c r="AT33" t="inlineStr"/>
-      <c r="AU33" s="2" t="n">
-        <v>46199</v>
-      </c>
-      <c r="AV33" t="inlineStr">
-        <is>
-          <t>Yolanda</t>
-        </is>
-      </c>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
       <c r="AW33" t="inlineStr"/>
       <c r="AX33" t="inlineStr"/>
-      <c r="AY33" t="inlineStr"/>
-      <c r="AZ33" t="inlineStr"/>
+      <c r="AY33" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="AZ33" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
       <c r="BA33" s="2" t="n">
         <v>46232</v>
       </c>
-      <c r="BB33" t="inlineStr"/>
+      <c r="BB33" t="n">
+        <v>72</v>
+      </c>
       <c r="BC33" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD33" t="inlineStr">
@@ -8058,12 +8060,12 @@
       </c>
       <c r="BW33" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX33" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>17/08/2026 14:59:16</t>
         </is>
       </c>
       <c r="BY33" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ002: Avance en Cuentas por pagar (por Fernando, 17/08/2026 17:33)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CD145"/>
+  <dimension ref="A1:CE145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -832,6 +832,11 @@
       <c r="CD1" t="inlineStr">
         <is>
           <t>ETAPA PREVIA CUARENTENA</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>E3 FOLIO DEVOLUCION AJUSTE</t>
         </is>
       </c>
     </row>
@@ -1098,6 +1103,7 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr"/>
       <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -1162,7 +1168,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>DEVOLUCION  8325 | [21/07/2026 11:16 · Reactivación] Etapa 'Destino final' reactivada</t>
+          <t>DEVOLUCION  8325 | [21/07/2026 11:16 · Reactivación] Etapa 'Destino final' reactivada | [17/08/2026 17:33 · Fernando] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1348,12 +1354,12 @@
       </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Reactivación</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>21/07/2026 11:16:37</t>
+          <t>17/08/2026 17:33:02</t>
         </is>
       </c>
       <c r="BY3" t="inlineStr"/>
@@ -1362,6 +1368,11 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr"/>
       <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr">
+        <is>
+          <t>3834</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -1658,6 +1669,7 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr"/>
       <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1810,6 +1822,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1962,6 +1975,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -2236,6 +2250,7 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr"/>
       <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -2528,6 +2543,7 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr"/>
       <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -2830,6 +2846,7 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr"/>
       <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -2982,6 +2999,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -3230,6 +3248,7 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr"/>
       <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -3382,6 +3401,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -3646,6 +3666,7 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr"/>
       <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -3860,6 +3881,7 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr"/>
       <c r="CD14" t="inlineStr"/>
+      <c r="CE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -4012,6 +4034,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -4164,6 +4187,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -4460,6 +4484,7 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr"/>
       <c r="CD17" t="inlineStr"/>
+      <c r="CE17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -4724,6 +4749,7 @@
           <t>Cuentas por pagar</t>
         </is>
       </c>
+      <c r="CE18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -4876,6 +4902,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -5028,6 +5055,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -5180,6 +5208,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -5390,6 +5419,7 @@
       <c r="CB22" t="inlineStr"/>
       <c r="CC22" t="inlineStr"/>
       <c r="CD22" t="inlineStr"/>
+      <c r="CE22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -5542,6 +5572,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -5806,6 +5837,7 @@
       <c r="CB24" t="inlineStr"/>
       <c r="CC24" t="inlineStr"/>
       <c r="CD24" t="inlineStr"/>
+      <c r="CE24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -6098,6 +6130,7 @@
       <c r="CB25" t="inlineStr"/>
       <c r="CC25" t="inlineStr"/>
       <c r="CD25" t="inlineStr"/>
+      <c r="CE25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -6350,6 +6383,7 @@
       <c r="CB26" t="inlineStr"/>
       <c r="CC26" t="inlineStr"/>
       <c r="CD26" t="inlineStr"/>
+      <c r="CE26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -6614,6 +6648,7 @@
       <c r="CB27" t="inlineStr"/>
       <c r="CC27" t="inlineStr"/>
       <c r="CD27" t="inlineStr"/>
+      <c r="CE27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -6910,6 +6945,7 @@
       <c r="CB28" t="inlineStr"/>
       <c r="CC28" t="inlineStr"/>
       <c r="CD28" t="inlineStr"/>
+      <c r="CE28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -7136,6 +7172,7 @@
       <c r="CB29" t="inlineStr"/>
       <c r="CC29" t="inlineStr"/>
       <c r="CD29" t="inlineStr"/>
+      <c r="CE29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -7288,6 +7325,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -7536,6 +7574,7 @@
       <c r="CB31" t="inlineStr"/>
       <c r="CC31" t="inlineStr"/>
       <c r="CD31" t="inlineStr"/>
+      <c r="CE31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -7808,6 +7847,7 @@
       <c r="CB32" t="inlineStr"/>
       <c r="CC32" t="inlineStr"/>
       <c r="CD32" t="inlineStr"/>
+      <c r="CE32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -8074,6 +8114,7 @@
       <c r="CB33" t="inlineStr"/>
       <c r="CC33" t="inlineStr"/>
       <c r="CD33" t="inlineStr"/>
+      <c r="CE33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -8288,6 +8329,7 @@
       <c r="CB34" t="inlineStr"/>
       <c r="CC34" t="inlineStr"/>
       <c r="CD34" t="inlineStr"/>
+      <c r="CE34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -8440,6 +8482,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -8732,6 +8775,7 @@
       <c r="CB36" t="inlineStr"/>
       <c r="CC36" t="inlineStr"/>
       <c r="CD36" t="inlineStr"/>
+      <c r="CE36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -9028,6 +9072,7 @@
       <c r="CB37" t="inlineStr"/>
       <c r="CC37" t="inlineStr"/>
       <c r="CD37" t="inlineStr"/>
+      <c r="CE37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -9180,6 +9225,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -9394,6 +9440,7 @@
       <c r="CB39" t="inlineStr"/>
       <c r="CC39" t="inlineStr"/>
       <c r="CD39" t="inlineStr"/>
+      <c r="CE39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -9620,6 +9667,7 @@
       <c r="CB40" t="inlineStr"/>
       <c r="CC40" t="inlineStr"/>
       <c r="CD40" t="inlineStr"/>
+      <c r="CE40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -9884,6 +9932,7 @@
       <c r="CB41" t="inlineStr"/>
       <c r="CC41" t="inlineStr"/>
       <c r="CD41" t="inlineStr"/>
+      <c r="CE41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -10100,6 +10149,7 @@
       <c r="CB42" t="inlineStr"/>
       <c r="CC42" t="inlineStr"/>
       <c r="CD42" t="inlineStr"/>
+      <c r="CE42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -10280,6 +10330,7 @@
           <t>Gestión</t>
         </is>
       </c>
+      <c r="CE43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -10432,6 +10483,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -10584,6 +10636,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -10848,6 +10901,7 @@
       <c r="CB46" t="inlineStr"/>
       <c r="CC46" t="inlineStr"/>
       <c r="CD46" t="inlineStr"/>
+      <c r="CE46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -11144,6 +11198,7 @@
       <c r="CB47" t="inlineStr"/>
       <c r="CC47" t="inlineStr"/>
       <c r="CD47" t="inlineStr"/>
+      <c r="CE47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -11436,6 +11491,7 @@
       <c r="CB48" t="inlineStr"/>
       <c r="CC48" t="inlineStr"/>
       <c r="CD48" t="inlineStr"/>
+      <c r="CE48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -11732,6 +11788,7 @@
       <c r="CB49" t="inlineStr"/>
       <c r="CC49" t="inlineStr"/>
       <c r="CD49" t="inlineStr"/>
+      <c r="CE49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -11992,6 +12049,7 @@
       <c r="CB50" t="inlineStr"/>
       <c r="CC50" t="inlineStr"/>
       <c r="CD50" t="inlineStr"/>
+      <c r="CE50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -12284,6 +12342,7 @@
       <c r="CB51" t="inlineStr"/>
       <c r="CC51" t="inlineStr"/>
       <c r="CD51" t="inlineStr"/>
+      <c r="CE51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -12512,6 +12571,7 @@
       <c r="CB52" t="inlineStr"/>
       <c r="CC52" t="inlineStr"/>
       <c r="CD52" t="inlineStr"/>
+      <c r="CE52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -12810,6 +12870,7 @@
       <c r="CB53" t="inlineStr"/>
       <c r="CC53" t="inlineStr"/>
       <c r="CD53" t="inlineStr"/>
+      <c r="CE53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -13070,6 +13131,7 @@
       <c r="CB54" t="inlineStr"/>
       <c r="CC54" t="inlineStr"/>
       <c r="CD54" t="inlineStr"/>
+      <c r="CE54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -13340,6 +13402,7 @@
       <c r="CB55" t="inlineStr"/>
       <c r="CC55" t="inlineStr"/>
       <c r="CD55" t="inlineStr"/>
+      <c r="CE55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -13600,6 +13663,7 @@
       <c r="CB56" t="inlineStr"/>
       <c r="CC56" t="inlineStr"/>
       <c r="CD56" t="inlineStr"/>
+      <c r="CE56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -13888,6 +13952,7 @@
       <c r="CB57" t="inlineStr"/>
       <c r="CC57" t="inlineStr"/>
       <c r="CD57" t="inlineStr"/>
+      <c r="CE57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -14128,6 +14193,7 @@
       <c r="CB58" t="inlineStr"/>
       <c r="CC58" t="inlineStr"/>
       <c r="CD58" t="inlineStr"/>
+      <c r="CE58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -14368,6 +14434,7 @@
       <c r="CB59" t="inlineStr"/>
       <c r="CC59" t="inlineStr"/>
       <c r="CD59" t="inlineStr"/>
+      <c r="CE59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -14628,6 +14695,7 @@
       <c r="CB60" t="inlineStr"/>
       <c r="CC60" t="inlineStr"/>
       <c r="CD60" t="inlineStr"/>
+      <c r="CE60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -14834,6 +14902,7 @@
       <c r="CB61" t="inlineStr"/>
       <c r="CC61" t="inlineStr"/>
       <c r="CD61" t="inlineStr"/>
+      <c r="CE61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -15122,6 +15191,7 @@
       <c r="CB62" t="inlineStr"/>
       <c r="CC62" t="inlineStr"/>
       <c r="CD62" t="inlineStr"/>
+      <c r="CE62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -15346,6 +15416,7 @@
           <t>Disposición final</t>
         </is>
       </c>
+      <c r="CE63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -15522,6 +15593,7 @@
           <t>Gestión</t>
         </is>
       </c>
+      <c r="CE64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -15740,6 +15812,7 @@
       <c r="CB65" t="inlineStr"/>
       <c r="CC65" t="inlineStr"/>
       <c r="CD65" t="inlineStr"/>
+      <c r="CE65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -16000,6 +16073,7 @@
       <c r="CB66" t="inlineStr"/>
       <c r="CC66" t="inlineStr"/>
       <c r="CD66" t="inlineStr"/>
+      <c r="CE66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -16260,6 +16334,7 @@
       <c r="CB67" t="inlineStr"/>
       <c r="CC67" t="inlineStr"/>
       <c r="CD67" t="inlineStr"/>
+      <c r="CE67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -16552,6 +16627,7 @@
       <c r="CB68" t="inlineStr"/>
       <c r="CC68" t="inlineStr"/>
       <c r="CD68" t="inlineStr"/>
+      <c r="CE68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -16840,6 +16916,7 @@
       <c r="CB69" t="inlineStr"/>
       <c r="CC69" t="inlineStr"/>
       <c r="CD69" t="inlineStr"/>
+      <c r="CE69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -17046,6 +17123,7 @@
       <c r="CB70" t="inlineStr"/>
       <c r="CC70" t="inlineStr"/>
       <c r="CD70" t="inlineStr"/>
+      <c r="CE70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -17266,6 +17344,7 @@
           <t>Disposición final</t>
         </is>
       </c>
+      <c r="CE71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -17414,6 +17493,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -17712,6 +17792,7 @@
       <c r="CB73" t="inlineStr"/>
       <c r="CC73" t="inlineStr"/>
       <c r="CD73" t="inlineStr"/>
+      <c r="CE73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -17922,6 +18003,7 @@
       <c r="CB74" t="inlineStr"/>
       <c r="CC74" t="inlineStr"/>
       <c r="CD74" t="inlineStr"/>
+      <c r="CE74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -18210,6 +18292,7 @@
       <c r="CB75" t="inlineStr"/>
       <c r="CC75" t="inlineStr"/>
       <c r="CD75" t="inlineStr"/>
+      <c r="CE75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -18480,6 +18563,7 @@
           <t>Cuentas por pagar</t>
         </is>
       </c>
+      <c r="CE76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -18686,6 +18770,7 @@
       <c r="CB77" t="inlineStr"/>
       <c r="CC77" t="inlineStr"/>
       <c r="CD77" t="inlineStr"/>
+      <c r="CE77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -18892,6 +18977,7 @@
       <c r="CB78" t="inlineStr"/>
       <c r="CC78" t="inlineStr"/>
       <c r="CD78" t="inlineStr"/>
+      <c r="CE78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -19098,6 +19184,7 @@
       <c r="CB79" t="inlineStr"/>
       <c r="CC79" t="inlineStr"/>
       <c r="CD79" t="inlineStr"/>
+      <c r="CE79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -19304,6 +19391,7 @@
       <c r="CB80" t="inlineStr"/>
       <c r="CC80" t="inlineStr"/>
       <c r="CD80" t="inlineStr"/>
+      <c r="CE80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -19452,6 +19540,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -19692,6 +19781,7 @@
       <c r="CB82" t="inlineStr"/>
       <c r="CC82" t="inlineStr"/>
       <c r="CD82" t="inlineStr"/>
+      <c r="CE82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -19898,6 +19988,7 @@
       <c r="CB83" t="inlineStr"/>
       <c r="CC83" t="inlineStr"/>
       <c r="CD83" t="inlineStr"/>
+      <c r="CE83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -20174,6 +20265,7 @@
           <t>Cuentas por pagar</t>
         </is>
       </c>
+      <c r="CE84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -20322,6 +20414,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -20528,6 +20621,7 @@
       <c r="CB86" t="inlineStr"/>
       <c r="CC86" t="inlineStr"/>
       <c r="CD86" t="inlineStr"/>
+      <c r="CE86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -20676,6 +20770,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -20824,6 +20919,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -21064,6 +21160,7 @@
       <c r="CB89" t="inlineStr"/>
       <c r="CC89" t="inlineStr"/>
       <c r="CD89" t="inlineStr"/>
+      <c r="CE89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -21270,6 +21367,7 @@
       <c r="CB90" t="inlineStr"/>
       <c r="CC90" t="inlineStr"/>
       <c r="CD90" t="inlineStr"/>
+      <c r="CE90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -21526,6 +21624,7 @@
       <c r="CB91" t="inlineStr"/>
       <c r="CC91" t="inlineStr"/>
       <c r="CD91" t="inlineStr"/>
+      <c r="CE91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -21740,6 +21839,7 @@
       <c r="CB92" t="inlineStr"/>
       <c r="CC92" t="inlineStr"/>
       <c r="CD92" t="inlineStr"/>
+      <c r="CE92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -21946,6 +22046,7 @@
       <c r="CB93" t="inlineStr"/>
       <c r="CC93" t="inlineStr"/>
       <c r="CD93" t="inlineStr"/>
+      <c r="CE93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -22166,6 +22267,7 @@
           <t>Disposición final</t>
         </is>
       </c>
+      <c r="CE94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -22406,6 +22508,7 @@
       <c r="CB95" t="inlineStr"/>
       <c r="CC95" t="inlineStr"/>
       <c r="CD95" t="inlineStr"/>
+      <c r="CE95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -22612,6 +22715,7 @@
       <c r="CB96" t="inlineStr"/>
       <c r="CC96" t="inlineStr"/>
       <c r="CD96" t="inlineStr"/>
+      <c r="CE96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -22866,6 +22970,7 @@
       <c r="CB97" t="inlineStr"/>
       <c r="CC97" t="inlineStr"/>
       <c r="CD97" t="inlineStr"/>
+      <c r="CE97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -23072,6 +23177,7 @@
       <c r="CB98" t="inlineStr"/>
       <c r="CC98" t="inlineStr"/>
       <c r="CD98" t="inlineStr"/>
+      <c r="CE98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -23312,6 +23418,7 @@
       <c r="CB99" t="inlineStr"/>
       <c r="CC99" t="inlineStr"/>
       <c r="CD99" t="inlineStr"/>
+      <c r="CE99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -23552,6 +23659,7 @@
       <c r="CB100" t="inlineStr"/>
       <c r="CC100" t="inlineStr"/>
       <c r="CD100" t="inlineStr"/>
+      <c r="CE100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -23792,6 +23900,7 @@
       <c r="CB101" t="inlineStr"/>
       <c r="CC101" t="inlineStr"/>
       <c r="CD101" t="inlineStr"/>
+      <c r="CE101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -23940,6 +24049,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -24232,6 +24342,7 @@
       <c r="CB103" t="inlineStr"/>
       <c r="CC103" t="inlineStr"/>
       <c r="CD103" t="inlineStr"/>
+      <c r="CE103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -24438,6 +24549,7 @@
       <c r="CB104" t="inlineStr"/>
       <c r="CC104" t="inlineStr"/>
       <c r="CD104" t="inlineStr"/>
+      <c r="CE104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -24678,6 +24790,7 @@
       <c r="CB105" t="inlineStr"/>
       <c r="CC105" t="inlineStr"/>
       <c r="CD105" t="inlineStr"/>
+      <c r="CE105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -24940,6 +25053,7 @@
       <c r="CB106" t="inlineStr"/>
       <c r="CC106" t="inlineStr"/>
       <c r="CD106" t="inlineStr"/>
+      <c r="CE106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -25200,6 +25314,7 @@
       <c r="CB107" t="inlineStr"/>
       <c r="CC107" t="inlineStr"/>
       <c r="CD107" t="inlineStr"/>
+      <c r="CE107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -25420,6 +25535,7 @@
           <t>Disposición final</t>
         </is>
       </c>
+      <c r="CE108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -25568,6 +25684,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -25774,6 +25891,7 @@
       <c r="CB110" t="inlineStr"/>
       <c r="CC110" t="inlineStr"/>
       <c r="CD110" t="inlineStr"/>
+      <c r="CE110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -25980,6 +26098,7 @@
       <c r="CB111" t="inlineStr"/>
       <c r="CC111" t="inlineStr"/>
       <c r="CD111" t="inlineStr"/>
+      <c r="CE111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -26240,6 +26359,7 @@
       <c r="CB112" t="inlineStr"/>
       <c r="CC112" t="inlineStr"/>
       <c r="CD112" t="inlineStr"/>
+      <c r="CE112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -26532,6 +26652,7 @@
       <c r="CB113" t="inlineStr"/>
       <c r="CC113" t="inlineStr"/>
       <c r="CD113" t="inlineStr"/>
+      <c r="CE113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -26820,6 +26941,7 @@
       <c r="CB114" t="inlineStr"/>
       <c r="CC114" t="inlineStr"/>
       <c r="CD114" t="inlineStr"/>
+      <c r="CE114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -27112,6 +27234,7 @@
       <c r="CB115" t="inlineStr"/>
       <c r="CC115" t="inlineStr"/>
       <c r="CD115" t="inlineStr"/>
+      <c r="CE115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -27318,6 +27441,7 @@
       <c r="CB116" t="inlineStr"/>
       <c r="CC116" t="inlineStr"/>
       <c r="CD116" t="inlineStr"/>
+      <c r="CE116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -27524,6 +27648,7 @@
       <c r="CB117" t="inlineStr"/>
       <c r="CC117" t="inlineStr"/>
       <c r="CD117" t="inlineStr"/>
+      <c r="CE117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -27730,6 +27855,7 @@
       <c r="CB118" t="inlineStr"/>
       <c r="CC118" t="inlineStr"/>
       <c r="CD118" t="inlineStr"/>
+      <c r="CE118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -27878,6 +28004,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -28026,6 +28153,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -28232,6 +28360,7 @@
       <c r="CB121" t="inlineStr"/>
       <c r="CC121" t="inlineStr"/>
       <c r="CD121" t="inlineStr"/>
+      <c r="CE121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -28438,6 +28567,7 @@
       <c r="CB122" t="inlineStr"/>
       <c r="CC122" t="inlineStr"/>
       <c r="CD122" t="inlineStr"/>
+      <c r="CE122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -28692,6 +28822,7 @@
       <c r="CB123" t="inlineStr"/>
       <c r="CC123" t="inlineStr"/>
       <c r="CD123" t="inlineStr"/>
+      <c r="CE123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -28898,6 +29029,7 @@
       <c r="CB124" t="inlineStr"/>
       <c r="CC124" t="inlineStr"/>
       <c r="CD124" t="inlineStr"/>
+      <c r="CE124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -29188,6 +29320,7 @@
       <c r="CB125" t="inlineStr"/>
       <c r="CC125" t="inlineStr"/>
       <c r="CD125" t="inlineStr"/>
+      <c r="CE125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -29336,6 +29469,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -29542,6 +29676,7 @@
       <c r="CB127" t="inlineStr"/>
       <c r="CC127" t="inlineStr"/>
       <c r="CD127" t="inlineStr"/>
+      <c r="CE127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -29748,6 +29883,7 @@
       <c r="CB128" t="inlineStr"/>
       <c r="CC128" t="inlineStr"/>
       <c r="CD128" t="inlineStr"/>
+      <c r="CE128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -29954,6 +30090,7 @@
       <c r="CB129" t="inlineStr"/>
       <c r="CC129" t="inlineStr"/>
       <c r="CD129" t="inlineStr"/>
+      <c r="CE129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -30210,6 +30347,7 @@
       <c r="CB130" t="inlineStr"/>
       <c r="CC130" t="inlineStr"/>
       <c r="CD130" t="inlineStr"/>
+      <c r="CE130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -30416,6 +30554,7 @@
       <c r="CB131" t="inlineStr"/>
       <c r="CC131" t="inlineStr"/>
       <c r="CD131" t="inlineStr"/>
+      <c r="CE131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -30708,6 +30847,7 @@
       <c r="CB132" t="inlineStr"/>
       <c r="CC132" t="inlineStr"/>
       <c r="CD132" t="inlineStr"/>
+      <c r="CE132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -30914,6 +31054,7 @@
       <c r="CB133" t="inlineStr"/>
       <c r="CC133" t="inlineStr"/>
       <c r="CD133" t="inlineStr"/>
+      <c r="CE133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -31120,6 +31261,7 @@
       <c r="CB134" t="inlineStr"/>
       <c r="CC134" t="inlineStr"/>
       <c r="CD134" t="inlineStr"/>
+      <c r="CE134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -31326,6 +31468,7 @@
       <c r="CB135" t="inlineStr"/>
       <c r="CC135" t="inlineStr"/>
       <c r="CD135" t="inlineStr"/>
+      <c r="CE135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -31546,6 +31689,7 @@
           <t>Disposición final</t>
         </is>
       </c>
+      <c r="CE136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -31694,6 +31838,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -31842,6 +31987,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -32048,6 +32194,7 @@
       <c r="CB139" t="inlineStr"/>
       <c r="CC139" t="inlineStr"/>
       <c r="CD139" t="inlineStr"/>
+      <c r="CE139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -32196,6 +32343,7 @@
           <t>Reporte de reclamo</t>
         </is>
       </c>
+      <c r="CE140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -32402,6 +32550,7 @@
       <c r="CB141" t="inlineStr"/>
       <c r="CC141" t="inlineStr"/>
       <c r="CD141" t="inlineStr"/>
+      <c r="CE141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -32692,6 +32841,7 @@
       <c r="CB142" t="inlineStr"/>
       <c r="CC142" t="inlineStr"/>
       <c r="CD142" t="inlineStr"/>
+      <c r="CE142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -32898,6 +33048,7 @@
       <c r="CB143" t="inlineStr"/>
       <c r="CC143" t="inlineStr"/>
       <c r="CD143" t="inlineStr"/>
+      <c r="CE143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -33154,6 +33305,7 @@
       <c r="CB144" t="inlineStr"/>
       <c r="CC144" t="inlineStr"/>
       <c r="CD144" t="inlineStr"/>
+      <c r="CE144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -33360,6 +33512,7 @@
       <c r="CB145" t="inlineStr"/>
       <c r="CC145" t="inlineStr"/>
       <c r="CD145" t="inlineStr"/>
+      <c r="CE145" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por Fernando (144 registros, 17/08/2026 17:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE145"/>
+  <dimension ref="A1:CH145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -834,6 +834,21 @@
       <c r="CE1" t="inlineStr">
         <is>
           <t>E3 FOLIO DEVOLUCION AJUSTE</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr">
+        <is>
+          <t>E3 FOLIO DEVOLUCION</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>E3 FOLIO AJUSTE</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>E3 NOTA CREDITO</t>
         </is>
       </c>
     </row>
@@ -1100,9 +1115,12 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr"/>
       <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="n">
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="n">
         <v>8382</v>
       </c>
+      <c r="CG2" t="inlineStr"/>
+      <c r="CH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -1367,9 +1385,12 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr"/>
       <c r="CD3" t="inlineStr"/>
-      <c r="CE3" t="n">
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="n">
         <v>8325</v>
       </c>
+      <c r="CG3" t="inlineStr"/>
+      <c r="CH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -1667,6 +1688,9 @@
       <c r="CC4" t="inlineStr"/>
       <c r="CD4" t="inlineStr"/>
       <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="inlineStr"/>
+      <c r="CH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1820,6 +1844,9 @@
         </is>
       </c>
       <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="inlineStr"/>
+      <c r="CH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1973,6 +2000,9 @@
         </is>
       </c>
       <c r="CE6" t="inlineStr"/>
+      <c r="CF6" t="inlineStr"/>
+      <c r="CG6" t="inlineStr"/>
+      <c r="CH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -2248,6 +2278,9 @@
       <c r="CC7" t="inlineStr"/>
       <c r="CD7" t="inlineStr"/>
       <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="inlineStr"/>
+      <c r="CH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -2540,9 +2573,12 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr"/>
       <c r="CD8" t="inlineStr"/>
-      <c r="CE8" t="n">
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="n">
         <v>7984</v>
       </c>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -2845,9 +2881,12 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr"/>
       <c r="CD9" t="inlineStr"/>
-      <c r="CE9" t="n">
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="n">
         <v>8361</v>
       </c>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -3001,6 +3040,9 @@
         </is>
       </c>
       <c r="CE10" t="inlineStr"/>
+      <c r="CF10" t="inlineStr"/>
+      <c r="CG10" t="inlineStr"/>
+      <c r="CH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -3250,6 +3292,9 @@
       <c r="CC11" t="inlineStr"/>
       <c r="CD11" t="inlineStr"/>
       <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -3403,6 +3448,9 @@
         </is>
       </c>
       <c r="CE12" t="inlineStr"/>
+      <c r="CF12" t="inlineStr"/>
+      <c r="CG12" t="inlineStr"/>
+      <c r="CH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -3667,9 +3715,12 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr"/>
       <c r="CD13" t="inlineStr"/>
-      <c r="CE13" t="n">
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="n">
         <v>8375</v>
       </c>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -3885,6 +3936,9 @@
       <c r="CC14" t="inlineStr"/>
       <c r="CD14" t="inlineStr"/>
       <c r="CE14" t="inlineStr"/>
+      <c r="CF14" t="inlineStr"/>
+      <c r="CG14" t="inlineStr"/>
+      <c r="CH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -4038,6 +4092,9 @@
         </is>
       </c>
       <c r="CE15" t="inlineStr"/>
+      <c r="CF15" t="inlineStr"/>
+      <c r="CG15" t="inlineStr"/>
+      <c r="CH15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -4191,6 +4248,9 @@
         </is>
       </c>
       <c r="CE16" t="inlineStr"/>
+      <c r="CF16" t="inlineStr"/>
+      <c r="CG16" t="inlineStr"/>
+      <c r="CH16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -4487,9 +4547,12 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr"/>
       <c r="CD17" t="inlineStr"/>
-      <c r="CE17" t="n">
+      <c r="CE17" t="inlineStr"/>
+      <c r="CF17" t="n">
         <v>34298</v>
       </c>
+      <c r="CG17" t="inlineStr"/>
+      <c r="CH17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -4755,6 +4818,9 @@
         </is>
       </c>
       <c r="CE18" t="inlineStr"/>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr"/>
+      <c r="CH18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -4908,6 +4974,9 @@
         </is>
       </c>
       <c r="CE19" t="inlineStr"/>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr"/>
+      <c r="CH19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -5061,6 +5130,9 @@
         </is>
       </c>
       <c r="CE20" t="inlineStr"/>
+      <c r="CF20" t="inlineStr"/>
+      <c r="CG20" t="inlineStr"/>
+      <c r="CH20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -5214,6 +5286,9 @@
         </is>
       </c>
       <c r="CE21" t="inlineStr"/>
+      <c r="CF21" t="inlineStr"/>
+      <c r="CG21" t="inlineStr"/>
+      <c r="CH21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -5425,6 +5500,9 @@
       <c r="CC22" t="inlineStr"/>
       <c r="CD22" t="inlineStr"/>
       <c r="CE22" t="inlineStr"/>
+      <c r="CF22" t="inlineStr"/>
+      <c r="CG22" t="inlineStr"/>
+      <c r="CH22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -5578,6 +5656,9 @@
         </is>
       </c>
       <c r="CE23" t="inlineStr"/>
+      <c r="CF23" t="inlineStr"/>
+      <c r="CG23" t="inlineStr"/>
+      <c r="CH23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -5842,9 +5923,12 @@
       <c r="CB24" t="inlineStr"/>
       <c r="CC24" t="inlineStr"/>
       <c r="CD24" t="inlineStr"/>
-      <c r="CE24" t="n">
+      <c r="CE24" t="inlineStr"/>
+      <c r="CF24" t="n">
         <v>8354</v>
       </c>
+      <c r="CG24" t="inlineStr"/>
+      <c r="CH24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -6137,9 +6221,12 @@
       <c r="CB25" t="inlineStr"/>
       <c r="CC25" t="inlineStr"/>
       <c r="CD25" t="inlineStr"/>
-      <c r="CE25" t="n">
+      <c r="CE25" t="inlineStr"/>
+      <c r="CF25" t="n">
         <v>8302</v>
       </c>
+      <c r="CG25" t="inlineStr"/>
+      <c r="CH25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -6393,6 +6480,9 @@
       <c r="CC26" t="inlineStr"/>
       <c r="CD26" t="inlineStr"/>
       <c r="CE26" t="inlineStr"/>
+      <c r="CF26" t="inlineStr"/>
+      <c r="CG26" t="inlineStr"/>
+      <c r="CH26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -6657,9 +6747,12 @@
       <c r="CB27" t="inlineStr"/>
       <c r="CC27" t="inlineStr"/>
       <c r="CD27" t="inlineStr"/>
-      <c r="CE27" t="n">
+      <c r="CE27" t="inlineStr"/>
+      <c r="CF27" t="n">
         <v>8341</v>
       </c>
+      <c r="CG27" t="inlineStr"/>
+      <c r="CH27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -6956,9 +7049,12 @@
       <c r="CB28" t="inlineStr"/>
       <c r="CC28" t="inlineStr"/>
       <c r="CD28" t="inlineStr"/>
-      <c r="CE28" t="n">
+      <c r="CE28" t="inlineStr"/>
+      <c r="CF28" t="n">
         <v>35811</v>
       </c>
+      <c r="CG28" t="inlineStr"/>
+      <c r="CH28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -7186,6 +7282,9 @@
       <c r="CC29" t="inlineStr"/>
       <c r="CD29" t="inlineStr"/>
       <c r="CE29" t="inlineStr"/>
+      <c r="CF29" t="inlineStr"/>
+      <c r="CG29" t="inlineStr"/>
+      <c r="CH29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -7339,6 +7438,9 @@
         </is>
       </c>
       <c r="CE30" t="inlineStr"/>
+      <c r="CF30" t="inlineStr"/>
+      <c r="CG30" t="inlineStr"/>
+      <c r="CH30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -7588,6 +7690,9 @@
       <c r="CC31" t="inlineStr"/>
       <c r="CD31" t="inlineStr"/>
       <c r="CE31" t="inlineStr"/>
+      <c r="CF31" t="inlineStr"/>
+      <c r="CG31" t="inlineStr"/>
+      <c r="CH31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -7860,9 +7965,12 @@
       <c r="CB32" t="inlineStr"/>
       <c r="CC32" t="inlineStr"/>
       <c r="CD32" t="inlineStr"/>
-      <c r="CE32" t="n">
+      <c r="CE32" t="inlineStr"/>
+      <c r="CF32" t="n">
         <v>8359</v>
       </c>
+      <c r="CG32" t="inlineStr"/>
+      <c r="CH32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -8129,9 +8237,12 @@
       <c r="CB33" t="inlineStr"/>
       <c r="CC33" t="inlineStr"/>
       <c r="CD33" t="inlineStr"/>
-      <c r="CE33" t="n">
+      <c r="CE33" t="inlineStr"/>
+      <c r="CF33" t="n">
         <v>8335</v>
       </c>
+      <c r="CG33" t="inlineStr"/>
+      <c r="CH33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -8347,6 +8458,9 @@
       <c r="CC34" t="inlineStr"/>
       <c r="CD34" t="inlineStr"/>
       <c r="CE34" t="inlineStr"/>
+      <c r="CF34" t="inlineStr"/>
+      <c r="CG34" t="inlineStr"/>
+      <c r="CH34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -8500,6 +8614,9 @@
         </is>
       </c>
       <c r="CE35" t="inlineStr"/>
+      <c r="CF35" t="inlineStr"/>
+      <c r="CG35" t="inlineStr"/>
+      <c r="CH35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -8792,9 +8909,12 @@
       <c r="CB36" t="inlineStr"/>
       <c r="CC36" t="inlineStr"/>
       <c r="CD36" t="inlineStr"/>
-      <c r="CE36" t="n">
+      <c r="CE36" t="inlineStr"/>
+      <c r="CF36" t="n">
         <v>8345</v>
       </c>
+      <c r="CG36" t="inlineStr"/>
+      <c r="CH36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -9091,9 +9211,12 @@
       <c r="CB37" t="inlineStr"/>
       <c r="CC37" t="inlineStr"/>
       <c r="CD37" t="inlineStr"/>
-      <c r="CE37" t="n">
+      <c r="CE37" t="inlineStr"/>
+      <c r="CF37" t="n">
         <v>8282</v>
       </c>
+      <c r="CG37" t="inlineStr"/>
+      <c r="CH37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -9247,6 +9370,9 @@
         </is>
       </c>
       <c r="CE38" t="inlineStr"/>
+      <c r="CF38" t="inlineStr"/>
+      <c r="CG38" t="inlineStr"/>
+      <c r="CH38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -9462,6 +9588,9 @@
       <c r="CC39" t="inlineStr"/>
       <c r="CD39" t="inlineStr"/>
       <c r="CE39" t="inlineStr"/>
+      <c r="CF39" t="inlineStr"/>
+      <c r="CG39" t="inlineStr"/>
+      <c r="CH39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -9689,6 +9818,9 @@
       <c r="CC40" t="inlineStr"/>
       <c r="CD40" t="inlineStr"/>
       <c r="CE40" t="inlineStr"/>
+      <c r="CF40" t="inlineStr"/>
+      <c r="CG40" t="inlineStr"/>
+      <c r="CH40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -9953,9 +10085,12 @@
       <c r="CB41" t="inlineStr"/>
       <c r="CC41" t="inlineStr"/>
       <c r="CD41" t="inlineStr"/>
-      <c r="CE41" t="n">
+      <c r="CE41" t="inlineStr"/>
+      <c r="CF41" t="n">
         <v>8367</v>
       </c>
+      <c r="CG41" t="inlineStr"/>
+      <c r="CH41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -10173,6 +10308,9 @@
       <c r="CC42" t="inlineStr"/>
       <c r="CD42" t="inlineStr"/>
       <c r="CE42" t="inlineStr"/>
+      <c r="CF42" t="inlineStr"/>
+      <c r="CG42" t="inlineStr"/>
+      <c r="CH42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -10354,6 +10492,9 @@
         </is>
       </c>
       <c r="CE43" t="inlineStr"/>
+      <c r="CF43" t="inlineStr"/>
+      <c r="CG43" t="inlineStr"/>
+      <c r="CH43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -10507,6 +10648,9 @@
         </is>
       </c>
       <c r="CE44" t="inlineStr"/>
+      <c r="CF44" t="inlineStr"/>
+      <c r="CG44" t="inlineStr"/>
+      <c r="CH44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -10660,6 +10804,9 @@
         </is>
       </c>
       <c r="CE45" t="inlineStr"/>
+      <c r="CF45" t="inlineStr"/>
+      <c r="CG45" t="inlineStr"/>
+      <c r="CH45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -10924,9 +11071,12 @@
       <c r="CB46" t="inlineStr"/>
       <c r="CC46" t="inlineStr"/>
       <c r="CD46" t="inlineStr"/>
-      <c r="CE46" t="n">
+      <c r="CE46" t="inlineStr"/>
+      <c r="CF46" t="n">
         <v>8352</v>
       </c>
+      <c r="CG46" t="inlineStr"/>
+      <c r="CH46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -11223,9 +11373,12 @@
       <c r="CB47" t="inlineStr"/>
       <c r="CC47" t="inlineStr"/>
       <c r="CD47" t="inlineStr"/>
-      <c r="CE47" t="n">
+      <c r="CE47" t="inlineStr"/>
+      <c r="CF47" t="n">
         <v>8349</v>
       </c>
+      <c r="CG47" t="inlineStr"/>
+      <c r="CH47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -11518,9 +11671,12 @@
       <c r="CB48" t="inlineStr"/>
       <c r="CC48" t="inlineStr"/>
       <c r="CD48" t="inlineStr"/>
-      <c r="CE48" t="n">
+      <c r="CE48" t="inlineStr"/>
+      <c r="CF48" t="n">
         <v>8274</v>
       </c>
+      <c r="CG48" t="inlineStr"/>
+      <c r="CH48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -11817,9 +11973,12 @@
       <c r="CB49" t="inlineStr"/>
       <c r="CC49" t="inlineStr"/>
       <c r="CD49" t="inlineStr"/>
-      <c r="CE49" t="n">
+      <c r="CE49" t="inlineStr"/>
+      <c r="CF49" t="n">
         <v>8334</v>
       </c>
+      <c r="CG49" t="inlineStr"/>
+      <c r="CH49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -12080,9 +12239,12 @@
       <c r="CB50" t="inlineStr"/>
       <c r="CC50" t="inlineStr"/>
       <c r="CD50" t="inlineStr"/>
-      <c r="CE50" t="n">
+      <c r="CE50" t="inlineStr"/>
+      <c r="CF50" t="n">
         <v>8382</v>
       </c>
+      <c r="CG50" t="inlineStr"/>
+      <c r="CH50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -12375,10 +12537,11 @@
       <c r="CB51" t="inlineStr"/>
       <c r="CC51" t="inlineStr"/>
       <c r="CD51" t="inlineStr"/>
-      <c r="CE51" t="inlineStr">
-        <is>
-          <t>NC 41151</t>
-        </is>
+      <c r="CE51" t="inlineStr"/>
+      <c r="CF51" t="inlineStr"/>
+      <c r="CG51" t="inlineStr"/>
+      <c r="CH51" t="n">
+        <v>41151</v>
       </c>
     </row>
     <row r="52">
@@ -12609,6 +12772,9 @@
       <c r="CC52" t="inlineStr"/>
       <c r="CD52" t="inlineStr"/>
       <c r="CE52" t="inlineStr"/>
+      <c r="CF52" t="inlineStr"/>
+      <c r="CG52" t="inlineStr"/>
+      <c r="CH52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -12907,9 +13073,12 @@
       <c r="CB53" t="inlineStr"/>
       <c r="CC53" t="inlineStr"/>
       <c r="CD53" t="inlineStr"/>
-      <c r="CE53" t="n">
+      <c r="CE53" t="inlineStr"/>
+      <c r="CF53" t="n">
         <v>8361</v>
       </c>
+      <c r="CG53" t="inlineStr"/>
+      <c r="CH53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -13170,9 +13339,12 @@
       <c r="CB54" t="inlineStr"/>
       <c r="CC54" t="inlineStr"/>
       <c r="CD54" t="inlineStr"/>
-      <c r="CE54" t="n">
+      <c r="CE54" t="inlineStr"/>
+      <c r="CF54" t="n">
         <v>8375</v>
       </c>
+      <c r="CG54" t="inlineStr"/>
+      <c r="CH54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -13444,6 +13616,9 @@
       <c r="CC55" t="inlineStr"/>
       <c r="CD55" t="inlineStr"/>
       <c r="CE55" t="inlineStr"/>
+      <c r="CF55" t="inlineStr"/>
+      <c r="CG55" t="inlineStr"/>
+      <c r="CH55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -13704,9 +13879,12 @@
       <c r="CB56" t="inlineStr"/>
       <c r="CC56" t="inlineStr"/>
       <c r="CD56" t="inlineStr"/>
-      <c r="CE56" t="n">
+      <c r="CE56" t="inlineStr"/>
+      <c r="CF56" t="n">
         <v>8325</v>
       </c>
+      <c r="CG56" t="inlineStr"/>
+      <c r="CH56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -13995,9 +14173,12 @@
       <c r="CB57" t="inlineStr"/>
       <c r="CC57" t="inlineStr"/>
       <c r="CD57" t="inlineStr"/>
-      <c r="CE57" t="n">
+      <c r="CE57" t="inlineStr"/>
+      <c r="CF57" t="n">
         <v>8350</v>
       </c>
+      <c r="CG57" t="inlineStr"/>
+      <c r="CH57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -14239,6 +14420,9 @@
       <c r="CC58" t="inlineStr"/>
       <c r="CD58" t="inlineStr"/>
       <c r="CE58" t="inlineStr"/>
+      <c r="CF58" t="inlineStr"/>
+      <c r="CG58" t="inlineStr"/>
+      <c r="CH58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -14480,6 +14664,9 @@
       <c r="CC59" t="inlineStr"/>
       <c r="CD59" t="inlineStr"/>
       <c r="CE59" t="inlineStr"/>
+      <c r="CF59" t="inlineStr"/>
+      <c r="CG59" t="inlineStr"/>
+      <c r="CH59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -14740,9 +14927,12 @@
       <c r="CB60" t="inlineStr"/>
       <c r="CC60" t="inlineStr"/>
       <c r="CD60" t="inlineStr"/>
-      <c r="CE60" t="n">
+      <c r="CE60" t="inlineStr"/>
+      <c r="CF60" t="n">
         <v>8341</v>
       </c>
+      <c r="CG60" t="inlineStr"/>
+      <c r="CH60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -14950,6 +15140,9 @@
       <c r="CC61" t="inlineStr"/>
       <c r="CD61" t="inlineStr"/>
       <c r="CE61" t="inlineStr"/>
+      <c r="CF61" t="inlineStr"/>
+      <c r="CG61" t="inlineStr"/>
+      <c r="CH61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -15238,9 +15431,12 @@
       <c r="CB62" t="inlineStr"/>
       <c r="CC62" t="inlineStr"/>
       <c r="CD62" t="inlineStr"/>
-      <c r="CE62" t="n">
+      <c r="CE62" t="inlineStr"/>
+      <c r="CF62" t="n">
         <v>8345</v>
       </c>
+      <c r="CG62" t="inlineStr"/>
+      <c r="CH62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -15466,6 +15662,9 @@
         </is>
       </c>
       <c r="CE63" t="inlineStr"/>
+      <c r="CF63" t="inlineStr"/>
+      <c r="CG63" t="inlineStr"/>
+      <c r="CH63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -15643,6 +15842,9 @@
         </is>
       </c>
       <c r="CE64" t="inlineStr"/>
+      <c r="CF64" t="inlineStr"/>
+      <c r="CG64" t="inlineStr"/>
+      <c r="CH64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -15862,6 +16064,9 @@
       <c r="CC65" t="inlineStr"/>
       <c r="CD65" t="inlineStr"/>
       <c r="CE65" t="inlineStr"/>
+      <c r="CF65" t="inlineStr"/>
+      <c r="CG65" t="inlineStr"/>
+      <c r="CH65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -16122,9 +16327,12 @@
       <c r="CB66" t="inlineStr"/>
       <c r="CC66" t="inlineStr"/>
       <c r="CD66" t="inlineStr"/>
-      <c r="CE66" t="n">
+      <c r="CE66" t="inlineStr"/>
+      <c r="CF66" t="n">
         <v>8367</v>
       </c>
+      <c r="CG66" t="inlineStr"/>
+      <c r="CH66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -16385,9 +16593,12 @@
       <c r="CB67" t="inlineStr"/>
       <c r="CC67" t="inlineStr"/>
       <c r="CD67" t="inlineStr"/>
-      <c r="CE67" t="n">
+      <c r="CE67" t="inlineStr"/>
+      <c r="CF67" t="n">
         <v>8352</v>
       </c>
+      <c r="CG67" t="inlineStr"/>
+      <c r="CH67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -16680,9 +16891,12 @@
       <c r="CB68" t="inlineStr"/>
       <c r="CC68" t="inlineStr"/>
       <c r="CD68" t="inlineStr"/>
-      <c r="CE68" t="n">
+      <c r="CE68" t="inlineStr"/>
+      <c r="CF68" t="n">
         <v>8349</v>
       </c>
+      <c r="CG68" t="inlineStr"/>
+      <c r="CH68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -16971,11 +17185,14 @@
       <c r="CB69" t="inlineStr"/>
       <c r="CC69" t="inlineStr"/>
       <c r="CD69" t="inlineStr"/>
-      <c r="CE69" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 8330-8274</t>
-        </is>
-      </c>
+      <c r="CE69" t="inlineStr"/>
+      <c r="CF69" t="n">
+        <v>8330</v>
+      </c>
+      <c r="CG69" t="n">
+        <v>8274</v>
+      </c>
+      <c r="CH69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -17183,6 +17400,9 @@
       <c r="CC70" t="inlineStr"/>
       <c r="CD70" t="inlineStr"/>
       <c r="CE70" t="inlineStr"/>
+      <c r="CF70" t="inlineStr"/>
+      <c r="CG70" t="inlineStr"/>
+      <c r="CH70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -17404,6 +17624,9 @@
         </is>
       </c>
       <c r="CE71" t="inlineStr"/>
+      <c r="CF71" t="inlineStr"/>
+      <c r="CG71" t="inlineStr"/>
+      <c r="CH71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -17553,6 +17776,9 @@
         </is>
       </c>
       <c r="CE72" t="inlineStr"/>
+      <c r="CF72" t="inlineStr"/>
+      <c r="CG72" t="inlineStr"/>
+      <c r="CH72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -17851,9 +18077,12 @@
       <c r="CB73" t="inlineStr"/>
       <c r="CC73" t="inlineStr"/>
       <c r="CD73" t="inlineStr"/>
-      <c r="CE73" t="n">
+      <c r="CE73" t="inlineStr"/>
+      <c r="CF73" t="n">
         <v>8347</v>
       </c>
+      <c r="CG73" t="inlineStr"/>
+      <c r="CH73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -18065,6 +18294,9 @@
       <c r="CC74" t="inlineStr"/>
       <c r="CD74" t="inlineStr"/>
       <c r="CE74" t="inlineStr"/>
+      <c r="CF74" t="inlineStr"/>
+      <c r="CG74" t="inlineStr"/>
+      <c r="CH74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -18354,6 +18586,9 @@
       <c r="CC75" t="inlineStr"/>
       <c r="CD75" t="inlineStr"/>
       <c r="CE75" t="inlineStr"/>
+      <c r="CF75" t="inlineStr"/>
+      <c r="CG75" t="inlineStr"/>
+      <c r="CH75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -18624,10 +18859,11 @@
           <t>Cuentas por pagar</t>
         </is>
       </c>
-      <c r="CE76" t="inlineStr">
-        <is>
-          <t>NC 36291</t>
-        </is>
+      <c r="CE76" t="inlineStr"/>
+      <c r="CF76" t="inlineStr"/>
+      <c r="CG76" t="inlineStr"/>
+      <c r="CH76" t="n">
+        <v>36291</v>
       </c>
     </row>
     <row r="77">
@@ -18836,6 +19072,9 @@
       <c r="CC77" t="inlineStr"/>
       <c r="CD77" t="inlineStr"/>
       <c r="CE77" t="inlineStr"/>
+      <c r="CF77" t="inlineStr"/>
+      <c r="CG77" t="inlineStr"/>
+      <c r="CH77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -19043,6 +19282,9 @@
       <c r="CC78" t="inlineStr"/>
       <c r="CD78" t="inlineStr"/>
       <c r="CE78" t="inlineStr"/>
+      <c r="CF78" t="inlineStr"/>
+      <c r="CG78" t="inlineStr"/>
+      <c r="CH78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -19250,6 +19492,9 @@
       <c r="CC79" t="inlineStr"/>
       <c r="CD79" t="inlineStr"/>
       <c r="CE79" t="inlineStr"/>
+      <c r="CF79" t="inlineStr"/>
+      <c r="CG79" t="inlineStr"/>
+      <c r="CH79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -19457,6 +19702,9 @@
       <c r="CC80" t="inlineStr"/>
       <c r="CD80" t="inlineStr"/>
       <c r="CE80" t="inlineStr"/>
+      <c r="CF80" t="inlineStr"/>
+      <c r="CG80" t="inlineStr"/>
+      <c r="CH80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -19606,6 +19854,9 @@
         </is>
       </c>
       <c r="CE81" t="inlineStr"/>
+      <c r="CF81" t="inlineStr"/>
+      <c r="CG81" t="inlineStr"/>
+      <c r="CH81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -19847,6 +20098,9 @@
       <c r="CC82" t="inlineStr"/>
       <c r="CD82" t="inlineStr"/>
       <c r="CE82" t="inlineStr"/>
+      <c r="CF82" t="inlineStr"/>
+      <c r="CG82" t="inlineStr"/>
+      <c r="CH82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -20054,6 +20308,9 @@
       <c r="CC83" t="inlineStr"/>
       <c r="CD83" t="inlineStr"/>
       <c r="CE83" t="inlineStr"/>
+      <c r="CF83" t="inlineStr"/>
+      <c r="CG83" t="inlineStr"/>
+      <c r="CH83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -20330,9 +20587,12 @@
           <t>Cuentas por pagar</t>
         </is>
       </c>
-      <c r="CE84" t="n">
+      <c r="CE84" t="inlineStr"/>
+      <c r="CF84" t="n">
         <v>8359</v>
       </c>
+      <c r="CG84" t="inlineStr"/>
+      <c r="CH84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -20482,6 +20742,9 @@
         </is>
       </c>
       <c r="CE85" t="inlineStr"/>
+      <c r="CF85" t="inlineStr"/>
+      <c r="CG85" t="inlineStr"/>
+      <c r="CH85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -20689,6 +20952,9 @@
       <c r="CC86" t="inlineStr"/>
       <c r="CD86" t="inlineStr"/>
       <c r="CE86" t="inlineStr"/>
+      <c r="CF86" t="inlineStr"/>
+      <c r="CG86" t="inlineStr"/>
+      <c r="CH86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -20838,6 +21104,9 @@
         </is>
       </c>
       <c r="CE87" t="inlineStr"/>
+      <c r="CF87" t="inlineStr"/>
+      <c r="CG87" t="inlineStr"/>
+      <c r="CH87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -20987,6 +21256,9 @@
         </is>
       </c>
       <c r="CE88" t="inlineStr"/>
+      <c r="CF88" t="inlineStr"/>
+      <c r="CG88" t="inlineStr"/>
+      <c r="CH88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -21228,6 +21500,9 @@
       <c r="CC89" t="inlineStr"/>
       <c r="CD89" t="inlineStr"/>
       <c r="CE89" t="inlineStr"/>
+      <c r="CF89" t="inlineStr"/>
+      <c r="CG89" t="inlineStr"/>
+      <c r="CH89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -21435,6 +21710,9 @@
       <c r="CC90" t="inlineStr"/>
       <c r="CD90" t="inlineStr"/>
       <c r="CE90" t="inlineStr"/>
+      <c r="CF90" t="inlineStr"/>
+      <c r="CG90" t="inlineStr"/>
+      <c r="CH90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -21691,9 +21969,12 @@
       <c r="CB91" t="inlineStr"/>
       <c r="CC91" t="inlineStr"/>
       <c r="CD91" t="inlineStr"/>
-      <c r="CE91" t="n">
+      <c r="CE91" t="inlineStr"/>
+      <c r="CF91" t="n">
         <v>8382</v>
       </c>
+      <c r="CG91" t="inlineStr"/>
+      <c r="CH91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -21909,6 +22190,9 @@
       <c r="CC92" t="inlineStr"/>
       <c r="CD92" t="inlineStr"/>
       <c r="CE92" t="inlineStr"/>
+      <c r="CF92" t="inlineStr"/>
+      <c r="CG92" t="inlineStr"/>
+      <c r="CH92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -22116,6 +22400,9 @@
       <c r="CC93" t="inlineStr"/>
       <c r="CD93" t="inlineStr"/>
       <c r="CE93" t="inlineStr"/>
+      <c r="CF93" t="inlineStr"/>
+      <c r="CG93" t="inlineStr"/>
+      <c r="CH93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -22337,6 +22624,9 @@
         </is>
       </c>
       <c r="CE94" t="inlineStr"/>
+      <c r="CF94" t="inlineStr"/>
+      <c r="CG94" t="inlineStr"/>
+      <c r="CH94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -22578,6 +22868,9 @@
       <c r="CC95" t="inlineStr"/>
       <c r="CD95" t="inlineStr"/>
       <c r="CE95" t="inlineStr"/>
+      <c r="CF95" t="inlineStr"/>
+      <c r="CG95" t="inlineStr"/>
+      <c r="CH95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -22785,6 +23078,9 @@
       <c r="CC96" t="inlineStr"/>
       <c r="CD96" t="inlineStr"/>
       <c r="CE96" t="inlineStr"/>
+      <c r="CF96" t="inlineStr"/>
+      <c r="CG96" t="inlineStr"/>
+      <c r="CH96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -23039,9 +23335,12 @@
       <c r="CB97" t="inlineStr"/>
       <c r="CC97" t="inlineStr"/>
       <c r="CD97" t="inlineStr"/>
-      <c r="CE97" t="n">
+      <c r="CE97" t="inlineStr"/>
+      <c r="CF97" t="n">
         <v>8375</v>
       </c>
+      <c r="CG97" t="inlineStr"/>
+      <c r="CH97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -23249,6 +23548,9 @@
       <c r="CC98" t="inlineStr"/>
       <c r="CD98" t="inlineStr"/>
       <c r="CE98" t="inlineStr"/>
+      <c r="CF98" t="inlineStr"/>
+      <c r="CG98" t="inlineStr"/>
+      <c r="CH98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -23490,6 +23792,9 @@
       <c r="CC99" t="inlineStr"/>
       <c r="CD99" t="inlineStr"/>
       <c r="CE99" t="inlineStr"/>
+      <c r="CF99" t="inlineStr"/>
+      <c r="CG99" t="inlineStr"/>
+      <c r="CH99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -23731,6 +24036,9 @@
       <c r="CC100" t="inlineStr"/>
       <c r="CD100" t="inlineStr"/>
       <c r="CE100" t="inlineStr"/>
+      <c r="CF100" t="inlineStr"/>
+      <c r="CG100" t="inlineStr"/>
+      <c r="CH100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -23972,6 +24280,9 @@
       <c r="CC101" t="inlineStr"/>
       <c r="CD101" t="inlineStr"/>
       <c r="CE101" t="inlineStr"/>
+      <c r="CF101" t="inlineStr"/>
+      <c r="CG101" t="inlineStr"/>
+      <c r="CH101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -24121,6 +24432,9 @@
         </is>
       </c>
       <c r="CE102" t="inlineStr"/>
+      <c r="CF102" t="inlineStr"/>
+      <c r="CG102" t="inlineStr"/>
+      <c r="CH102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -24413,9 +24727,12 @@
       <c r="CB103" t="inlineStr"/>
       <c r="CC103" t="inlineStr"/>
       <c r="CD103" t="inlineStr"/>
-      <c r="CE103" t="n">
+      <c r="CE103" t="inlineStr"/>
+      <c r="CF103" t="n">
         <v>8383</v>
       </c>
+      <c r="CG103" t="inlineStr"/>
+      <c r="CH103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -24623,6 +24940,9 @@
       <c r="CC104" t="inlineStr"/>
       <c r="CD104" t="inlineStr"/>
       <c r="CE104" t="inlineStr"/>
+      <c r="CF104" t="inlineStr"/>
+      <c r="CG104" t="inlineStr"/>
+      <c r="CH104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -24864,6 +25184,9 @@
       <c r="CC105" t="inlineStr"/>
       <c r="CD105" t="inlineStr"/>
       <c r="CE105" t="inlineStr"/>
+      <c r="CF105" t="inlineStr"/>
+      <c r="CG105" t="inlineStr"/>
+      <c r="CH105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -25126,9 +25449,12 @@
       <c r="CB106" t="inlineStr"/>
       <c r="CC106" t="inlineStr"/>
       <c r="CD106" t="inlineStr"/>
-      <c r="CE106" t="n">
+      <c r="CE106" t="inlineStr"/>
+      <c r="CF106" t="n">
         <v>8359</v>
       </c>
+      <c r="CG106" t="inlineStr"/>
+      <c r="CH106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -25389,9 +25715,12 @@
       <c r="CB107" t="inlineStr"/>
       <c r="CC107" t="inlineStr"/>
       <c r="CD107" t="inlineStr"/>
-      <c r="CE107" t="n">
+      <c r="CE107" t="inlineStr"/>
+      <c r="CF107" t="n">
         <v>8345</v>
       </c>
+      <c r="CG107" t="inlineStr"/>
+      <c r="CH107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -25613,6 +25942,9 @@
         </is>
       </c>
       <c r="CE108" t="inlineStr"/>
+      <c r="CF108" t="inlineStr"/>
+      <c r="CG108" t="inlineStr"/>
+      <c r="CH108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -25762,6 +26094,9 @@
         </is>
       </c>
       <c r="CE109" t="inlineStr"/>
+      <c r="CF109" t="inlineStr"/>
+      <c r="CG109" t="inlineStr"/>
+      <c r="CH109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -25969,6 +26304,9 @@
       <c r="CC110" t="inlineStr"/>
       <c r="CD110" t="inlineStr"/>
       <c r="CE110" t="inlineStr"/>
+      <c r="CF110" t="inlineStr"/>
+      <c r="CG110" t="inlineStr"/>
+      <c r="CH110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -26176,6 +26514,9 @@
       <c r="CC111" t="inlineStr"/>
       <c r="CD111" t="inlineStr"/>
       <c r="CE111" t="inlineStr"/>
+      <c r="CF111" t="inlineStr"/>
+      <c r="CG111" t="inlineStr"/>
+      <c r="CH111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -26436,9 +26777,12 @@
       <c r="CB112" t="inlineStr"/>
       <c r="CC112" t="inlineStr"/>
       <c r="CD112" t="inlineStr"/>
-      <c r="CE112" t="n">
+      <c r="CE112" t="inlineStr"/>
+      <c r="CF112" t="n">
         <v>8352</v>
       </c>
+      <c r="CG112" t="inlineStr"/>
+      <c r="CH112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -26731,9 +27075,12 @@
       <c r="CB113" t="inlineStr"/>
       <c r="CC113" t="inlineStr"/>
       <c r="CD113" t="inlineStr"/>
-      <c r="CE113" t="n">
+      <c r="CE113" t="inlineStr"/>
+      <c r="CF113" t="n">
         <v>8349</v>
       </c>
+      <c r="CG113" t="inlineStr"/>
+      <c r="CH113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -27022,9 +27369,12 @@
       <c r="CB114" t="inlineStr"/>
       <c r="CC114" t="inlineStr"/>
       <c r="CD114" t="inlineStr"/>
-      <c r="CE114" t="n">
+      <c r="CE114" t="inlineStr"/>
+      <c r="CF114" t="n">
         <v>8330</v>
       </c>
+      <c r="CG114" t="inlineStr"/>
+      <c r="CH114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -27317,9 +27667,12 @@
       <c r="CB115" t="inlineStr"/>
       <c r="CC115" t="inlineStr"/>
       <c r="CD115" t="inlineStr"/>
-      <c r="CE115" t="n">
+      <c r="CE115" t="inlineStr"/>
+      <c r="CF115" t="n">
         <v>8334</v>
       </c>
+      <c r="CG115" t="inlineStr"/>
+      <c r="CH115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -27527,6 +27880,9 @@
       <c r="CC116" t="inlineStr"/>
       <c r="CD116" t="inlineStr"/>
       <c r="CE116" t="inlineStr"/>
+      <c r="CF116" t="inlineStr"/>
+      <c r="CG116" t="inlineStr"/>
+      <c r="CH116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -27734,6 +28090,9 @@
       <c r="CC117" t="inlineStr"/>
       <c r="CD117" t="inlineStr"/>
       <c r="CE117" t="inlineStr"/>
+      <c r="CF117" t="inlineStr"/>
+      <c r="CG117" t="inlineStr"/>
+      <c r="CH117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -27941,6 +28300,9 @@
       <c r="CC118" t="inlineStr"/>
       <c r="CD118" t="inlineStr"/>
       <c r="CE118" t="inlineStr"/>
+      <c r="CF118" t="inlineStr"/>
+      <c r="CG118" t="inlineStr"/>
+      <c r="CH118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -28090,6 +28452,9 @@
         </is>
       </c>
       <c r="CE119" t="inlineStr"/>
+      <c r="CF119" t="inlineStr"/>
+      <c r="CG119" t="inlineStr"/>
+      <c r="CH119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -28239,6 +28604,9 @@
         </is>
       </c>
       <c r="CE120" t="inlineStr"/>
+      <c r="CF120" t="inlineStr"/>
+      <c r="CG120" t="inlineStr"/>
+      <c r="CH120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -28446,6 +28814,9 @@
       <c r="CC121" t="inlineStr"/>
       <c r="CD121" t="inlineStr"/>
       <c r="CE121" t="inlineStr"/>
+      <c r="CF121" t="inlineStr"/>
+      <c r="CG121" t="inlineStr"/>
+      <c r="CH121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -28653,6 +29024,9 @@
       <c r="CC122" t="inlineStr"/>
       <c r="CD122" t="inlineStr"/>
       <c r="CE122" t="inlineStr"/>
+      <c r="CF122" t="inlineStr"/>
+      <c r="CG122" t="inlineStr"/>
+      <c r="CH122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -28907,9 +29281,12 @@
       <c r="CB123" t="inlineStr"/>
       <c r="CC123" t="inlineStr"/>
       <c r="CD123" t="inlineStr"/>
-      <c r="CE123" t="n">
+      <c r="CE123" t="inlineStr"/>
+      <c r="CF123" t="n">
         <v>8384</v>
       </c>
+      <c r="CG123" t="inlineStr"/>
+      <c r="CH123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -29117,6 +29494,9 @@
       <c r="CC124" t="inlineStr"/>
       <c r="CD124" t="inlineStr"/>
       <c r="CE124" t="inlineStr"/>
+      <c r="CF124" t="inlineStr"/>
+      <c r="CG124" t="inlineStr"/>
+      <c r="CH124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -29407,9 +29787,12 @@
       <c r="CB125" t="inlineStr"/>
       <c r="CC125" t="inlineStr"/>
       <c r="CD125" t="inlineStr"/>
-      <c r="CE125" t="n">
+      <c r="CE125" t="inlineStr"/>
+      <c r="CF125" t="n">
         <v>8378</v>
       </c>
+      <c r="CG125" t="inlineStr"/>
+      <c r="CH125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -29559,6 +29942,9 @@
         </is>
       </c>
       <c r="CE126" t="inlineStr"/>
+      <c r="CF126" t="inlineStr"/>
+      <c r="CG126" t="inlineStr"/>
+      <c r="CH126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -29766,6 +30152,9 @@
       <c r="CC127" t="inlineStr"/>
       <c r="CD127" t="inlineStr"/>
       <c r="CE127" t="inlineStr"/>
+      <c r="CF127" t="inlineStr"/>
+      <c r="CG127" t="inlineStr"/>
+      <c r="CH127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -29973,6 +30362,9 @@
       <c r="CC128" t="inlineStr"/>
       <c r="CD128" t="inlineStr"/>
       <c r="CE128" t="inlineStr"/>
+      <c r="CF128" t="inlineStr"/>
+      <c r="CG128" t="inlineStr"/>
+      <c r="CH128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -30180,6 +30572,9 @@
       <c r="CC129" t="inlineStr"/>
       <c r="CD129" t="inlineStr"/>
       <c r="CE129" t="inlineStr"/>
+      <c r="CF129" t="inlineStr"/>
+      <c r="CG129" t="inlineStr"/>
+      <c r="CH129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -30436,9 +30831,12 @@
       <c r="CB130" t="inlineStr"/>
       <c r="CC130" t="inlineStr"/>
       <c r="CD130" t="inlineStr"/>
-      <c r="CE130" t="n">
+      <c r="CE130" t="inlineStr"/>
+      <c r="CF130" t="n">
         <v>8374</v>
       </c>
+      <c r="CG130" t="inlineStr"/>
+      <c r="CH130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -30646,6 +31044,9 @@
       <c r="CC131" t="inlineStr"/>
       <c r="CD131" t="inlineStr"/>
       <c r="CE131" t="inlineStr"/>
+      <c r="CF131" t="inlineStr"/>
+      <c r="CG131" t="inlineStr"/>
+      <c r="CH131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -30938,9 +31339,12 @@
       <c r="CB132" t="inlineStr"/>
       <c r="CC132" t="inlineStr"/>
       <c r="CD132" t="inlineStr"/>
-      <c r="CE132" t="n">
+      <c r="CE132" t="inlineStr"/>
+      <c r="CF132" t="n">
         <v>8383</v>
       </c>
+      <c r="CG132" t="inlineStr"/>
+      <c r="CH132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -31148,6 +31552,9 @@
       <c r="CC133" t="inlineStr"/>
       <c r="CD133" t="inlineStr"/>
       <c r="CE133" t="inlineStr"/>
+      <c r="CF133" t="inlineStr"/>
+      <c r="CG133" t="inlineStr"/>
+      <c r="CH133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -31355,6 +31762,9 @@
       <c r="CC134" t="inlineStr"/>
       <c r="CD134" t="inlineStr"/>
       <c r="CE134" t="inlineStr"/>
+      <c r="CF134" t="inlineStr"/>
+      <c r="CG134" t="inlineStr"/>
+      <c r="CH134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -31562,6 +31972,9 @@
       <c r="CC135" t="inlineStr"/>
       <c r="CD135" t="inlineStr"/>
       <c r="CE135" t="inlineStr"/>
+      <c r="CF135" t="inlineStr"/>
+      <c r="CG135" t="inlineStr"/>
+      <c r="CH135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -31783,6 +32196,9 @@
         </is>
       </c>
       <c r="CE136" t="inlineStr"/>
+      <c r="CF136" t="inlineStr"/>
+      <c r="CG136" t="inlineStr"/>
+      <c r="CH136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -31932,6 +32348,9 @@
         </is>
       </c>
       <c r="CE137" t="inlineStr"/>
+      <c r="CF137" t="inlineStr"/>
+      <c r="CG137" t="inlineStr"/>
+      <c r="CH137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -32081,6 +32500,9 @@
         </is>
       </c>
       <c r="CE138" t="inlineStr"/>
+      <c r="CF138" t="inlineStr"/>
+      <c r="CG138" t="inlineStr"/>
+      <c r="CH138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -32288,6 +32710,9 @@
       <c r="CC139" t="inlineStr"/>
       <c r="CD139" t="inlineStr"/>
       <c r="CE139" t="inlineStr"/>
+      <c r="CF139" t="inlineStr"/>
+      <c r="CG139" t="inlineStr"/>
+      <c r="CH139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -32437,6 +32862,9 @@
         </is>
       </c>
       <c r="CE140" t="inlineStr"/>
+      <c r="CF140" t="inlineStr"/>
+      <c r="CG140" t="inlineStr"/>
+      <c r="CH140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -32644,6 +33072,9 @@
       <c r="CC141" t="inlineStr"/>
       <c r="CD141" t="inlineStr"/>
       <c r="CE141" t="inlineStr"/>
+      <c r="CF141" t="inlineStr"/>
+      <c r="CG141" t="inlineStr"/>
+      <c r="CH141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -32934,9 +33365,12 @@
       <c r="CB142" t="inlineStr"/>
       <c r="CC142" t="inlineStr"/>
       <c r="CD142" t="inlineStr"/>
-      <c r="CE142" t="n">
+      <c r="CE142" t="inlineStr"/>
+      <c r="CF142" t="n">
         <v>8378</v>
       </c>
+      <c r="CG142" t="inlineStr"/>
+      <c r="CH142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -33144,6 +33578,9 @@
       <c r="CC143" t="inlineStr"/>
       <c r="CD143" t="inlineStr"/>
       <c r="CE143" t="inlineStr"/>
+      <c r="CF143" t="inlineStr"/>
+      <c r="CG143" t="inlineStr"/>
+      <c r="CH143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -33400,9 +33837,12 @@
       <c r="CB144" t="inlineStr"/>
       <c r="CC144" t="inlineStr"/>
       <c r="CD144" t="inlineStr"/>
-      <c r="CE144" t="n">
+      <c r="CE144" t="inlineStr"/>
+      <c r="CF144" t="n">
         <v>8359</v>
       </c>
+      <c r="CG144" t="inlineStr"/>
+      <c r="CH144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -33610,6 +34050,9 @@
       <c r="CC145" t="inlineStr"/>
       <c r="CD145" t="inlineStr"/>
       <c r="CE145" t="inlineStr"/>
+      <c r="CF145" t="inlineStr"/>
+      <c r="CG145" t="inlineStr"/>
+      <c r="CH145" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Carga masiva de base de datos por fernando treviño (193 registros, 22/08/2026 12:25)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34087,10 +34087,18 @@
       <c r="H146" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
-      <c r="L146" t="inlineStr"/>
+      <c r="I146" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J146" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K146" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L146" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr"/>
@@ -34199,10 +34207,18 @@
       <c r="H147" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
+      <c r="I147" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J147" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K147" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L147" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M147" t="inlineStr"/>
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr"/>
@@ -34311,10 +34327,18 @@
       <c r="H148" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
+      <c r="I148" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J148" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K148" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L148" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="inlineStr"/>
       <c r="O148" t="inlineStr"/>
@@ -34423,10 +34447,18 @@
       <c r="H149" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
+      <c r="I149" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J149" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K149" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L149" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
       <c r="O149" t="inlineStr"/>
@@ -34535,10 +34567,18 @@
       <c r="H150" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr"/>
+      <c r="I150" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J150" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K150" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L150" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr"/>
@@ -34647,10 +34687,18 @@
       <c r="H151" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr"/>
+      <c r="I151" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J151" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K151" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L151" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M151" t="inlineStr"/>
       <c r="N151" t="inlineStr"/>
       <c r="O151" t="inlineStr"/>
@@ -34759,10 +34807,18 @@
       <c r="H152" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
+      <c r="I152" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J152" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K152" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L152" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr"/>
       <c r="O152" t="inlineStr"/>
@@ -34871,10 +34927,18 @@
       <c r="H153" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr"/>
+      <c r="I153" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J153" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K153" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L153" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M153" t="inlineStr"/>
       <c r="N153" t="inlineStr"/>
       <c r="O153" t="inlineStr"/>
@@ -34980,11 +35044,7 @@
           <t>MIRIAM</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>no se envia</t>
-        </is>
-      </c>
+      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr"/>
@@ -35097,10 +35157,18 @@
       <c r="H155" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr"/>
+      <c r="I155" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J155" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K155" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L155" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M155" t="inlineStr"/>
       <c r="N155" t="inlineStr"/>
       <c r="O155" t="inlineStr"/>
@@ -35209,10 +35277,18 @@
       <c r="H156" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
+      <c r="I156" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J156" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K156" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L156" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M156" t="inlineStr"/>
       <c r="N156" t="inlineStr"/>
       <c r="O156" t="inlineStr"/>
@@ -35321,10 +35397,18 @@
       <c r="H157" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr"/>
+      <c r="I157" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J157" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K157" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L157" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M157" t="inlineStr"/>
       <c r="N157" t="inlineStr"/>
       <c r="O157" t="inlineStr"/>
@@ -35433,10 +35517,18 @@
       <c r="H158" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I158" t="inlineStr"/>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr"/>
+      <c r="I158" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J158" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K158" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L158" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M158" t="inlineStr"/>
       <c r="N158" t="inlineStr"/>
       <c r="O158" t="inlineStr"/>
@@ -35545,10 +35637,18 @@
       <c r="H159" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I159" t="inlineStr"/>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr"/>
+      <c r="I159" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J159" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K159" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L159" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M159" t="inlineStr"/>
       <c r="N159" t="inlineStr"/>
       <c r="O159" t="inlineStr"/>
@@ -35657,10 +35757,18 @@
       <c r="H160" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
+      <c r="I160" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J160" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K160" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L160" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M160" t="inlineStr"/>
       <c r="N160" t="inlineStr"/>
       <c r="O160" t="inlineStr"/>
@@ -35769,10 +35877,18 @@
       <c r="H161" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I161" t="inlineStr"/>
-      <c r="J161" t="inlineStr"/>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
+      <c r="I161" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J161" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K161" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L161" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M161" t="inlineStr"/>
       <c r="N161" t="inlineStr"/>
       <c r="O161" t="inlineStr"/>
@@ -35881,10 +35997,18 @@
       <c r="H162" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I162" t="inlineStr"/>
-      <c r="J162" t="inlineStr"/>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
+      <c r="I162" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J162" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K162" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L162" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M162" t="inlineStr"/>
       <c r="N162" t="inlineStr"/>
       <c r="O162" t="inlineStr"/>
@@ -35993,10 +36117,18 @@
       <c r="H163" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I163" t="inlineStr"/>
-      <c r="J163" t="inlineStr"/>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+      <c r="I163" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J163" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K163" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L163" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="inlineStr"/>
       <c r="O163" t="inlineStr"/>
@@ -36105,10 +36237,18 @@
       <c r="H164" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
+      <c r="I164" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J164" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K164" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L164" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="inlineStr"/>
       <c r="O164" t="inlineStr"/>
@@ -36217,10 +36357,18 @@
       <c r="H165" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
+      <c r="I165" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J165" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K165" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L165" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M165" t="inlineStr"/>
       <c r="N165" t="inlineStr"/>
       <c r="O165" t="inlineStr"/>
@@ -36329,10 +36477,18 @@
       <c r="H166" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
+      <c r="I166" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J166" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K166" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L166" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M166" t="inlineStr"/>
       <c r="N166" t="inlineStr"/>
       <c r="O166" t="inlineStr"/>
@@ -36441,10 +36597,18 @@
       <c r="H167" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I167" t="inlineStr"/>
-      <c r="J167" t="inlineStr"/>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+      <c r="I167" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J167" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K167" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L167" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="inlineStr"/>
@@ -36553,10 +36717,18 @@
       <c r="H168" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
+      <c r="I168" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J168" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K168" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L168" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M168" t="inlineStr"/>
       <c r="N168" t="inlineStr"/>
       <c r="O168" t="inlineStr"/>
@@ -36665,10 +36837,18 @@
       <c r="H169" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
+      <c r="I169" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J169" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K169" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L169" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M169" t="inlineStr"/>
       <c r="N169" t="inlineStr"/>
       <c r="O169" t="inlineStr"/>
@@ -36777,10 +36957,18 @@
       <c r="H170" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
+      <c r="I170" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J170" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K170" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L170" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="inlineStr"/>
       <c r="O170" t="inlineStr"/>
@@ -36889,10 +37077,18 @@
       <c r="H171" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+      <c r="I171" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J171" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K171" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L171" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M171" t="inlineStr"/>
       <c r="N171" t="inlineStr"/>
       <c r="O171" t="inlineStr"/>
@@ -37221,10 +37417,18 @@
       <c r="H174" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
+      <c r="I174" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J174" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K174" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L174" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M174" t="inlineStr"/>
       <c r="N174" t="inlineStr"/>
       <c r="O174" t="inlineStr"/>
@@ -37333,10 +37537,18 @@
       <c r="H175" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
+      <c r="I175" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J175" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K175" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L175" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
       <c r="O175" t="inlineStr"/>
@@ -37445,10 +37657,18 @@
       <c r="H176" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I176" t="inlineStr"/>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
+      <c r="I176" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J176" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K176" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L176" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M176" t="inlineStr"/>
       <c r="N176" t="inlineStr"/>
       <c r="O176" t="inlineStr"/>
@@ -37557,10 +37777,18 @@
       <c r="H177" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
+      <c r="I177" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J177" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K177" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L177" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
       <c r="O177" t="inlineStr"/>
@@ -37669,10 +37897,18 @@
       <c r="H178" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I178" t="inlineStr"/>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
+      <c r="I178" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J178" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K178" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L178" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr"/>
       <c r="O178" t="inlineStr"/>
@@ -37781,10 +38017,18 @@
       <c r="H179" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I179" t="inlineStr"/>
-      <c r="J179" t="inlineStr"/>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr"/>
+      <c r="I179" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J179" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K179" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L179" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M179" t="inlineStr"/>
       <c r="N179" t="inlineStr"/>
       <c r="O179" t="inlineStr"/>
@@ -37893,10 +38137,18 @@
       <c r="H180" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I180" t="inlineStr"/>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
+      <c r="I180" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J180" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K180" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L180" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr"/>
@@ -38005,10 +38257,18 @@
       <c r="H181" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I181" t="inlineStr"/>
-      <c r="J181" t="inlineStr"/>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr"/>
+      <c r="I181" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J181" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K181" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L181" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M181" t="inlineStr"/>
       <c r="N181" t="inlineStr"/>
       <c r="O181" t="inlineStr"/>
@@ -38117,10 +38377,18 @@
       <c r="H182" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I182" t="inlineStr"/>
-      <c r="J182" t="inlineStr"/>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr"/>
+      <c r="I182" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J182" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K182" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L182" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M182" t="inlineStr"/>
       <c r="N182" t="inlineStr"/>
       <c r="O182" t="inlineStr"/>
@@ -38229,10 +38497,18 @@
       <c r="H183" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I183" t="inlineStr"/>
-      <c r="J183" t="inlineStr"/>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr"/>
+      <c r="I183" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J183" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K183" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L183" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
       <c r="O183" t="inlineStr"/>
@@ -38341,10 +38617,18 @@
       <c r="H184" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
+      <c r="I184" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J184" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K184" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L184" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr"/>
       <c r="O184" t="inlineStr"/>
@@ -38453,10 +38737,18 @@
       <c r="H185" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I185" t="inlineStr"/>
-      <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr"/>
+      <c r="I185" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J185" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K185" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L185" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="inlineStr"/>
       <c r="O185" t="inlineStr"/>
@@ -38675,10 +38967,18 @@
       <c r="H187" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I187" t="inlineStr"/>
-      <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr"/>
+      <c r="I187" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J187" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K187" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L187" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="inlineStr"/>
       <c r="O187" t="inlineStr"/>
@@ -38787,10 +39087,18 @@
       <c r="H188" s="1" t="n">
         <v>46253</v>
       </c>
-      <c r="I188" t="inlineStr"/>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
+      <c r="I188" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="J188" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="K188" s="1" t="n">
+        <v>46343</v>
+      </c>
+      <c r="L188" s="1" t="n">
+        <v>46343</v>
+      </c>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr"/>
       <c r="O188" t="inlineStr"/>
@@ -39229,10 +39537,18 @@
       <c r="H192" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
+      <c r="I192" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J192" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K192" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L192" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
       <c r="O192" t="inlineStr"/>
@@ -39451,10 +39767,18 @@
       <c r="H194" s="1" t="n">
         <v>46252</v>
       </c>
-      <c r="I194" t="inlineStr"/>
-      <c r="J194" t="inlineStr"/>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr"/>
+      <c r="I194" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="J194" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="K194" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="L194" s="1" t="n">
+        <v>46342</v>
+      </c>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr"/>
       <c r="O194" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MY0207: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por YOLANDA, 24/08/2026 13:27)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -23690,12 +23690,12 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>DESTRUCCION</t>
+          <t>DESTRUCCION | [24/08/2026 13:27 · YOLANDA] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
@@ -23790,13 +23790,23 @@
       <c r="AV99" t="inlineStr"/>
       <c r="AW99" t="inlineStr"/>
       <c r="AX99" t="inlineStr"/>
-      <c r="AY99" t="inlineStr"/>
-      <c r="AZ99" t="inlineStr"/>
-      <c r="BA99" t="inlineStr"/>
-      <c r="BB99" t="inlineStr"/>
+      <c r="AY99" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="AZ99" t="inlineStr">
+        <is>
+          <t>YOLANDA</t>
+        </is>
+      </c>
+      <c r="BA99" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="BB99" t="n">
+        <v>26</v>
+      </c>
       <c r="BC99" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD99" t="inlineStr"/>
@@ -23856,12 +23866,12 @@
       </c>
       <c r="BW99" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>YOLANDA</t>
         </is>
       </c>
       <c r="BX99" t="inlineStr">
         <is>
-          <t>2026-08-10 00:00:00</t>
+          <t>24/08/2026 13:27:09</t>
         </is>
       </c>
       <c r="BY99" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL050: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Francisco, 25/08/2026 08:33)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -36344,24 +36344,54 @@
       <c r="N163" t="inlineStr"/>
       <c r="O163" t="inlineStr"/>
       <c r="P163" t="inlineStr"/>
-      <c r="Q163" t="inlineStr"/>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S163" t="inlineStr"/>
       <c r="T163" t="inlineStr"/>
       <c r="U163" t="inlineStr"/>
-      <c r="V163" t="inlineStr"/>
-      <c r="W163" t="inlineStr"/>
-      <c r="X163" t="inlineStr"/>
-      <c r="Y163" t="inlineStr"/>
-      <c r="Z163" t="inlineStr"/>
-      <c r="AA163" t="inlineStr"/>
-      <c r="AB163" t="inlineStr"/>
-      <c r="AC163" t="inlineStr"/>
-      <c r="AD163" t="inlineStr"/>
+      <c r="V163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="X163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="Z163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AB163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC163" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD163" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE163" t="inlineStr"/>
       <c r="AF163" t="inlineStr"/>
       <c r="AG163" t="inlineStr"/>
@@ -36406,8 +36436,16 @@
       <c r="BT163" t="inlineStr"/>
       <c r="BU163" t="inlineStr"/>
       <c r="BV163" t="inlineStr"/>
-      <c r="BW163" t="inlineStr"/>
-      <c r="BX163" t="inlineStr"/>
+      <c r="BW163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BX163" t="inlineStr">
+        <is>
+          <t>25/08/2026 08:33:34</t>
+        </is>
+      </c>
       <c r="BY163" t="inlineStr"/>
       <c r="BZ163" t="inlineStr"/>
       <c r="CA163" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL001: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Francisco, 25/08/2026 08:36)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34218,24 +34218,54 @@
       <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr"/>
-      <c r="Q146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>[25/08/2026 08:36 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S146" t="inlineStr"/>
       <c r="T146" t="inlineStr"/>
       <c r="U146" t="inlineStr"/>
-      <c r="V146" t="inlineStr"/>
-      <c r="W146" t="inlineStr"/>
-      <c r="X146" t="inlineStr"/>
-      <c r="Y146" t="inlineStr"/>
-      <c r="Z146" t="inlineStr"/>
-      <c r="AA146" t="inlineStr"/>
-      <c r="AB146" t="inlineStr"/>
-      <c r="AC146" t="inlineStr"/>
-      <c r="AD146" t="inlineStr"/>
+      <c r="V146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="X146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="Z146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AB146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC146" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE146" t="inlineStr"/>
       <c r="AF146" t="inlineStr"/>
       <c r="AG146" t="inlineStr"/>
@@ -34280,8 +34310,16 @@
       <c r="BT146" t="inlineStr"/>
       <c r="BU146" t="inlineStr"/>
       <c r="BV146" t="inlineStr"/>
-      <c r="BW146" t="inlineStr"/>
-      <c r="BX146" t="inlineStr"/>
+      <c r="BW146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BX146" t="inlineStr">
+        <is>
+          <t>25/08/2026 08:36:24</t>
+        </is>
+      </c>
       <c r="BY146" t="inlineStr"/>
       <c r="BZ146" t="inlineStr"/>
       <c r="CA146" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL001: Etapa 2 TERMINADA · Recolección → pasa a Disposición final (por Francisco, 25/08/2026 08:51)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34220,15 +34220,19 @@
       <c r="P146" t="inlineStr"/>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:36 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[25/08/2026 08:36 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:51 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S146" t="inlineStr"/>
+          <t>Disposición final</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T146" t="inlineStr"/>
       <c r="U146" t="inlineStr"/>
       <c r="V146" s="2" t="n">
@@ -34267,17 +34271,49 @@
         </is>
       </c>
       <c r="AE146" t="inlineStr"/>
-      <c r="AF146" t="inlineStr"/>
-      <c r="AG146" t="inlineStr"/>
-      <c r="AH146" t="inlineStr"/>
-      <c r="AI146" t="inlineStr"/>
-      <c r="AJ146" t="inlineStr"/>
-      <c r="AK146" t="inlineStr"/>
-      <c r="AL146" t="inlineStr"/>
-      <c r="AM146" t="inlineStr"/>
-      <c r="AN146" t="inlineStr"/>
-      <c r="AO146" t="inlineStr"/>
-      <c r="AP146" t="inlineStr"/>
+      <c r="AF146" t="inlineStr">
+        <is>
+          <t>Recolecta proveedor el 28 de agosto</t>
+        </is>
+      </c>
+      <c r="AG146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AH146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AI146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AJ146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AK146" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AL146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AM146" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="AN146" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="AO146" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP146" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ146" t="inlineStr"/>
       <c r="AR146" t="inlineStr"/>
       <c r="AS146" t="inlineStr"/>
@@ -34291,7 +34327,11 @@
       <c r="BA146" t="inlineStr"/>
       <c r="BB146" t="inlineStr"/>
       <c r="BC146" t="inlineStr"/>
-      <c r="BD146" t="inlineStr"/>
+      <c r="BD146" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE146" t="inlineStr"/>
       <c r="BF146" t="inlineStr"/>
       <c r="BG146" t="inlineStr"/>
@@ -34308,7 +34348,9 @@
       <c r="BR146" t="inlineStr"/>
       <c r="BS146" t="inlineStr"/>
       <c r="BT146" t="inlineStr"/>
-      <c r="BU146" t="inlineStr"/>
+      <c r="BU146" s="2" t="n">
+        <v>46279</v>
+      </c>
       <c r="BV146" t="inlineStr"/>
       <c r="BW146" t="inlineStr">
         <is>
@@ -34317,7 +34359,7 @@
       </c>
       <c r="BX146" t="inlineStr">
         <is>
-          <t>25/08/2026 08:36:24</t>
+          <t>25/08/2026 08:51:33</t>
         </is>
       </c>
       <c r="BY146" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL038: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Francisco, 25/08/2026 08:53)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34422,24 +34422,54 @@
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>[25/08/2026 08:53 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S147" t="inlineStr"/>
       <c r="T147" t="inlineStr"/>
       <c r="U147" t="inlineStr"/>
-      <c r="V147" t="inlineStr"/>
-      <c r="W147" t="inlineStr"/>
-      <c r="X147" t="inlineStr"/>
-      <c r="Y147" t="inlineStr"/>
-      <c r="Z147" t="inlineStr"/>
-      <c r="AA147" t="inlineStr"/>
-      <c r="AB147" t="inlineStr"/>
-      <c r="AC147" t="inlineStr"/>
-      <c r="AD147" t="inlineStr"/>
+      <c r="V147" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="X147" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="Z147" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AB147" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC147" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE147" t="inlineStr"/>
       <c r="AF147" t="inlineStr"/>
       <c r="AG147" t="inlineStr"/>
@@ -34484,8 +34514,16 @@
       <c r="BT147" t="inlineStr"/>
       <c r="BU147" t="inlineStr"/>
       <c r="BV147" t="inlineStr"/>
-      <c r="BW147" t="inlineStr"/>
-      <c r="BX147" t="inlineStr"/>
+      <c r="BW147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BX147" t="inlineStr">
+        <is>
+          <t>25/08/2026 08:53:40</t>
+        </is>
+      </c>
       <c r="BY147" t="inlineStr"/>
       <c r="BZ147" t="inlineStr"/>
       <c r="CA147" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL003: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Francisco, 25/08/2026 08:54)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34584,24 +34584,54 @@
       <c r="N148" t="inlineStr"/>
       <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>[25/08/2026 08:54 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S148" t="inlineStr"/>
       <c r="T148" t="inlineStr"/>
       <c r="U148" t="inlineStr"/>
-      <c r="V148" t="inlineStr"/>
-      <c r="W148" t="inlineStr"/>
-      <c r="X148" t="inlineStr"/>
-      <c r="Y148" t="inlineStr"/>
-      <c r="Z148" t="inlineStr"/>
-      <c r="AA148" t="inlineStr"/>
-      <c r="AB148" t="inlineStr"/>
-      <c r="AC148" t="inlineStr"/>
-      <c r="AD148" t="inlineStr"/>
+      <c r="V148" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="X148" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="Z148" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AB148" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC148" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE148" t="inlineStr"/>
       <c r="AF148" t="inlineStr"/>
       <c r="AG148" t="inlineStr"/>
@@ -34646,8 +34676,16 @@
       <c r="BT148" t="inlineStr"/>
       <c r="BU148" t="inlineStr"/>
       <c r="BV148" t="inlineStr"/>
-      <c r="BW148" t="inlineStr"/>
-      <c r="BX148" t="inlineStr"/>
+      <c r="BW148" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BX148" t="inlineStr">
+        <is>
+          <t>25/08/2026 08:54:18</t>
+        </is>
+      </c>
       <c r="BY148" t="inlineStr"/>
       <c r="BZ148" t="inlineStr"/>
       <c r="CA148" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL050: Etapa 2 TERMINADA · Recolección → pasa a Disposición final (por Francisco, 25/08/2026 08:55)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -36502,15 +36502,19 @@
       <c r="P163" t="inlineStr"/>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S163" t="inlineStr"/>
+          <t>Disposición final</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T163" t="inlineStr"/>
       <c r="U163" t="inlineStr"/>
       <c r="V163" s="2" t="n">
@@ -36549,17 +36553,49 @@
         </is>
       </c>
       <c r="AE163" t="inlineStr"/>
-      <c r="AF163" t="inlineStr"/>
-      <c r="AG163" t="inlineStr"/>
-      <c r="AH163" t="inlineStr"/>
-      <c r="AI163" t="inlineStr"/>
-      <c r="AJ163" t="inlineStr"/>
-      <c r="AK163" t="inlineStr"/>
-      <c r="AL163" t="inlineStr"/>
-      <c r="AM163" t="inlineStr"/>
-      <c r="AN163" t="inlineStr"/>
-      <c r="AO163" t="inlineStr"/>
-      <c r="AP163" t="inlineStr"/>
+      <c r="AF163" t="inlineStr">
+        <is>
+          <t>Proveedor recolecta el 25 de agosto</t>
+        </is>
+      </c>
+      <c r="AG163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AH163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AI163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AJ163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AK163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AL163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AM163" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AN163" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="AO163" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP163" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ163" t="inlineStr"/>
       <c r="AR163" t="inlineStr"/>
       <c r="AS163" t="inlineStr"/>
@@ -36573,7 +36609,11 @@
       <c r="BA163" t="inlineStr"/>
       <c r="BB163" t="inlineStr"/>
       <c r="BC163" t="inlineStr"/>
-      <c r="BD163" t="inlineStr"/>
+      <c r="BD163" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE163" t="inlineStr"/>
       <c r="BF163" t="inlineStr"/>
       <c r="BG163" t="inlineStr"/>
@@ -36590,7 +36630,9 @@
       <c r="BR163" t="inlineStr"/>
       <c r="BS163" t="inlineStr"/>
       <c r="BT163" t="inlineStr"/>
-      <c r="BU163" t="inlineStr"/>
+      <c r="BU163" s="2" t="n">
+        <v>46279</v>
+      </c>
       <c r="BV163" t="inlineStr"/>
       <c r="BW163" t="inlineStr">
         <is>
@@ -36599,7 +36641,7 @@
       </c>
       <c r="BX163" t="inlineStr">
         <is>
-          <t>25/08/2026 08:33:34</t>
+          <t>25/08/2026 08:55:51</t>
         </is>
       </c>
       <c r="BY163" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL026: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Francisco, 25/08/2026 08:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -38904,24 +38904,54 @@
       <c r="N181" t="inlineStr"/>
       <c r="O181" t="inlineStr"/>
       <c r="P181" t="inlineStr"/>
-      <c r="Q181" t="inlineStr"/>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>[25/08/2026 08:56 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R181" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S181" t="inlineStr"/>
       <c r="T181" t="inlineStr"/>
       <c r="U181" t="inlineStr"/>
-      <c r="V181" t="inlineStr"/>
-      <c r="W181" t="inlineStr"/>
-      <c r="X181" t="inlineStr"/>
-      <c r="Y181" t="inlineStr"/>
-      <c r="Z181" t="inlineStr"/>
-      <c r="AA181" t="inlineStr"/>
-      <c r="AB181" t="inlineStr"/>
-      <c r="AC181" t="inlineStr"/>
-      <c r="AD181" t="inlineStr"/>
+      <c r="V181" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="X181" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="Z181" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AB181" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>7</v>
+      </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE181" t="inlineStr"/>
       <c r="AF181" t="inlineStr"/>
       <c r="AG181" t="inlineStr"/>
@@ -38966,8 +38996,16 @@
       <c r="BT181" t="inlineStr"/>
       <c r="BU181" t="inlineStr"/>
       <c r="BV181" t="inlineStr"/>
-      <c r="BW181" t="inlineStr"/>
-      <c r="BX181" t="inlineStr"/>
+      <c r="BW181" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BX181" t="inlineStr">
+        <is>
+          <t>25/08/2026 08:56:52</t>
+        </is>
+      </c>
       <c r="BY181" t="inlineStr"/>
       <c r="BZ181" t="inlineStr"/>
       <c r="CA181" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL038: Etapa 2 TERMINADA · Destrucción → pasa a Disposición final (por Francisco, 29/08/2026 13:02)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34424,15 +34424,19 @@
       <c r="P147" t="inlineStr"/>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:53 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[25/08/2026 08:53 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [29/08/2026 13:02 · Francisco] Etapa 2 TERMINADA · Destrucción → pasa a Disposición final</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S147" t="inlineStr"/>
+          <t>Disposición final</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="T147" t="inlineStr"/>
       <c r="U147" t="inlineStr"/>
       <c r="V147" s="2" t="n">
@@ -34471,17 +34475,47 @@
         </is>
       </c>
       <c r="AE147" t="inlineStr"/>
-      <c r="AF147" t="inlineStr"/>
-      <c r="AG147" t="inlineStr"/>
-      <c r="AH147" t="inlineStr"/>
-      <c r="AI147" t="inlineStr"/>
-      <c r="AJ147" t="inlineStr"/>
-      <c r="AK147" t="inlineStr"/>
-      <c r="AL147" t="inlineStr"/>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>Se compartio al proveedor la evidencia de la destrucción, en espera de la nota de credito.</t>
+        </is>
+      </c>
+      <c r="AG147" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="AH147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AI147" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="AK147" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="AL147" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
       <c r="AM147" t="inlineStr"/>
-      <c r="AN147" t="inlineStr"/>
-      <c r="AO147" t="inlineStr"/>
-      <c r="AP147" t="inlineStr"/>
+      <c r="AN147" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="AO147" t="n">
+        <v>4</v>
+      </c>
+      <c r="AP147" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ147" t="inlineStr"/>
       <c r="AR147" t="inlineStr"/>
       <c r="AS147" t="inlineStr"/>
@@ -34495,7 +34529,11 @@
       <c r="BA147" t="inlineStr"/>
       <c r="BB147" t="inlineStr"/>
       <c r="BC147" t="inlineStr"/>
-      <c r="BD147" t="inlineStr"/>
+      <c r="BD147" t="inlineStr">
+        <is>
+          <t>Destrucción</t>
+        </is>
+      </c>
       <c r="BE147" t="inlineStr"/>
       <c r="BF147" t="inlineStr"/>
       <c r="BG147" t="inlineStr"/>
@@ -34521,7 +34559,7 @@
       </c>
       <c r="BX147" t="inlineStr">
         <is>
-          <t>25/08/2026 08:53:40</t>
+          <t>29/08/2026 13:02:27</t>
         </is>
       </c>
       <c r="BY147" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL003: Avance en Gestión (por Francisco, 29/08/2026 13:03)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34624,7 +34624,7 @@
       <c r="P148" t="inlineStr"/>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:54 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[25/08/2026 08:54 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [29/08/2026 13:03 · Francisco] Avance en Gestión</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -34632,7 +34632,11 @@
           <t>Gestión</t>
         </is>
       </c>
-      <c r="S148" t="inlineStr"/>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T148" t="inlineStr"/>
       <c r="U148" t="inlineStr"/>
       <c r="V148" s="2" t="n">
@@ -34671,15 +34675,23 @@
         </is>
       </c>
       <c r="AE148" t="inlineStr"/>
-      <c r="AF148" t="inlineStr"/>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>En proceso de recolección por parte del proveedor.</t>
+        </is>
+      </c>
       <c r="AG148" t="inlineStr"/>
       <c r="AH148" t="inlineStr"/>
       <c r="AI148" t="inlineStr"/>
       <c r="AJ148" t="inlineStr"/>
       <c r="AK148" t="inlineStr"/>
       <c r="AL148" t="inlineStr"/>
-      <c r="AM148" t="inlineStr"/>
-      <c r="AN148" t="inlineStr"/>
+      <c r="AM148" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="AN148" s="2" t="n">
+        <v>46289</v>
+      </c>
       <c r="AO148" t="inlineStr"/>
       <c r="AP148" t="inlineStr"/>
       <c r="AQ148" t="inlineStr"/>
@@ -34721,7 +34733,7 @@
       </c>
       <c r="BX148" t="inlineStr">
         <is>
-          <t>25/08/2026 08:54:18</t>
+          <t>29/08/2026 13:03:48</t>
         </is>
       </c>
       <c r="BY148" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL050: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por Francisco, 29/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -36552,12 +36552,12 @@
       <c r="P163" t="inlineStr"/>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
+          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [29/08/2026 13:06 · Francisco] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S163" t="inlineStr">
@@ -36665,7 +36665,13 @@
         </is>
       </c>
       <c r="BE163" t="inlineStr"/>
-      <c r="BF163" t="inlineStr"/>
+      <c r="BF163" t="inlineStr">
+        <is>
+          <t>Se realizó la devolución a proveedor, las notas de credito ya fueron generadas. 
+De este folio quedo pendiente la clave 29138 ya que el producto fisicamente no pertenece a esa clave. 
+Devoluciones hara el ajuste correspondiente para pasarlo a su clave correcta y poder enviar a proveedor.</t>
+        </is>
+      </c>
       <c r="BG163" t="inlineStr"/>
       <c r="BH163" t="inlineStr"/>
       <c r="BI163" t="inlineStr"/>
@@ -36674,16 +36680,38 @@
       <c r="BL163" t="inlineStr"/>
       <c r="BM163" t="inlineStr"/>
       <c r="BN163" t="inlineStr"/>
-      <c r="BO163" t="inlineStr"/>
-      <c r="BP163" t="inlineStr"/>
-      <c r="BQ163" t="inlineStr"/>
-      <c r="BR163" t="inlineStr"/>
-      <c r="BS163" t="inlineStr"/>
-      <c r="BT163" t="inlineStr"/>
+      <c r="BO163" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BP163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BQ163" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BR163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BS163" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BT163" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
       <c r="BU163" s="2" t="n">
         <v>46279</v>
       </c>
-      <c r="BV163" t="inlineStr"/>
+      <c r="BV163" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW163" t="inlineStr">
         <is>
           <t>Francisco</t>
@@ -36691,7 +36719,7 @@
       </c>
       <c r="BX163" t="inlineStr">
         <is>
-          <t>25/08/2026 08:55:51</t>
+          <t>29/08/2026 13:06:47</t>
         </is>
       </c>
       <c r="BY163" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL001: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por Francisco, 29/08/2026 13:14)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -34220,12 +34220,12 @@
       <c r="P146" t="inlineStr"/>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:36 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:51 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
+          <t>[25/08/2026 08:36 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:51 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [29/08/2026 13:14 · Francisco] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S146" t="inlineStr">
@@ -34333,7 +34333,11 @@
         </is>
       </c>
       <c r="BE146" t="inlineStr"/>
-      <c r="BF146" t="inlineStr"/>
+      <c r="BF146" t="inlineStr">
+        <is>
+          <t>Proveedor recolecto el material, se tuvieron unas incidencias de unos productos no encontrados fisicamente vs el reporte original</t>
+        </is>
+      </c>
       <c r="BG146" t="inlineStr"/>
       <c r="BH146" t="inlineStr"/>
       <c r="BI146" t="inlineStr"/>
@@ -34342,16 +34346,38 @@
       <c r="BL146" t="inlineStr"/>
       <c r="BM146" t="inlineStr"/>
       <c r="BN146" t="inlineStr"/>
-      <c r="BO146" t="inlineStr"/>
-      <c r="BP146" t="inlineStr"/>
-      <c r="BQ146" t="inlineStr"/>
-      <c r="BR146" t="inlineStr"/>
-      <c r="BS146" t="inlineStr"/>
-      <c r="BT146" t="inlineStr"/>
+      <c r="BO146" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BP146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BQ146" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BR146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
+      <c r="BS146" s="2" t="n">
+        <v>46263</v>
+      </c>
+      <c r="BT146" t="inlineStr">
+        <is>
+          <t>Francisco</t>
+        </is>
+      </c>
       <c r="BU146" s="2" t="n">
         <v>46279</v>
       </c>
-      <c r="BV146" t="inlineStr"/>
+      <c r="BV146" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW146" t="inlineStr">
         <is>
           <t>Francisco</t>
@@ -34359,7 +34385,7 @@
       </c>
       <c r="BX146" t="inlineStr">
         <is>
-          <t>25/08/2026 08:51:33</t>
+          <t>29/08/2026 13:14:23</t>
         </is>
       </c>
       <c r="BY146" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Avance en Disposición final (por yolanda, 01/09/2026 08:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8453,7 +8453,11 @@
         </is>
       </c>
       <c r="BE34" t="inlineStr"/>
-      <c r="BF34" t="inlineStr"/>
+      <c r="BF34" t="inlineStr">
+        <is>
+          <t>cambio fisico</t>
+        </is>
+      </c>
       <c r="BG34" t="inlineStr"/>
       <c r="BH34" t="inlineStr"/>
       <c r="BI34" t="inlineStr"/>
@@ -8464,8 +8468,14 @@
       <c r="BN34" t="inlineStr"/>
       <c r="BO34" t="inlineStr"/>
       <c r="BP34" t="inlineStr"/>
-      <c r="BQ34" t="inlineStr"/>
-      <c r="BR34" t="inlineStr"/>
+      <c r="BQ34" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BR34" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BS34" t="inlineStr"/>
       <c r="BT34" t="inlineStr"/>
       <c r="BU34" s="2" t="n">
@@ -8476,8 +8486,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BW34" t="inlineStr"/>
-      <c r="BX34" t="inlineStr"/>
+      <c r="BW34" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX34" t="inlineStr">
+        <is>
+          <t>01/09/2026 08:11:53</t>
+        </is>
+      </c>
       <c r="BY34" t="inlineStr"/>
       <c r="BZ34" t="inlineStr"/>
       <c r="CA34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Avance en Disposición final (por yolanda, 01/09/2026 08:13)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:11:58</t>
+          <t>01/09/2026 08:13:36</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Avance en Disposición final (por yolanda, 01/09/2026 08:14)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:13:36</t>
+          <t>01/09/2026 08:14:20</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Avance en Disposición final (por Yolanda Jeronimo, 01/09/2026 08:17)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8488,12 +8488,12 @@
       </c>
       <c r="BW34" t="inlineStr">
         <is>
-          <t>yolanda</t>
+          <t>Yolanda Jeronimo</t>
         </is>
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:14:20</t>
+          <t>01/09/2026 08:17:34</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Avance en Disposición final (por Yolanda Jeronimo, 01/09/2026 08:18)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,7 +8334,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:18 · Yolanda Jeronimo] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:17:55</t>
+          <t>01/09/2026 08:18:08</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 08:21)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,12 +8334,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:18 · Yolanda Jeronimo] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:18 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:21 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -8453,11 +8453,7 @@
         </is>
       </c>
       <c r="BE34" t="inlineStr"/>
-      <c r="BF34" t="inlineStr">
-        <is>
-          <t>cambio fisico</t>
-        </is>
-      </c>
+      <c r="BF34" t="inlineStr"/>
       <c r="BG34" t="inlineStr"/>
       <c r="BH34" t="inlineStr"/>
       <c r="BI34" t="inlineStr"/>
@@ -8468,32 +8464,32 @@
       <c r="BN34" t="inlineStr"/>
       <c r="BO34" t="inlineStr"/>
       <c r="BP34" t="inlineStr"/>
-      <c r="BQ34" s="2" t="n">
+      <c r="BQ34" t="inlineStr"/>
+      <c r="BR34" t="inlineStr"/>
+      <c r="BS34" s="2" t="n">
         <v>46266</v>
       </c>
-      <c r="BR34" t="inlineStr">
+      <c r="BT34" t="inlineStr">
         <is>
           <t>yolanda</t>
         </is>
       </c>
-      <c r="BS34" t="inlineStr"/>
-      <c r="BT34" t="inlineStr"/>
       <c r="BU34" s="2" t="n">
         <v>46229</v>
       </c>
       <c r="BV34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW34" t="inlineStr">
         <is>
-          <t>Yolanda Jeronimo</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:18:08</t>
+          <t>01/09/2026 08:21:07</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-MZ033: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por Yolanda Jeronimo, 01/09/2026 08:21)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8334,12 +8334,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:18 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:21 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>DEVOLUCION | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:11 · yolanda] Avance en Disposición final | [01/09/2026 08:13 · yolanda] Avance en Disposición final | [01/09/2026 08:14 · yolanda] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:17 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:18 · Yolanda Jeronimo] Avance en Disposición final | [01/09/2026 08:21 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar | [01/09/2026 08:21 · Yolanda Jeronimo] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -8438,13 +8438,23 @@
       <c r="AV34" t="inlineStr"/>
       <c r="AW34" t="inlineStr"/>
       <c r="AX34" t="inlineStr"/>
-      <c r="AY34" t="inlineStr"/>
-      <c r="AZ34" t="inlineStr"/>
-      <c r="BA34" t="inlineStr"/>
-      <c r="BB34" t="inlineStr"/>
+      <c r="AY34" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t>Yolanda Jeronimo</t>
+        </is>
+      </c>
+      <c r="BA34" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="BB34" t="n">
+        <v>87</v>
+      </c>
       <c r="BC34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD34" t="inlineStr">
@@ -8484,12 +8494,12 @@
       </c>
       <c r="BW34" t="inlineStr">
         <is>
-          <t>yolanda</t>
+          <t>Yolanda Jeronimo</t>
         </is>
       </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>01/09/2026 08:21:07</t>
+          <t>01/09/2026 08:21:36</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB041: Avance en Disposición final (por yolanda, 01/09/2026 08:23)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20904,7 +20904,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 08:23 · yolanda] Avance en Disposición final</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -21019,7 +21019,11 @@
         </is>
       </c>
       <c r="BE86" t="inlineStr"/>
-      <c r="BF86" t="inlineStr"/>
+      <c r="BF86" t="inlineStr">
+        <is>
+          <t>cambio fisico</t>
+        </is>
+      </c>
       <c r="BG86" t="inlineStr"/>
       <c r="BH86" t="inlineStr"/>
       <c r="BI86" t="inlineStr"/>
@@ -21030,8 +21034,14 @@
       <c r="BN86" t="inlineStr"/>
       <c r="BO86" t="inlineStr"/>
       <c r="BP86" t="inlineStr"/>
-      <c r="BQ86" t="inlineStr"/>
-      <c r="BR86" t="inlineStr"/>
+      <c r="BQ86" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BR86" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BS86" t="inlineStr"/>
       <c r="BT86" t="inlineStr"/>
       <c r="BU86" s="2" t="n">
@@ -21042,8 +21052,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="BW86" t="inlineStr"/>
-      <c r="BX86" t="inlineStr"/>
+      <c r="BW86" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX86" t="inlineStr">
+        <is>
+          <t>01/09/2026 08:23:53</t>
+        </is>
+      </c>
       <c r="BY86" t="inlineStr"/>
       <c r="BZ86" t="inlineStr"/>
       <c r="CA86" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB041: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 08:24)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20904,12 +20904,12 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:23 · yolanda] Avance en Disposición final | [01/09/2026 08:23 · yolanda] Avance en Disposición final</t>
+          <t>DEVOLUCION | [01/09/2026 08:23 · yolanda] Avance en Disposición final | [01/09/2026 08:24 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -21034,22 +21034,22 @@
       <c r="BN86" t="inlineStr"/>
       <c r="BO86" t="inlineStr"/>
       <c r="BP86" t="inlineStr"/>
-      <c r="BQ86" s="2" t="n">
+      <c r="BQ86" t="inlineStr"/>
+      <c r="BR86" t="inlineStr"/>
+      <c r="BS86" s="2" t="n">
         <v>46266</v>
       </c>
-      <c r="BR86" t="inlineStr">
+      <c r="BT86" t="inlineStr">
         <is>
           <t>yolanda</t>
         </is>
       </c>
-      <c r="BS86" t="inlineStr"/>
-      <c r="BT86" t="inlineStr"/>
       <c r="BU86" s="2" t="n">
         <v>46252</v>
       </c>
       <c r="BV86" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BW86" t="inlineStr">
@@ -21059,7 +21059,7 @@
       </c>
       <c r="BX86" t="inlineStr">
         <is>
-          <t>01/09/2026 08:23:55</t>
+          <t>01/09/2026 08:24:16</t>
         </is>
       </c>
       <c r="BY86" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB041: Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO (por Yolanda Jeronimo, 01/09/2026 08:25)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20904,12 +20904,12 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:23 · yolanda] Avance en Disposición final | [01/09/2026 08:24 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>DEVOLUCION | [01/09/2026 08:23 · yolanda] Avance en Disposición final | [01/09/2026 08:24 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar | [01/09/2026 08:25 · Yolanda Jeronimo] Etapa Cuentas por pagar TERMINADA · PROCESO FINALIZADO</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Cuentas por pagar</t>
+          <t>FINALIZADO</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -20995,7 +20995,7 @@
       <c r="AQ86" t="inlineStr"/>
       <c r="AR86" t="inlineStr">
         <is>
-          <t>Recolección</t>
+          <t>cambio fisico</t>
         </is>
       </c>
       <c r="AS86" t="inlineStr"/>
@@ -21004,13 +21004,23 @@
       <c r="AV86" t="inlineStr"/>
       <c r="AW86" t="inlineStr"/>
       <c r="AX86" t="inlineStr"/>
-      <c r="AY86" t="inlineStr"/>
-      <c r="AZ86" t="inlineStr"/>
-      <c r="BA86" t="inlineStr"/>
-      <c r="BB86" t="inlineStr"/>
+      <c r="AY86" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AZ86" t="inlineStr">
+        <is>
+          <t>Yolanda Jeronimo</t>
+        </is>
+      </c>
+      <c r="BA86" s="2" t="n">
+        <v>46252</v>
+      </c>
+      <c r="BB86" t="n">
+        <v>67</v>
+      </c>
       <c r="BC86" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="BD86" t="inlineStr">
@@ -21054,12 +21064,12 @@
       </c>
       <c r="BW86" t="inlineStr">
         <is>
-          <t>yolanda</t>
+          <t>Yolanda Jeronimo</t>
         </is>
       </c>
       <c r="BX86" t="inlineStr">
         <is>
-          <t>01/09/2026 08:24:16</t>
+          <t>01/09/2026 08:25:57</t>
         </is>
       </c>
       <c r="BY86" t="inlineStr"/>
@@ -21069,7 +21079,11 @@
       <c r="CC86" t="inlineStr"/>
       <c r="CD86" t="inlineStr"/>
       <c r="CE86" t="inlineStr"/>
-      <c r="CF86" t="inlineStr"/>
+      <c r="CF86" t="inlineStr">
+        <is>
+          <t>8422</t>
+        </is>
+      </c>
       <c r="CG86" t="inlineStr"/>
       <c r="CH86" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB022: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 08:36)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -17554,12 +17554,12 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 08:36 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
@@ -17669,7 +17669,11 @@
         </is>
       </c>
       <c r="BE71" t="inlineStr"/>
-      <c r="BF71" t="inlineStr"/>
+      <c r="BF71" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
       <c r="BG71" t="inlineStr"/>
       <c r="BH71" t="inlineStr"/>
       <c r="BI71" t="inlineStr"/>
@@ -17680,20 +17684,40 @@
       <c r="BN71" t="inlineStr"/>
       <c r="BO71" t="inlineStr"/>
       <c r="BP71" t="inlineStr"/>
-      <c r="BQ71" t="inlineStr"/>
-      <c r="BR71" t="inlineStr"/>
-      <c r="BS71" t="inlineStr"/>
-      <c r="BT71" t="inlineStr"/>
+      <c r="BQ71" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BR71" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BS71" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT71" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU71" s="2" t="n">
         <v>46244</v>
       </c>
       <c r="BV71" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BW71" t="inlineStr"/>
-      <c r="BX71" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="BW71" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX71" t="inlineStr">
+        <is>
+          <t>01/09/2026 08:36:42</t>
+        </is>
+      </c>
       <c r="BY71" t="inlineStr">
         <is>
           <t>SÍ</t>
@@ -21081,7 +21105,7 @@
       <c r="CE86" t="inlineStr"/>
       <c r="CF86" t="inlineStr">
         <is>
-          <t>8422</t>
+          <t>8422.0</t>
         </is>
       </c>
       <c r="CG86" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB022: Avance en Cuentas por pagar (por yolanda, 01/09/2026 08:40)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -17554,7 +17554,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>DEVOLUCION | [01/09/2026 08:36 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>DEVOLUCION | [01/09/2026 08:36 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar | [01/09/2026 08:40 · yolanda] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -17650,13 +17650,21 @@
       </c>
       <c r="AS71" t="inlineStr"/>
       <c r="AT71" t="inlineStr"/>
-      <c r="AU71" t="inlineStr"/>
-      <c r="AV71" t="inlineStr"/>
+      <c r="AU71" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="AW71" t="inlineStr"/>
       <c r="AX71" t="inlineStr"/>
       <c r="AY71" t="inlineStr"/>
       <c r="AZ71" t="inlineStr"/>
-      <c r="BA71" t="inlineStr"/>
+      <c r="BA71" s="2" t="n">
+        <v>46252</v>
+      </c>
       <c r="BB71" t="inlineStr"/>
       <c r="BC71" t="inlineStr">
         <is>
@@ -17715,7 +17723,7 @@
       </c>
       <c r="BX71" t="inlineStr">
         <is>
-          <t>01/09/2026 08:36:42</t>
+          <t>01/09/2026 08:40:25</t>
         </is>
       </c>
       <c r="BY71" t="inlineStr">
@@ -17739,7 +17747,11 @@
         </is>
       </c>
       <c r="CE71" t="inlineStr"/>
-      <c r="CF71" t="inlineStr"/>
+      <c r="CF71" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
       <c r="CG71" t="inlineStr"/>
       <c r="CH71" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Folio DC-AB038: Avance en Cuentas por pagar (por Yolanda Jeronimo, 01/09/2026 08:50)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -17749,7 +17749,7 @@
       <c r="CE71" t="inlineStr"/>
       <c r="CF71" t="inlineStr">
         <is>
-          <t>8427</t>
+          <t>8427.0</t>
         </is>
       </c>
       <c r="CG71" t="inlineStr"/>
@@ -20504,7 +20504,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -20692,12 +20692,12 @@
       </c>
       <c r="BW84" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>Yolanda Jeronimo</t>
         </is>
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>13/07/2026 13:43:39</t>
+          <t>01/09/2026 08:50:33</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">
@@ -20723,7 +20723,7 @@
       <c r="CE84" t="inlineStr"/>
       <c r="CF84" t="inlineStr">
         <is>
-          <t>8359.0</t>
+          <t>8359</t>
         </is>
       </c>
       <c r="CG84" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB038: Avance en Cuentas por pagar (por yolanda, 01/09/2026 08:51)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20504,7 +20504,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -20692,12 +20692,12 @@
       </c>
       <c r="BW84" t="inlineStr">
         <is>
-          <t>Yolanda Jeronimo</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>01/09/2026 08:50:34</t>
+          <t>01/09/2026 08:51:38</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">
@@ -20723,7 +20723,7 @@
       <c r="CE84" t="inlineStr"/>
       <c r="CF84" t="inlineStr">
         <is>
-          <t>8359</t>
+          <t>8359.0</t>
         </is>
       </c>
       <c r="CG84" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-AB038: Avance en Cuentas por pagar (por Yolanda Jeronimo, 01/09/2026 08:51)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20504,7 +20504,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:51 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -20692,12 +20692,12 @@
       </c>
       <c r="BW84" t="inlineStr">
         <is>
-          <t>yolanda</t>
+          <t>Yolanda Jeronimo</t>
         </is>
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>01/09/2026 08:51:38</t>
+          <t>01/09/2026 08:51:40</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-AB038: Avance en Cuentas por pagar (por Yolanda Jeronimo, 01/09/2026 08:53)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20504,7 +20504,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:51 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -20697,7 +20697,7 @@
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>01/09/2026 08:51:40</t>
+          <t>01/09/2026 08:53:56</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-AB038: Avance en Cuentas por pagar (por Yolanda Jeronimo, 01/09/2026 08:57)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20504,7 +20504,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:57 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -20697,7 +20697,7 @@
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>01/09/2026 08:53:56</t>
+          <t>01/09/2026 08:57:20</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-AB038: 1 reclamación(es) de INTERRUPTORES Y GABINETES ELECTRICOS SA DE CV liberadas de cuarentena → Reporte de reclamo (por Admin cuarentena, 01/09/2026 09:10)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -20504,12 +20504,12 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:57 · Yolanda Jeronimo] Avance en Cuentas por pagar</t>
+          <t>DEVOLUCION 8359 | [01/09/2026 08:50 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:51 · yolanda] Avance en Cuentas por pagar | [01/09/2026 08:53 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 08:57 · Yolanda Jeronimo] Avance en Cuentas por pagar | [01/09/2026 09:10 · Admin cuarentena] 1 reclamación(es) de INTERRUPTORES Y GABINETES ELECTRICOS SA DE CV liberadas de cuarentena → Reporte de reclamo</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -20692,17 +20692,17 @@
       </c>
       <c r="BW84" t="inlineStr">
         <is>
-          <t>Yolanda Jeronimo</t>
+          <t>Admin cuarentena</t>
         </is>
       </c>
       <c r="BX84" t="inlineStr">
         <is>
-          <t>01/09/2026 08:57:20</t>
+          <t>01/09/2026 09:10:52</t>
         </is>
       </c>
       <c r="BY84" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>LIBERADA</t>
         </is>
       </c>
       <c r="BZ84" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-MY010: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por Yolanda Jeronimo, 01/09/2026 09:53)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -22422,12 +22422,12 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 09:53 · Yolanda Jeronimo] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
@@ -22537,7 +22537,11 @@
         </is>
       </c>
       <c r="BE93" t="inlineStr"/>
-      <c r="BF93" t="inlineStr"/>
+      <c r="BF93" t="inlineStr">
+        <is>
+          <t>8435 pend-46386  --1 pza</t>
+        </is>
+      </c>
       <c r="BG93" t="inlineStr"/>
       <c r="BH93" t="inlineStr"/>
       <c r="BI93" t="inlineStr"/>
@@ -22550,18 +22554,32 @@
       <c r="BP93" t="inlineStr"/>
       <c r="BQ93" t="inlineStr"/>
       <c r="BR93" t="inlineStr"/>
-      <c r="BS93" t="inlineStr"/>
-      <c r="BT93" t="inlineStr"/>
+      <c r="BS93" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT93" t="inlineStr">
+        <is>
+          <t>Yolanda Jeronimo</t>
+        </is>
+      </c>
       <c r="BU93" s="2" t="n">
         <v>46285</v>
       </c>
       <c r="BV93" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BW93" t="inlineStr"/>
-      <c r="BX93" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="BW93" t="inlineStr">
+        <is>
+          <t>Yolanda Jeronimo</t>
+        </is>
+      </c>
+      <c r="BX93" t="inlineStr">
+        <is>
+          <t>01/09/2026 09:53:13</t>
+        </is>
+      </c>
       <c r="BY93" t="inlineStr"/>
       <c r="BZ93" t="inlineStr"/>
       <c r="CA93" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JN006: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 09:56)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -28880,12 +28880,12 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 09:56 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
@@ -28995,7 +28995,11 @@
         </is>
       </c>
       <c r="BE121" t="inlineStr"/>
-      <c r="BF121" t="inlineStr"/>
+      <c r="BF121" t="inlineStr">
+        <is>
+          <t>8427</t>
+        </is>
+      </c>
       <c r="BG121" t="inlineStr"/>
       <c r="BH121" t="inlineStr"/>
       <c r="BI121" t="inlineStr"/>
@@ -29008,18 +29012,32 @@
       <c r="BP121" t="inlineStr"/>
       <c r="BQ121" t="inlineStr"/>
       <c r="BR121" t="inlineStr"/>
-      <c r="BS121" t="inlineStr"/>
-      <c r="BT121" t="inlineStr"/>
+      <c r="BS121" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT121" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU121" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="BV121" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BW121" t="inlineStr"/>
-      <c r="BX121" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="BW121" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX121" t="inlineStr">
+        <is>
+          <t>01/09/2026 09:56:52</t>
+        </is>
+      </c>
       <c r="BY121" t="inlineStr"/>
       <c r="BZ121" t="inlineStr"/>
       <c r="CA121" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JN015: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 10:07)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -30240,12 +30240,12 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>DEVOLUCION</t>
+          <t>DEVOLUCION | [01/09/2026 10:07 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S127" t="inlineStr">
@@ -30355,7 +30355,11 @@
         </is>
       </c>
       <c r="BE127" t="inlineStr"/>
-      <c r="BF127" t="inlineStr"/>
+      <c r="BF127" t="inlineStr">
+        <is>
+          <t>8429</t>
+        </is>
+      </c>
       <c r="BG127" t="inlineStr"/>
       <c r="BH127" t="inlineStr"/>
       <c r="BI127" t="inlineStr"/>
@@ -30368,18 +30372,32 @@
       <c r="BP127" t="inlineStr"/>
       <c r="BQ127" t="inlineStr"/>
       <c r="BR127" t="inlineStr"/>
-      <c r="BS127" t="inlineStr"/>
-      <c r="BT127" t="inlineStr"/>
+      <c r="BS127" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT127" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU127" s="2" t="n">
         <v>46303</v>
       </c>
       <c r="BV127" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="BW127" t="inlineStr"/>
-      <c r="BX127" t="inlineStr"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="BW127" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="BX127" t="inlineStr">
+        <is>
+          <t>01/09/2026 10:07:26</t>
+        </is>
+      </c>
       <c r="BY127" t="inlineStr"/>
       <c r="BZ127" t="inlineStr"/>
       <c r="CA127" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL021: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por Yolanda, 01/09/2026 10:11)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -40544,10 +40544,14 @@
       <c r="N192" t="inlineStr"/>
       <c r="O192" t="inlineStr"/>
       <c r="P192" t="inlineStr"/>
-      <c r="Q192" t="inlineStr"/>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+        </is>
+      </c>
       <c r="R192" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S192" t="inlineStr"/>
@@ -40557,11 +40561,25 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr"/>
       <c r="Y192" t="inlineStr"/>
-      <c r="Z192" t="inlineStr"/>
-      <c r="AA192" t="inlineStr"/>
-      <c r="AB192" t="inlineStr"/>
-      <c r="AC192" t="inlineStr"/>
-      <c r="AD192" t="inlineStr"/>
+      <c r="Z192" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="AB192" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE192" t="inlineStr"/>
       <c r="AF192" t="inlineStr"/>
       <c r="AG192" t="inlineStr"/>
@@ -40606,8 +40624,16 @@
       <c r="BT192" t="inlineStr"/>
       <c r="BU192" t="inlineStr"/>
       <c r="BV192" t="inlineStr"/>
-      <c r="BW192" t="inlineStr"/>
-      <c r="BX192" t="inlineStr"/>
+      <c r="BW192" t="inlineStr">
+        <is>
+          <t>Yolanda</t>
+        </is>
+      </c>
+      <c r="BX192" t="inlineStr">
+        <is>
+          <t>01/09/2026 10:11:58</t>
+        </is>
+      </c>
       <c r="BY192" t="inlineStr"/>
       <c r="BZ192" t="inlineStr"/>
       <c r="CA192" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL021: Etapa 2 TERMINADA · Recolección → pasa a Disposición final (por yolanda, 01/09/2026 10:12)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -40546,15 +40546,19 @@
       <c r="P192" t="inlineStr"/>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:12 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S192" t="inlineStr"/>
+          <t>Disposición final</t>
+        </is>
+      </c>
+      <c r="S192" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T192" t="inlineStr"/>
       <c r="U192" t="inlineStr"/>
       <c r="V192" t="inlineStr"/>
@@ -40581,17 +40585,45 @@
         </is>
       </c>
       <c r="AE192" t="inlineStr"/>
-      <c r="AF192" t="inlineStr"/>
+      <c r="AF192" t="inlineStr">
+        <is>
+          <t>recoleccion</t>
+        </is>
+      </c>
       <c r="AG192" t="inlineStr"/>
-      <c r="AH192" t="inlineStr"/>
+      <c r="AH192" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="AI192" t="inlineStr"/>
-      <c r="AJ192" t="inlineStr"/>
-      <c r="AK192" t="inlineStr"/>
-      <c r="AL192" t="inlineStr"/>
-      <c r="AM192" t="inlineStr"/>
-      <c r="AN192" t="inlineStr"/>
-      <c r="AO192" t="inlineStr"/>
-      <c r="AP192" t="inlineStr"/>
+      <c r="AJ192" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AK192" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AL192" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AM192" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AN192" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="AO192" t="n">
+        <v>7</v>
+      </c>
+      <c r="AP192" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ192" t="inlineStr"/>
       <c r="AR192" t="inlineStr"/>
       <c r="AS192" t="inlineStr"/>
@@ -40605,7 +40637,11 @@
       <c r="BA192" t="inlineStr"/>
       <c r="BB192" t="inlineStr"/>
       <c r="BC192" t="inlineStr"/>
-      <c r="BD192" t="inlineStr"/>
+      <c r="BD192" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE192" t="inlineStr"/>
       <c r="BF192" t="inlineStr"/>
       <c r="BG192" t="inlineStr"/>
@@ -40622,16 +40658,18 @@
       <c r="BR192" t="inlineStr"/>
       <c r="BS192" t="inlineStr"/>
       <c r="BT192" t="inlineStr"/>
-      <c r="BU192" t="inlineStr"/>
+      <c r="BU192" s="2" t="n">
+        <v>46286</v>
+      </c>
       <c r="BV192" t="inlineStr"/>
       <c r="BW192" t="inlineStr">
         <is>
-          <t>Yolanda</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX192" t="inlineStr">
         <is>
-          <t>01/09/2026 10:11:58</t>
+          <t>01/09/2026 10:12:38</t>
         </is>
       </c>
       <c r="BY192" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL021: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 10:13)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -40546,12 +40546,12 @@
       <c r="P192" t="inlineStr"/>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:12 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
+          <t>[01/09/2026 10:11 · Yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:12 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [01/09/2026 10:13 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R192" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S192" t="inlineStr">
@@ -40643,7 +40643,11 @@
         </is>
       </c>
       <c r="BE192" t="inlineStr"/>
-      <c r="BF192" t="inlineStr"/>
+      <c r="BF192" t="inlineStr">
+        <is>
+          <t>8429 clave 59290  1 pend</t>
+        </is>
+      </c>
       <c r="BG192" t="inlineStr"/>
       <c r="BH192" t="inlineStr"/>
       <c r="BI192" t="inlineStr"/>
@@ -40656,12 +40660,22 @@
       <c r="BP192" t="inlineStr"/>
       <c r="BQ192" t="inlineStr"/>
       <c r="BR192" t="inlineStr"/>
-      <c r="BS192" t="inlineStr"/>
-      <c r="BT192" t="inlineStr"/>
+      <c r="BS192" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT192" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU192" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="BV192" t="inlineStr"/>
+      <c r="BV192" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW192" t="inlineStr">
         <is>
           <t>yolanda</t>
@@ -40669,7 +40683,7 @@
       </c>
       <c r="BX192" t="inlineStr">
         <is>
-          <t>01/09/2026 10:12:38</t>
+          <t>01/09/2026 10:13:16</t>
         </is>
       </c>
       <c r="BY192" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL050: Avance en Cuentas por pagar (por yolanda, 01/09/2026 10:14)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -36724,7 +36724,7 @@
       <c r="P163" t="inlineStr"/>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [29/08/2026 13:06 · Francisco] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
+          <t>[25/08/2026 08:33 · Francisco] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [25/08/2026 08:55 · Francisco] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [29/08/2026 13:06 · Francisco] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar | [01/09/2026 10:14 · yolanda] Avance en Cuentas por pagar</t>
         </is>
       </c>
       <c r="R163" t="inlineStr">
@@ -36819,16 +36819,28 @@
         </is>
       </c>
       <c r="AQ163" t="inlineStr"/>
-      <c r="AR163" t="inlineStr"/>
+      <c r="AR163" t="inlineStr">
+        <is>
+          <t>8425</t>
+        </is>
+      </c>
       <c r="AS163" t="inlineStr"/>
       <c r="AT163" t="inlineStr"/>
-      <c r="AU163" t="inlineStr"/>
-      <c r="AV163" t="inlineStr"/>
+      <c r="AU163" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AV163" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="AW163" t="inlineStr"/>
       <c r="AX163" t="inlineStr"/>
       <c r="AY163" t="inlineStr"/>
       <c r="AZ163" t="inlineStr"/>
-      <c r="BA163" t="inlineStr"/>
+      <c r="BA163" s="2" t="n">
+        <v>46342</v>
+      </c>
       <c r="BB163" t="inlineStr"/>
       <c r="BC163" t="inlineStr"/>
       <c r="BD163" t="inlineStr">
@@ -36886,12 +36898,12 @@
       </c>
       <c r="BW163" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX163" t="inlineStr">
         <is>
-          <t>29/08/2026 13:06:47</t>
+          <t>01/09/2026 10:14:25</t>
         </is>
       </c>
       <c r="BY163" t="inlineStr"/>

</xml_diff>

<commit_message>
Folio DC-JL024: Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días (por Admin cuarentena, 01/09/2026 10:16)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -39028,7 +39028,11 @@
       <c r="N180" t="inlineStr"/>
       <c r="O180" t="inlineStr"/>
       <c r="P180" t="inlineStr"/>
-      <c r="Q180" t="inlineStr"/>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días</t>
+        </is>
+      </c>
       <c r="R180" t="inlineStr">
         <is>
           <t>Cuarentena</t>
@@ -39090,8 +39094,16 @@
       <c r="BT180" t="inlineStr"/>
       <c r="BU180" t="inlineStr"/>
       <c r="BV180" t="inlineStr"/>
-      <c r="BW180" t="inlineStr"/>
-      <c r="BX180" t="inlineStr"/>
+      <c r="BW180" t="inlineStr">
+        <is>
+          <t>Admin cuarentena</t>
+        </is>
+      </c>
+      <c r="BX180" t="inlineStr">
+        <is>
+          <t>01/09/2026 10:16:31</t>
+        </is>
+      </c>
       <c r="BY180" t="inlineStr">
         <is>
           <t>SÍ</t>
@@ -39101,10 +39113,10 @@
         <v>46258</v>
       </c>
       <c r="CA180" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="CB180" s="1" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="CC180" t="inlineStr"/>
       <c r="CD180" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-JL024: 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo (por Admin cuarentena, 01/09/2026 10:16)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -39030,12 +39030,12 @@
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días</t>
+          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>Cuarentena</t>
+          <t>Reporte de reclamo</t>
         </is>
       </c>
       <c r="S180" t="inlineStr"/>
@@ -39101,12 +39101,12 @@
       </c>
       <c r="BX180" t="inlineStr">
         <is>
-          <t>01/09/2026 10:16:31</t>
+          <t>01/09/2026 10:16:43</t>
         </is>
       </c>
       <c r="BY180" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>LIBERADA</t>
         </is>
       </c>
       <c r="BZ180" s="1" t="n">

</xml_diff>

<commit_message>
Folio DC-JL024: Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión (por yolanda, 01/09/2026 10:18)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -39030,12 +39030,12 @@
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo</t>
+          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>Reporte de reclamo</t>
+          <t>Gestión</t>
         </is>
       </c>
       <c r="S180" t="inlineStr"/>
@@ -39045,11 +39045,25 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr"/>
       <c r="Y180" t="inlineStr"/>
-      <c r="Z180" t="inlineStr"/>
-      <c r="AA180" t="inlineStr"/>
-      <c r="AB180" t="inlineStr"/>
-      <c r="AC180" t="inlineStr"/>
-      <c r="AD180" t="inlineStr"/>
+      <c r="Z180" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AB180" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>14</v>
+      </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AE180" t="inlineStr"/>
       <c r="AF180" t="inlineStr"/>
       <c r="AG180" t="inlineStr"/>
@@ -39096,12 +39110,12 @@
       <c r="BV180" t="inlineStr"/>
       <c r="BW180" t="inlineStr">
         <is>
-          <t>Admin cuarentena</t>
+          <t>yolanda</t>
         </is>
       </c>
       <c r="BX180" t="inlineStr">
         <is>
-          <t>01/09/2026 10:16:43</t>
+          <t>01/09/2026 10:18:00</t>
         </is>
       </c>
       <c r="BY180" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-JL024: Etapa 2 TERMINADA · Recolección → pasa a Disposición final (por yolanda, 01/09/2026 10:18)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -39030,15 +39030,19 @@
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión</t>
+          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:18 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>Gestión</t>
-        </is>
-      </c>
-      <c r="S180" t="inlineStr"/>
+          <t>Disposición final</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="T180" t="inlineStr"/>
       <c r="U180" t="inlineStr"/>
       <c r="V180" t="inlineStr"/>
@@ -39065,17 +39069,45 @@
         </is>
       </c>
       <c r="AE180" t="inlineStr"/>
-      <c r="AF180" t="inlineStr"/>
+      <c r="AF180" t="inlineStr">
+        <is>
+          <t>recoleccion</t>
+        </is>
+      </c>
       <c r="AG180" t="inlineStr"/>
-      <c r="AH180" t="inlineStr"/>
+      <c r="AH180" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="AI180" t="inlineStr"/>
-      <c r="AJ180" t="inlineStr"/>
-      <c r="AK180" t="inlineStr"/>
-      <c r="AL180" t="inlineStr"/>
-      <c r="AM180" t="inlineStr"/>
-      <c r="AN180" t="inlineStr"/>
-      <c r="AO180" t="inlineStr"/>
-      <c r="AP180" t="inlineStr"/>
+      <c r="AJ180" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AK180" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AL180" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
+      <c r="AM180" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AN180" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="AO180" t="n">
+        <v>7</v>
+      </c>
+      <c r="AP180" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AQ180" t="inlineStr"/>
       <c r="AR180" t="inlineStr"/>
       <c r="AS180" t="inlineStr"/>
@@ -39089,7 +39121,11 @@
       <c r="BA180" t="inlineStr"/>
       <c r="BB180" t="inlineStr"/>
       <c r="BC180" t="inlineStr"/>
-      <c r="BD180" t="inlineStr"/>
+      <c r="BD180" t="inlineStr">
+        <is>
+          <t>Recolección</t>
+        </is>
+      </c>
       <c r="BE180" t="inlineStr"/>
       <c r="BF180" t="inlineStr"/>
       <c r="BG180" t="inlineStr"/>
@@ -39106,7 +39142,9 @@
       <c r="BR180" t="inlineStr"/>
       <c r="BS180" t="inlineStr"/>
       <c r="BT180" t="inlineStr"/>
-      <c r="BU180" t="inlineStr"/>
+      <c r="BU180" s="2" t="n">
+        <v>46286</v>
+      </c>
       <c r="BV180" t="inlineStr"/>
       <c r="BW180" t="inlineStr">
         <is>
@@ -39115,7 +39153,7 @@
       </c>
       <c r="BX180" t="inlineStr">
         <is>
-          <t>01/09/2026 10:18:00</t>
+          <t>01/09/2026 10:18:35</t>
         </is>
       </c>
       <c r="BY180" t="inlineStr">

</xml_diff>

<commit_message>
Folio DC-JL024: Etapa Disposición final TERMINADA → pasa a Cuentas por pagar (por yolanda, 01/09/2026 10:19)
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -39030,12 +39030,12 @@
       <c r="P180" t="inlineStr"/>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:18 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final</t>
+          <t>[01/09/2026 10:16 · Admin cuarentena] Duración de cuarentena de INDUSTRIAL DE TERMINALES, S.A. DE C.V. ajustada a 29 días | [01/09/2026 10:16 · Admin cuarentena] 1 reclamación(es) de INDUSTRIAL DE TERMINALES, S.A. DE C.V. liberadas de cuarentena → Reporte de reclamo | [01/09/2026 10:18 · yolanda] Etapa 1 (Reporte de reclamo) TERMINADA → pasa a Gestión | [01/09/2026 10:18 · yolanda] Etapa 2 TERMINADA · Recolección → pasa a Disposición final | [01/09/2026 10:19 · yolanda] Etapa Disposición final TERMINADA → pasa a Cuentas por pagar</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>Disposición final</t>
+          <t>Cuentas por pagar</t>
         </is>
       </c>
       <c r="S180" t="inlineStr">
@@ -39127,7 +39127,11 @@
         </is>
       </c>
       <c r="BE180" t="inlineStr"/>
-      <c r="BF180" t="inlineStr"/>
+      <c r="BF180" t="inlineStr">
+        <is>
+          <t>8411</t>
+        </is>
+      </c>
       <c r="BG180" t="inlineStr"/>
       <c r="BH180" t="inlineStr"/>
       <c r="BI180" t="inlineStr"/>
@@ -39140,12 +39144,22 @@
       <c r="BP180" t="inlineStr"/>
       <c r="BQ180" t="inlineStr"/>
       <c r="BR180" t="inlineStr"/>
-      <c r="BS180" t="inlineStr"/>
-      <c r="BT180" t="inlineStr"/>
+      <c r="BS180" s="2" t="n">
+        <v>46266</v>
+      </c>
+      <c r="BT180" t="inlineStr">
+        <is>
+          <t>yolanda</t>
+        </is>
+      </c>
       <c r="BU180" s="2" t="n">
         <v>46286</v>
       </c>
-      <c r="BV180" t="inlineStr"/>
+      <c r="BV180" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="BW180" t="inlineStr">
         <is>
           <t>yolanda</t>
@@ -39153,7 +39167,7 @@
       </c>
       <c r="BX180" t="inlineStr">
         <is>
-          <t>01/09/2026 10:18:35</t>
+          <t>01/09/2026 10:19:24</t>
         </is>
       </c>
       <c r="BY180" t="inlineStr">

</xml_diff>